<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-02
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -775,7 +775,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>3510</v>
+        <v>3566</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
@@ -783,10 +783,10 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>6.98</v>
+        <v>6.99</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>13.4</v>
+        <v>15.2</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>-2.13</v>
@@ -813,23 +813,23 @@
       <c r="W2" s="2" t="inlineStr"/>
       <c r="X2" s="2" t="inlineStr"/>
       <c r="Y2" s="2" t="n">
-        <v>98.40000000000001</v>
+        <v>98.95</v>
       </c>
       <c r="Z2" s="2" t="n">
-        <v>26.17</v>
+        <v>28.1</v>
       </c>
       <c r="AA2" s="2" t="n"/>
       <c r="AB2" s="2" t="n">
-        <v>8.039999999999999</v>
+        <v>11.63</v>
       </c>
       <c r="AC2" s="2" t="n">
-        <v>-4.85</v>
+        <v>0.39</v>
       </c>
       <c r="AD2" s="2" t="n">
-        <v>-1.9</v>
+        <v>-1.6</v>
       </c>
       <c r="AE2" s="2" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="n">
@@ -843,40 +843,40 @@
         </is>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>3271.6</v>
+        <v>3282.8</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>3146.2</v>
+        <v>3151.8</v>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>3113.325</v>
+        <v>3116.125</v>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>3220.217</v>
+        <v>3222.083</v>
       </c>
       <c r="AO2" s="2" t="n">
-        <v>3364.87</v>
+        <v>3365.99</v>
       </c>
       <c r="AP2" s="2" t="n">
-        <v>3676.476</v>
+        <v>3677.036</v>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>2696.635</v>
+        <v>2696.915</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>2.5169</v>
+        <v>2.6139</v>
       </c>
       <c r="AS2" s="2" t="n">
-        <v>-0.5225</v>
+        <v>-0.4762</v>
       </c>
       <c r="AT2" s="2" t="n">
-        <v>-2.2712</v>
+        <v>-2.2547</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>0.3456</v>
+        <v>0.3535</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>0.984</v>
+        <v>0.9895</v>
       </c>
     </row>
     <row r="3">
@@ -891,7 +891,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>16245</v>
+        <v>16700</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -899,10 +899,10 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>5.28</v>
+        <v>5.3</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>8.9</v>
+        <v>12</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>38.24</v>
@@ -931,23 +931,23 @@
       <c r="W3" s="2" t="inlineStr"/>
       <c r="X3" s="2" t="inlineStr"/>
       <c r="Y3" s="2" t="n">
-        <v>89.16</v>
+        <v>90.08</v>
       </c>
       <c r="Z3" s="2" t="n">
-        <v>22.79</v>
+        <v>26.05</v>
       </c>
       <c r="AA3" s="2" t="n"/>
       <c r="AB3" s="2" t="n">
-        <v>5.89</v>
+        <v>10.18</v>
       </c>
       <c r="AC3" s="2" t="n">
-        <v>-8.300000000000001</v>
+        <v>-6.23</v>
       </c>
       <c r="AD3" s="2" t="n">
-        <v>32.8</v>
+        <v>33.5</v>
       </c>
       <c r="AE3" s="2" t="n">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="inlineStr"/>
@@ -959,40 +959,40 @@
         </is>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>15096.31</v>
+        <v>15187.31</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>14637.224</v>
+        <v>14682.724</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>14927.862</v>
+        <v>14950.612</v>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>15294.741</v>
+        <v>15309.908</v>
       </c>
       <c r="AO3" s="2" t="n">
-        <v>15217.145</v>
+        <v>15226.245</v>
       </c>
       <c r="AP3" s="2" t="n">
-        <v>16269.472</v>
+        <v>16274.022</v>
       </c>
       <c r="AQ3" s="2" t="n">
-        <v>13116.153</v>
+        <v>13118.428</v>
       </c>
       <c r="AR3" s="2" t="n">
-        <v>0.7063</v>
+        <v>0.8702</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>-0.847</v>
+        <v>-0.769</v>
       </c>
       <c r="AT3" s="2" t="n">
-        <v>-0.0013</v>
+        <v>0.0298</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>0.0472</v>
+        <v>0.0618</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>0.8915999999999999</v>
+        <v>0.9008</v>
       </c>
     </row>
     <row r="4">
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>11835</v>
+        <v>12110</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
@@ -1015,13 +1015,13 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>11.54</v>
+        <v>11.58</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>43.7</v>
+        <v>47</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>106.01</v>
+        <v>109.71</v>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
@@ -1051,23 +1051,23 @@
       <c r="W4" s="2" t="inlineStr"/>
       <c r="X4" s="2" t="inlineStr"/>
       <c r="Y4" s="2" t="n">
-        <v>160.86</v>
+        <v>162.06</v>
       </c>
       <c r="Z4" s="2" t="n">
-        <v>70.8</v>
+        <v>74.19</v>
       </c>
       <c r="AA4" s="2" t="n"/>
       <c r="AB4" s="2" t="n">
-        <v>-2.22</v>
+        <v>-2.93</v>
       </c>
       <c r="AC4" s="2" t="n">
-        <v>3.17</v>
+        <v>6.27</v>
       </c>
       <c r="AD4" s="2" t="n">
-        <v>58.1</v>
+        <v>58.6</v>
       </c>
       <c r="AE4" s="2" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="inlineStr"/>
@@ -1079,40 +1079,40 @@
         </is>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>11404</v>
+        <v>11459</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>10831.593</v>
+        <v>10859.093</v>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>10492.086</v>
+        <v>10505.836</v>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>10300.773</v>
+        <v>10309.939</v>
       </c>
       <c r="AO4" s="2" t="n">
-        <v>9794.697</v>
+        <v>9800.197</v>
       </c>
       <c r="AP4" s="2" t="n">
-        <v>9988.618</v>
+        <v>9991.368</v>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>7090.009</v>
+        <v>7088.811</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>3.664</v>
+        <v>3.8053</v>
       </c>
       <c r="AS4" s="2" t="n">
-        <v>1.5801</v>
+        <v>1.6503</v>
       </c>
       <c r="AT4" s="2" t="n">
-        <v>1.3654</v>
+        <v>1.3953</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>1.1393</v>
+        <v>1.1539</v>
       </c>
       <c r="AV4" s="2" t="n">
-        <v>1.6086</v>
+        <v>1.6206</v>
       </c>
     </row>
     <row r="5">
@@ -1127,7 +1127,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>5988</v>
+        <v>5997</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -1138,7 +1138,7 @@
         <v>1.05</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>-8.699999999999999</v>
+        <v>-8.6</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>-1.27</v>
@@ -1158,26 +1158,24 @@
       <c r="R5" s="2" t="inlineStr"/>
       <c r="S5" s="2" t="inlineStr"/>
       <c r="T5" s="2" t="inlineStr"/>
-      <c r="U5" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
+      <c r="U5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="V5" s="2" t="inlineStr"/>
       <c r="W5" s="2" t="inlineStr"/>
       <c r="X5" s="2" t="inlineStr"/>
       <c r="Y5" s="2" t="n">
-        <v>25.93</v>
+        <v>25.97</v>
       </c>
       <c r="Z5" s="2" t="n">
-        <v>-14</v>
+        <v>-13.72</v>
       </c>
       <c r="AA5" s="2" t="n"/>
       <c r="AB5" s="2" t="n">
-        <v>-2.15</v>
+        <v>-0.57</v>
       </c>
       <c r="AC5" s="2" t="n">
-        <v>-2.1</v>
+        <v>-1.19</v>
       </c>
       <c r="AD5" s="2" t="n">
         <v>-0.4</v>
@@ -1197,40 +1195,40 @@
         </is>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>5900.6</v>
+        <v>5902.4</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>5862.049</v>
+        <v>5862.949</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>5805.951</v>
+        <v>5806.401</v>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>5874.052</v>
+        <v>5874.352</v>
       </c>
       <c r="AO5" s="2" t="n">
-        <v>6027.132</v>
+        <v>6027.312</v>
       </c>
       <c r="AP5" s="2" t="n">
-        <v>6621.203</v>
+        <v>6621.293</v>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>6198.412</v>
+        <v>6198.457</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.8471</v>
+        <v>0.8552</v>
       </c>
       <c r="AS5" s="2" t="n">
-        <v>-0.1545</v>
+        <v>-0.1505</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>-1.2444</v>
+        <v>-1.2429</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>-0.5435</v>
+        <v>-0.5427999999999999</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>0.2593</v>
+        <v>0.2597</v>
       </c>
     </row>
     <row r="6">
@@ -1245,7 +1243,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>8907</v>
+        <v>8880</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -1256,7 +1254,7 @@
         <v>0.88</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>-4.9</v>
+        <v>-5.1</v>
       </c>
       <c r="G6" s="2" t="n">
         <v>-2.11</v>
@@ -1283,20 +1281,20 @@
       <c r="W6" s="2" t="inlineStr"/>
       <c r="X6" s="2" t="inlineStr"/>
       <c r="Y6" s="2" t="n">
-        <v>41.28</v>
+        <v>41.19</v>
       </c>
       <c r="Z6" s="2" t="n">
-        <v>-4.58</v>
+        <v>-4.81</v>
       </c>
       <c r="AA6" s="2" t="n"/>
       <c r="AB6" s="2" t="n">
-        <v>2.33</v>
+        <v>2.59</v>
       </c>
       <c r="AC6" s="2" t="n">
-        <v>-0.87</v>
+        <v>-0.36</v>
       </c>
       <c r="AD6" s="2" t="n">
-        <v>7.5</v>
+        <v>7.4</v>
       </c>
       <c r="AE6" s="2" t="n">
         <v>80</v>
@@ -1313,40 +1311,40 @@
         </is>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>8605.6</v>
+        <v>8600.200000000001</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>8378</v>
+        <v>8375.299999999999</v>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>8280.299999999999</v>
+        <v>8278.950000000001</v>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>8418.6</v>
+        <v>8417.700000000001</v>
       </c>
       <c r="AO6" s="2" t="n">
-        <v>8795.299999999999</v>
+        <v>8794.76</v>
       </c>
       <c r="AP6" s="2" t="n">
-        <v>9722.124</v>
+        <v>9721.853999999999</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>8683.386</v>
+        <v>8683.251</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>1.5066</v>
+        <v>1.4893</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>-0.0731</v>
+        <v>-0.0815</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>-1.1092</v>
+        <v>-1.1123</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>-0.1825</v>
+        <v>-0.1839</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>0.4128</v>
+        <v>0.4119</v>
       </c>
     </row>
     <row r="7">
@@ -1361,7 +1359,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>5641</v>
+        <v>5622</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -1372,7 +1370,7 @@
         <v>1.23</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>4.6</v>
+        <v>4.3</v>
       </c>
       <c r="G7" s="2" t="n">
         <v>94.59</v>
@@ -1411,20 +1409,20 @@
       </c>
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="n">
-        <v>35.16</v>
+        <v>35.07</v>
       </c>
       <c r="Z7" s="2" t="n">
-        <v>-6.02</v>
+        <v>-6.17</v>
       </c>
       <c r="AA7" s="2" t="n"/>
       <c r="AB7" s="2" t="n">
-        <v>-6.53</v>
+        <v>-6.85</v>
       </c>
       <c r="AC7" s="2" t="n">
-        <v>-2.54</v>
+        <v>-4.22</v>
       </c>
       <c r="AD7" s="2" t="n">
-        <v>97.3</v>
+        <v>97.09999999999999</v>
       </c>
       <c r="AE7" s="2" t="n">
         <v>15</v>
@@ -1445,40 +1443,40 @@
         </is>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>5743.8</v>
+        <v>5740</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>5782.46</v>
+        <v>5780.56</v>
       </c>
       <c r="AM7" s="2" t="n">
-        <v>5718.94</v>
+        <v>5717.99</v>
       </c>
       <c r="AN7" s="2" t="n">
-        <v>5714.245</v>
+        <v>5713.612</v>
       </c>
       <c r="AO7" s="2" t="n">
-        <v>5616.416</v>
+        <v>5616.036</v>
       </c>
       <c r="AP7" s="2" t="n">
-        <v>5337.845</v>
+        <v>5337.655</v>
       </c>
       <c r="AQ7" s="2" t="n">
-        <v>5261.155</v>
+        <v>5261.06</v>
       </c>
       <c r="AR7" s="2" t="n">
-        <v>0.6258</v>
+        <v>0.6085</v>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>0.0638</v>
+        <v>0.0552</v>
       </c>
       <c r="AT7" s="2" t="n">
-        <v>0.4522</v>
+        <v>0.4487</v>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>0.2792</v>
+        <v>0.2773</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>0.3516</v>
+        <v>0.3507</v>
       </c>
     </row>
     <row r="8">
@@ -1493,7 +1491,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2277.5</v>
+        <v>2247.5</v>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
@@ -1501,10 +1499,10 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.16</v>
+        <v>0.15</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>-0.1</v>
+        <v>-1.4</v>
       </c>
       <c r="G8" s="2" t="n">
         <v>80.33</v>
@@ -1535,23 +1533,23 @@
       </c>
       <c r="X8" s="2" t="inlineStr"/>
       <c r="Y8" s="2" t="n">
-        <v>22.25</v>
+        <v>21.9</v>
       </c>
       <c r="Z8" s="2" t="n">
-        <v>-10.25</v>
+        <v>-11.29</v>
       </c>
       <c r="AA8" s="2" t="n"/>
       <c r="AB8" s="2" t="n">
-        <v>-5.71</v>
+        <v>-7.14</v>
       </c>
       <c r="AC8" s="2" t="n">
-        <v>-4.82</v>
+        <v>-7.73</v>
       </c>
       <c r="AD8" s="2" t="n">
-        <v>82.8</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="AE8" s="2" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="AF8" s="2" t="inlineStr"/>
       <c r="AG8" s="2" t="inlineStr"/>
@@ -1565,40 +1563,40 @@
         </is>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>2303.3</v>
+        <v>2297.3</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>2313.565</v>
+        <v>2310.565</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>2290.067</v>
+        <v>2288.567</v>
       </c>
       <c r="AN8" s="2" t="n">
-        <v>2310.873</v>
+        <v>2309.873</v>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>2272.076</v>
+        <v>2271.476</v>
       </c>
       <c r="AP8" s="2" t="n">
-        <v>2212.471</v>
+        <v>2212.171</v>
       </c>
       <c r="AQ8" s="2" t="n">
-        <v>2247.216</v>
+        <v>2247.066</v>
       </c>
       <c r="AR8" s="2" t="n">
-        <v>0.9072</v>
+        <v>0.8386</v>
       </c>
       <c r="AS8" s="2" t="n">
-        <v>-0.2802</v>
+        <v>-0.3141</v>
       </c>
       <c r="AT8" s="2" t="n">
-        <v>0.4573</v>
+        <v>0.4435</v>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>0.0853</v>
+        <v>0.07820000000000001</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>0.2225</v>
+        <v>0.219</v>
       </c>
     </row>
     <row r="9">
@@ -1613,7 +1611,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>2730.5</v>
+        <v>2708</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
@@ -1621,10 +1619,10 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>-0.47</v>
+        <v>-0.48</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>1.2</v>
+        <v>0.4</v>
       </c>
       <c r="G9" s="2" t="n">
         <v>98.16</v>
@@ -1653,23 +1651,23 @@
       <c r="W9" s="2" t="inlineStr"/>
       <c r="X9" s="2" t="inlineStr"/>
       <c r="Y9" s="2" t="n">
-        <v>-37.96</v>
+        <v>-38.17</v>
       </c>
       <c r="Z9" s="2" t="n">
-        <v>-24.72</v>
+        <v>-25.04</v>
       </c>
       <c r="AA9" s="2" t="n"/>
       <c r="AB9" s="2" t="n">
-        <v>-5.19</v>
+        <v>-6.05</v>
       </c>
       <c r="AC9" s="2" t="n">
-        <v>-0.05</v>
+        <v>-0.79</v>
       </c>
       <c r="AD9" s="2" t="n">
-        <v>85.40000000000001</v>
+        <v>84.8</v>
       </c>
       <c r="AE9" s="2" t="n">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="inlineStr"/>
@@ -1683,40 +1681,40 @@
         </is>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>2767.1</v>
+        <v>2762.6</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>2811.321</v>
+        <v>2809.071</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>2775.596</v>
+        <v>2774.471</v>
       </c>
       <c r="AN9" s="2" t="n">
-        <v>2784.71</v>
+        <v>2783.96</v>
       </c>
       <c r="AO9" s="2" t="n">
-        <v>2745.93</v>
+        <v>2745.48</v>
       </c>
       <c r="AP9" s="2" t="n">
-        <v>2659.751</v>
+        <v>2659.526</v>
       </c>
       <c r="AQ9" s="2" t="n">
-        <v>2803.981</v>
+        <v>2803.869</v>
       </c>
       <c r="AR9" s="2" t="n">
-        <v>0.3859</v>
+        <v>0.344</v>
       </c>
       <c r="AS9" s="2" t="n">
-        <v>-0.3034</v>
+        <v>-0.3244</v>
       </c>
       <c r="AT9" s="2" t="n">
-        <v>0.1863</v>
+        <v>0.1777</v>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>0.1991</v>
+        <v>0.1947</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>-0.3796</v>
+        <v>-0.3817</v>
       </c>
     </row>
     <row r="10">
@@ -1731,7 +1729,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>11375</v>
+        <v>11245</v>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
@@ -1742,7 +1740,7 @@
         <v>2.32</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="G10" s="2" t="n">
         <v>6.32</v>
@@ -1773,23 +1771,23 @@
       <c r="W10" s="2" t="inlineStr"/>
       <c r="X10" s="2" t="inlineStr"/>
       <c r="Y10" s="2" t="n">
-        <v>31.54</v>
+        <v>31.22</v>
       </c>
       <c r="Z10" s="2" t="n">
-        <v>-5.35</v>
+        <v>-6.27</v>
       </c>
       <c r="AA10" s="2" t="n"/>
       <c r="AB10" s="2" t="n">
-        <v>-1.19</v>
+        <v>-1.97</v>
       </c>
       <c r="AC10" s="2" t="n">
-        <v>-10.2</v>
+        <v>-12.47</v>
       </c>
       <c r="AD10" s="2" t="n">
-        <v>44.5</v>
+        <v>43.8</v>
       </c>
       <c r="AE10" s="2" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="AF10" s="2" t="inlineStr"/>
       <c r="AG10" s="2" t="inlineStr"/>
@@ -1805,40 +1803,40 @@
         </is>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>11381</v>
+        <v>11355</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>11236.5</v>
+        <v>11223.5</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>11476</v>
+        <v>11469.5</v>
       </c>
       <c r="AN10" s="2" t="n">
-        <v>11729.5</v>
+        <v>11725.167</v>
       </c>
       <c r="AO10" s="2" t="n">
-        <v>11723</v>
+        <v>11720.4</v>
       </c>
       <c r="AP10" s="2" t="n">
-        <v>11325.092</v>
+        <v>11323.792</v>
       </c>
       <c r="AQ10" s="2" t="n">
-        <v>10642.221</v>
+        <v>10641.571</v>
       </c>
       <c r="AR10" s="2" t="n">
-        <v>-0.12</v>
+        <v>-0.1801</v>
       </c>
       <c r="AS10" s="2" t="n">
-        <v>-0.9585</v>
+        <v>-0.9874000000000001</v>
       </c>
       <c r="AT10" s="2" t="n">
-        <v>0.1745</v>
+        <v>0.1629</v>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>0.0614</v>
+        <v>0.0554</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>0.3154</v>
+        <v>0.3122</v>
       </c>
     </row>
     <row r="11">
@@ -1853,7 +1851,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>3335</v>
+        <v>3324</v>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
@@ -1861,10 +1859,10 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>1.02</v>
+        <v>1.01</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>2.8</v>
+        <v>2.5</v>
       </c>
       <c r="G11" s="2" t="n">
         <v>1.55</v>
@@ -1881,7 +1879,7 @@
         <v>-9</v>
       </c>
       <c r="Q11" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R11" s="2" t="inlineStr"/>
       <c r="S11" s="2" t="inlineStr"/>
@@ -1893,23 +1891,23 @@
       <c r="W11" s="2" t="inlineStr"/>
       <c r="X11" s="2" t="inlineStr"/>
       <c r="Y11" s="2" t="n">
-        <v>4.01</v>
+        <v>3.92</v>
       </c>
       <c r="Z11" s="2" t="n">
-        <v>-15.24</v>
+        <v>-15.23</v>
       </c>
       <c r="AA11" s="2" t="n"/>
       <c r="AB11" s="2" t="n">
-        <v>-2.86</v>
+        <v>-3.95</v>
       </c>
       <c r="AC11" s="2" t="n">
-        <v>0.33</v>
+        <v>-1.65</v>
       </c>
       <c r="AD11" s="2" t="n">
-        <v>15.5</v>
+        <v>15.4</v>
       </c>
       <c r="AE11" s="2" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="AF11" s="2" t="inlineStr"/>
       <c r="AG11" s="2" t="n">
@@ -1923,40 +1921,40 @@
         </is>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>3342.5</v>
+        <v>3340.3</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>3330.791</v>
+        <v>3329.691</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>3275.446</v>
+        <v>3274.896</v>
       </c>
       <c r="AN11" s="2" t="n">
-        <v>3266.985</v>
+        <v>3266.618</v>
       </c>
       <c r="AO11" s="2" t="n">
-        <v>3374.781</v>
+        <v>3374.561</v>
       </c>
       <c r="AP11" s="2" t="n">
-        <v>3370.297</v>
+        <v>3370.187</v>
       </c>
       <c r="AQ11" s="2" t="n">
-        <v>3229.755</v>
+        <v>3229.7</v>
       </c>
       <c r="AR11" s="2" t="n">
-        <v>1.1929</v>
+        <v>1.1753</v>
       </c>
       <c r="AS11" s="2" t="n">
-        <v>0.1089</v>
+        <v>0.1001</v>
       </c>
       <c r="AT11" s="2" t="n">
-        <v>-0.3603</v>
+        <v>-0.3637</v>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>0.345</v>
+        <v>0.3433</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>0.0401</v>
+        <v>0.0392</v>
       </c>
     </row>
     <row r="12">
@@ -1971,7 +1969,7 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>4292</v>
+        <v>4426</v>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
@@ -1979,10 +1977,10 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>8.01</v>
+        <v>8.029999999999999</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>8.1</v>
+        <v>11.5</v>
       </c>
       <c r="G12" s="2" t="n">
         <v>71.52</v>
@@ -2019,23 +2017,23 @@
       </c>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="n">
-        <v>120.08</v>
+        <v>121.17</v>
       </c>
       <c r="Z12" s="2" t="n">
-        <v>35.99</v>
+        <v>39.92</v>
       </c>
       <c r="AA12" s="2" t="n"/>
       <c r="AB12" s="2" t="n">
-        <v>8.18</v>
+        <v>13.52</v>
       </c>
       <c r="AC12" s="2" t="n">
-        <v>-4.53</v>
+        <v>5.34</v>
       </c>
       <c r="AD12" s="2" t="n">
-        <v>37.3</v>
+        <v>37.9</v>
       </c>
       <c r="AE12" s="2" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="AF12" s="2" t="inlineStr"/>
       <c r="AG12" s="2" t="inlineStr"/>
@@ -2047,40 +2045,40 @@
         </is>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>3943.8</v>
+        <v>3970.6</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>3877.247</v>
+        <v>3890.647</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>3853.691</v>
+        <v>3860.391</v>
       </c>
       <c r="AN12" s="2" t="n">
-        <v>3860.431</v>
+        <v>3864.897</v>
       </c>
       <c r="AO12" s="2" t="n">
-        <v>3757.717</v>
+        <v>3760.397</v>
       </c>
       <c r="AP12" s="2" t="n">
-        <v>4207.063</v>
+        <v>4208.403</v>
       </c>
       <c r="AQ12" s="2" t="n">
-        <v>3290.49</v>
+        <v>3291.16</v>
       </c>
       <c r="AR12" s="2" t="n">
-        <v>0.1052</v>
+        <v>0.2852</v>
       </c>
       <c r="AS12" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0914</v>
       </c>
       <c r="AT12" s="2" t="n">
-        <v>0.6045</v>
+        <v>0.642</v>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>-0.2437</v>
+        <v>-0.2272</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>1.2008</v>
+        <v>1.2117</v>
       </c>
     </row>
     <row r="13">
@@ -2095,7 +2093,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>2446.5</v>
+        <v>2485.5</v>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
@@ -2103,10 +2101,10 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>1.35</v>
+        <v>1.36</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>-2.4</v>
+        <v>-0.8</v>
       </c>
       <c r="G13" s="2" t="n">
         <v>16.11</v>
@@ -2123,7 +2121,9 @@
       <c r="Q13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="R13" s="2" t="inlineStr"/>
+      <c r="R13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="S13" s="2" t="inlineStr"/>
       <c r="T13" s="2" t="inlineStr"/>
       <c r="U13" s="2" t="inlineStr"/>
@@ -2133,23 +2133,23 @@
         <v>1</v>
       </c>
       <c r="Y13" s="2" t="n">
-        <v>39.67</v>
+        <v>40.12</v>
       </c>
       <c r="Z13" s="2" t="n">
-        <v>0.2</v>
+        <v>1.79</v>
       </c>
       <c r="AA13" s="2" t="n"/>
       <c r="AB13" s="2" t="n">
-        <v>6.23</v>
+        <v>8.69</v>
       </c>
       <c r="AC13" s="2" t="n">
-        <v>5.02</v>
+        <v>7.11</v>
       </c>
       <c r="AD13" s="2" t="n">
-        <v>9.1</v>
+        <v>9.4</v>
       </c>
       <c r="AE13" s="2" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="n">
@@ -2163,40 +2163,40 @@
         </is>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>2297.6</v>
+        <v>2305.4</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>2198.753</v>
+        <v>2202.653</v>
       </c>
       <c r="AM13" s="2" t="n">
-        <v>2142.539</v>
+        <v>2144.489</v>
       </c>
       <c r="AN13" s="2" t="n">
-        <v>2156.499</v>
+        <v>2157.799</v>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>2198.103</v>
+        <v>2198.883</v>
       </c>
       <c r="AP13" s="2" t="n">
-        <v>2526.154</v>
+        <v>2526.544</v>
       </c>
       <c r="AQ13" s="2" t="n">
-        <v>2310.015</v>
+        <v>2310.21</v>
       </c>
       <c r="AR13" s="2" t="n">
-        <v>2.9929</v>
+        <v>3.0905</v>
       </c>
       <c r="AS13" s="2" t="n">
-        <v>0.6228</v>
+        <v>0.6707</v>
       </c>
       <c r="AT13" s="2" t="n">
-        <v>-0.2497</v>
+        <v>-0.2313</v>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>-0.3334</v>
+        <v>-0.3254</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>0.3967</v>
+        <v>0.4012</v>
       </c>
     </row>
     <row r="14">
@@ -2211,7 +2211,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>60590</v>
+        <v>60180</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -2219,10 +2219,10 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>-2.8</v>
+        <v>-2.81</v>
       </c>
       <c r="F14" s="2" t="n">
-        <v>-9.699999999999999</v>
+        <v>-10.3</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>6.86</v>
@@ -2249,20 +2249,20 @@
       <c r="W14" s="2" t="inlineStr"/>
       <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="n">
-        <v>29.33</v>
+        <v>29.16</v>
       </c>
       <c r="Z14" s="2" t="n">
-        <v>-16.9</v>
+        <v>-17.31</v>
       </c>
       <c r="AA14" s="2" t="n"/>
       <c r="AB14" s="2" t="n">
-        <v>6.98</v>
+        <v>6.26</v>
       </c>
       <c r="AC14" s="2" t="n">
-        <v>1.53</v>
+        <v>3.12</v>
       </c>
       <c r="AD14" s="2" t="n">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="AE14" s="2" t="n">
         <v>76</v>
@@ -2279,40 +2279,40 @@
         </is>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>57877.8</v>
+        <v>57795.8</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>55011.685</v>
+        <v>54970.685</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>54255.992</v>
+        <v>54235.492</v>
       </c>
       <c r="AN14" s="2" t="n">
-        <v>56041.669</v>
+        <v>56028.002</v>
       </c>
       <c r="AO14" s="2" t="n">
-        <v>58259.921</v>
+        <v>58251.721</v>
       </c>
       <c r="AP14" s="2" t="n">
-        <v>65579.624</v>
+        <v>65575.524</v>
       </c>
       <c r="AQ14" s="2" t="n">
-        <v>64831.124</v>
+        <v>64829.074</v>
       </c>
       <c r="AR14" s="2" t="n">
-        <v>2.8131</v>
+        <v>2.7722</v>
       </c>
       <c r="AS14" s="2" t="n">
-        <v>-0.1974</v>
+        <v>-0.217</v>
       </c>
       <c r="AT14" s="2" t="n">
-        <v>-1.0657</v>
+        <v>-1.0728</v>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>-0.6555</v>
+        <v>-0.6587</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>0.2933</v>
+        <v>0.2916</v>
       </c>
     </row>
     <row r="15">
@@ -2327,7 +2327,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>4739</v>
+        <v>4758</v>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
@@ -2338,7 +2338,7 @@
         <v>-1.63</v>
       </c>
       <c r="F15" s="2" t="n">
-        <v>-10</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="G15" s="2" t="n">
         <v>-8.890000000000001</v>
@@ -2365,20 +2365,20 @@
       <c r="W15" s="2" t="inlineStr"/>
       <c r="X15" s="2" t="inlineStr"/>
       <c r="Y15" s="2" t="n">
-        <v>20.34</v>
+        <v>20.44</v>
       </c>
       <c r="Z15" s="2" t="n">
-        <v>-16.36</v>
+        <v>-15.92</v>
       </c>
       <c r="AA15" s="2" t="n"/>
       <c r="AB15" s="2" t="n">
-        <v>0.44</v>
+        <v>3.21</v>
       </c>
       <c r="AC15" s="2" t="n">
-        <v>-1.42</v>
+        <v>0.9</v>
       </c>
       <c r="AD15" s="2" t="n">
-        <v>0.9</v>
+        <v>1</v>
       </c>
       <c r="AE15" s="2" t="n">
         <v>82</v>
@@ -2395,40 +2395,40 @@
         </is>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>4666</v>
+        <v>4669.8</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>4515.3</v>
+        <v>4517.2</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>4439.4</v>
+        <v>4440.35</v>
       </c>
       <c r="AN15" s="2" t="n">
-        <v>4578.1</v>
+        <v>4578.733</v>
       </c>
       <c r="AO15" s="2" t="n">
-        <v>4978.28</v>
+        <v>4978.66</v>
       </c>
       <c r="AP15" s="2" t="n">
-        <v>5388.67</v>
+        <v>5388.86</v>
       </c>
       <c r="AQ15" s="2" t="n">
-        <v>5064.624</v>
+        <v>5064.719</v>
       </c>
       <c r="AR15" s="2" t="n">
-        <v>2.2541</v>
+        <v>2.277</v>
       </c>
       <c r="AS15" s="2" t="n">
-        <v>-0.2268</v>
+        <v>-0.2158</v>
       </c>
       <c r="AT15" s="2" t="n">
-        <v>-1.2046</v>
+        <v>-1.2007</v>
       </c>
       <c r="AU15" s="2" t="n">
-        <v>-0.386</v>
+        <v>-0.3842</v>
       </c>
       <c r="AV15" s="2" t="n">
-        <v>0.2034</v>
+        <v>0.2044</v>
       </c>
     </row>
     <row r="16">
@@ -2443,7 +2443,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>14500</v>
+        <v>14505</v>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
@@ -2454,7 +2454,7 @@
         <v>2.14</v>
       </c>
       <c r="F16" s="2" t="n">
-        <v>10.2</v>
+        <v>10.3</v>
       </c>
       <c r="G16" s="2" t="n">
         <v>32.35</v>
@@ -2491,17 +2491,17 @@
         <v>1</v>
       </c>
       <c r="Y16" s="2" t="n">
-        <v>35.74</v>
+        <v>35.75</v>
       </c>
       <c r="Z16" s="2" t="n">
-        <v>0.2</v>
+        <v>0.38</v>
       </c>
       <c r="AA16" s="2" t="n"/>
       <c r="AB16" s="2" t="n">
-        <v>4.45</v>
+        <v>4.09</v>
       </c>
       <c r="AC16" s="2" t="n">
-        <v>2.68</v>
+        <v>3.96</v>
       </c>
       <c r="AD16" s="2" t="n">
         <v>50.7</v>
@@ -2519,40 +2519,40 @@
         </is>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>14052.6</v>
+        <v>14053.6</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>13550.463</v>
+        <v>13550.963</v>
       </c>
       <c r="AM16" s="2" t="n">
-        <v>13167.184</v>
+        <v>13167.434</v>
       </c>
       <c r="AN16" s="2" t="n">
-        <v>13363.045</v>
+        <v>13363.212</v>
       </c>
       <c r="AO16" s="2" t="n">
-        <v>13506.637</v>
+        <v>13506.737</v>
       </c>
       <c r="AP16" s="2" t="n">
-        <v>13871.011</v>
+        <v>13871.061</v>
       </c>
       <c r="AQ16" s="2" t="n">
-        <v>12709.406</v>
+        <v>12709.431</v>
       </c>
       <c r="AR16" s="2" t="n">
-        <v>2.8414</v>
+        <v>2.8434</v>
       </c>
       <c r="AS16" s="2" t="n">
-        <v>0.2532</v>
+        <v>0.2541</v>
       </c>
       <c r="AT16" s="2" t="n">
-        <v>0.5779</v>
+        <v>0.5783</v>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>0.1143</v>
+        <v>0.1145</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>0.3574</v>
+        <v>0.3575</v>
       </c>
     </row>
     <row r="17">
@@ -2567,7 +2567,7 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>2135</v>
+        <v>2050</v>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
@@ -2575,10 +2575,10 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>1.36</v>
+        <v>1.34</v>
       </c>
       <c r="F17" s="2" t="n">
-        <v>-15.5</v>
+        <v>-18.9</v>
       </c>
       <c r="G17" s="2" t="n">
         <v>91.51000000000001</v>
@@ -2619,23 +2619,23 @@
       <c r="W17" s="2" t="inlineStr"/>
       <c r="X17" s="2" t="inlineStr"/>
       <c r="Y17" s="2" t="n">
-        <v>12.54</v>
+        <v>11.64</v>
       </c>
       <c r="Z17" s="2" t="n">
-        <v>-26.11</v>
+        <v>-28.74</v>
       </c>
       <c r="AA17" s="2" t="n"/>
       <c r="AB17" s="2" t="n">
-        <v>-27.18</v>
+        <v>-29.29</v>
       </c>
       <c r="AC17" s="2" t="n">
-        <v>-13.78</v>
+        <v>-16.46</v>
       </c>
       <c r="AD17" s="2" t="n">
-        <v>32.2</v>
+        <v>31</v>
       </c>
       <c r="AE17" s="2" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="AF17" s="2" t="inlineStr"/>
       <c r="AG17" s="2" t="inlineStr"/>
@@ -2651,40 +2651,40 @@
         </is>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>2236</v>
+        <v>2219</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>2506.8</v>
+        <v>2498.3</v>
       </c>
       <c r="AM17" s="2" t="n">
-        <v>2573.95</v>
+        <v>2569.7</v>
       </c>
       <c r="AN17" s="2" t="n">
-        <v>2583.833</v>
+        <v>2581</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>2612.96</v>
+        <v>2611.26</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>2650.29</v>
+        <v>2649.44</v>
       </c>
       <c r="AQ17" s="2" t="n">
-        <v>2441.54</v>
+        <v>2441.115</v>
       </c>
       <c r="AR17" s="2" t="n">
-        <v>-4.0829</v>
+        <v>-4.2454</v>
       </c>
       <c r="AS17" s="2" t="n">
-        <v>-1.7483</v>
+        <v>-1.8313</v>
       </c>
       <c r="AT17" s="2" t="n">
-        <v>-0.6927</v>
+        <v>-0.7261</v>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>-0.2319</v>
+        <v>-0.2485</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>0.1254</v>
+        <v>0.1164</v>
       </c>
     </row>
     <row r="18">
@@ -2699,7 +2699,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>3152</v>
+        <v>3158</v>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
@@ -2710,7 +2710,7 @@
         <v>3.75</v>
       </c>
       <c r="F18" s="2" t="n">
-        <v>7.8</v>
+        <v>8</v>
       </c>
       <c r="G18" s="2" t="n">
         <v>20.49</v>
@@ -2741,20 +2741,20 @@
         </is>
       </c>
       <c r="Y18" s="2" t="n">
-        <v>28.25</v>
+        <v>28.31</v>
       </c>
       <c r="Z18" s="2" t="n">
-        <v>1.23</v>
+        <v>1.55</v>
       </c>
       <c r="AA18" s="2" t="n"/>
       <c r="AB18" s="2" t="n">
-        <v>2.68</v>
+        <v>3.49</v>
       </c>
       <c r="AC18" s="2" t="n">
-        <v>-0.17</v>
+        <v>-0</v>
       </c>
       <c r="AD18" s="2" t="n">
-        <v>9.9</v>
+        <v>10</v>
       </c>
       <c r="AE18" s="2" t="n">
         <v>84</v>
@@ -2771,40 +2771,40 @@
         </is>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>3037.4</v>
+        <v>3038.6</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>2954.466</v>
+        <v>2955.066</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>2892.638</v>
+        <v>2892.938</v>
       </c>
       <c r="AN18" s="2" t="n">
-        <v>2939.072</v>
+        <v>2939.272</v>
       </c>
       <c r="AO18" s="2" t="n">
-        <v>2977.252</v>
+        <v>2977.372</v>
       </c>
       <c r="AP18" s="2" t="n">
-        <v>3245.261</v>
+        <v>3245.321</v>
       </c>
       <c r="AQ18" s="2" t="n">
-        <v>2728.502</v>
+        <v>2728.532</v>
       </c>
       <c r="AR18" s="2" t="n">
-        <v>2.1271</v>
+        <v>2.1381</v>
       </c>
       <c r="AS18" s="2" t="n">
-        <v>-0.0771</v>
+        <v>-0.0717</v>
       </c>
       <c r="AT18" s="2" t="n">
-        <v>-0.1541</v>
+        <v>-0.152</v>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>0.1801</v>
+        <v>0.1811</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>0.2825</v>
+        <v>0.2831</v>
       </c>
     </row>
     <row r="19">
@@ -2819,7 +2819,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>39050</v>
+        <v>39300</v>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
@@ -2827,10 +2827,10 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>3.62</v>
+        <v>3.63</v>
       </c>
       <c r="F19" s="2" t="n">
-        <v>34.7</v>
+        <v>35.6</v>
       </c>
       <c r="G19" s="2" t="n">
         <v>52.85</v>
@@ -2865,20 +2865,20 @@
         <v>1</v>
       </c>
       <c r="Y19" s="2" t="n">
-        <v>74.19</v>
+        <v>74.43000000000001</v>
       </c>
       <c r="Z19" s="2" t="n">
-        <v>30.99</v>
+        <v>31.72</v>
       </c>
       <c r="AA19" s="2" t="n"/>
       <c r="AB19" s="2" t="n">
-        <v>13.89</v>
+        <v>13.07</v>
       </c>
       <c r="AC19" s="2" t="n">
-        <v>9.050000000000001</v>
+        <v>11.01</v>
       </c>
       <c r="AD19" s="2" t="n">
-        <v>68.40000000000001</v>
+        <v>68.59999999999999</v>
       </c>
       <c r="AE19" s="2" t="n">
         <v>89</v>
@@ -2893,40 +2893,40 @@
         </is>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>35712</v>
+        <v>35762</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>33861</v>
+        <v>33886</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>33226</v>
+        <v>33238.5</v>
       </c>
       <c r="AN19" s="2" t="n">
-        <v>33746.667</v>
+        <v>33755</v>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>32948.3</v>
+        <v>32953.3</v>
       </c>
       <c r="AP19" s="2" t="n">
-        <v>30778.8</v>
+        <v>30781.3</v>
       </c>
       <c r="AQ19" s="2" t="n">
-        <v>27387.858</v>
+        <v>27389.108</v>
       </c>
       <c r="AR19" s="2" t="n">
-        <v>3.0637</v>
+        <v>3.1044</v>
       </c>
       <c r="AS19" s="2" t="n">
-        <v>0.4666</v>
+        <v>0.4864</v>
       </c>
       <c r="AT19" s="2" t="n">
-        <v>1.0074</v>
+        <v>1.0155</v>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>0.5659</v>
+        <v>0.5702</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>0.7419</v>
+        <v>0.7443</v>
       </c>
     </row>
     <row r="20">
@@ -2941,7 +2941,7 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>80630</v>
+        <v>79820</v>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
@@ -2952,10 +2952,10 @@
         <v>3.98</v>
       </c>
       <c r="F20" s="2" t="n">
-        <v>10.6</v>
+        <v>9.5</v>
       </c>
       <c r="G20" s="2" t="n">
-        <v>31.72</v>
+        <v>42.39</v>
       </c>
       <c r="H20" s="2" t="inlineStr"/>
       <c r="I20" s="2" t="inlineStr"/>
@@ -2969,7 +2969,7 @@
         <v>-9</v>
       </c>
       <c r="Q20" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
@@ -2983,23 +2983,23 @@
       <c r="W20" s="2" t="inlineStr"/>
       <c r="X20" s="2" t="inlineStr"/>
       <c r="Y20" s="2" t="n">
-        <v>52.1</v>
+        <v>51.79</v>
       </c>
       <c r="Z20" s="2" t="n">
-        <v>3.1</v>
+        <v>2.23</v>
       </c>
       <c r="AA20" s="2" t="n"/>
       <c r="AB20" s="2" t="n">
-        <v>-0.09</v>
+        <v>-2.74</v>
       </c>
       <c r="AC20" s="2" t="n">
-        <v>-6.18</v>
+        <v>-5.42</v>
       </c>
       <c r="AD20" s="2" t="n">
-        <v>45.6</v>
+        <v>45</v>
       </c>
       <c r="AE20" s="2" t="n">
-        <v>70</v>
+        <v>58</v>
       </c>
       <c r="AF20" s="2" t="inlineStr"/>
       <c r="AG20" s="2" t="inlineStr"/>
@@ -3011,40 +3011,40 @@
         </is>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>80058</v>
+        <v>79896</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>78546.5</v>
+        <v>78465.5</v>
       </c>
       <c r="AM20" s="2" t="n">
-        <v>77622.299</v>
+        <v>77581.799</v>
       </c>
       <c r="AN20" s="2" t="n">
-        <v>78847.656</v>
+        <v>78820.656</v>
       </c>
       <c r="AO20" s="2" t="n">
-        <v>79389.535</v>
+        <v>79373.33500000001</v>
       </c>
       <c r="AP20" s="2" t="n">
-        <v>78113.962</v>
+        <v>78105.86199999999</v>
       </c>
       <c r="AQ20" s="2" t="n">
-        <v>68835.439</v>
+        <v>68831.389</v>
       </c>
       <c r="AR20" s="2" t="n">
-        <v>1.4472</v>
+        <v>1.3921</v>
       </c>
       <c r="AS20" s="2" t="n">
-        <v>-0.3581</v>
+        <v>-0.385</v>
       </c>
       <c r="AT20" s="2" t="n">
-        <v>0.3695</v>
+        <v>0.3588</v>
       </c>
       <c r="AU20" s="2" t="n">
-        <v>0.1108</v>
+        <v>0.1054</v>
       </c>
       <c r="AV20" s="2" t="n">
-        <v>0.521</v>
+        <v>0.5179</v>
       </c>
     </row>
     <row r="21">
@@ -3059,7 +3059,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>46570</v>
+        <v>46770</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -3067,10 +3067,10 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>1.58</v>
+        <v>1.59</v>
       </c>
       <c r="F21" s="2" t="n">
-        <v>16.5</v>
+        <v>17</v>
       </c>
       <c r="G21" s="2" t="n">
         <v>2.66</v>
@@ -3105,20 +3105,20 @@
         <v>1</v>
       </c>
       <c r="Y21" s="2" t="n">
-        <v>47.67</v>
+        <v>47.81</v>
       </c>
       <c r="Z21" s="2" t="n">
-        <v>13.28</v>
+        <v>13.7</v>
       </c>
       <c r="AA21" s="2" t="n"/>
       <c r="AB21" s="2" t="n">
-        <v>11.26</v>
+        <v>10.29</v>
       </c>
       <c r="AC21" s="2" t="n">
-        <v>26.47</v>
+        <v>28.28</v>
       </c>
       <c r="AD21" s="2" t="n">
-        <v>23.5</v>
+        <v>23.6</v>
       </c>
       <c r="AE21" s="2" t="n">
         <v>89</v>
@@ -3135,40 +3135,40 @@
         </is>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>42882</v>
+        <v>42922</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>40590</v>
+        <v>40610</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>37593</v>
+        <v>37603</v>
       </c>
       <c r="AN21" s="2" t="n">
-        <v>36582.333</v>
+        <v>36589</v>
       </c>
       <c r="AO21" s="2" t="n">
-        <v>38098.6</v>
+        <v>38102.6</v>
       </c>
       <c r="AP21" s="2" t="n">
-        <v>41250.609</v>
+        <v>41252.609</v>
       </c>
       <c r="AQ21" s="2" t="n">
-        <v>38004.869</v>
+        <v>38005.869</v>
       </c>
       <c r="AR21" s="2" t="n">
-        <v>5.3975</v>
+        <v>5.4258</v>
       </c>
       <c r="AS21" s="2" t="n">
-        <v>3.2182</v>
+        <v>3.2329</v>
       </c>
       <c r="AT21" s="2" t="n">
-        <v>-0.3635</v>
+        <v>-0.3581</v>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>-0.0424</v>
+        <v>-0.0399</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>0.4767</v>
+        <v>0.4781</v>
       </c>
     </row>
     <row r="22">
@@ -3183,7 +3183,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>9809</v>
+        <v>9839</v>
       </c>
       <c r="D22" s="2" t="inlineStr">
         <is>
@@ -3194,7 +3194,7 @@
         <v>8.24</v>
       </c>
       <c r="F22" s="2" t="n">
-        <v>1.4</v>
+        <v>1.7</v>
       </c>
       <c r="G22" s="2" t="n">
         <v>-1.09</v>
@@ -3216,26 +3216,22 @@
       <c r="R22" s="2" t="inlineStr"/>
       <c r="S22" s="2" t="inlineStr"/>
       <c r="T22" s="2" t="inlineStr"/>
-      <c r="U22" s="2" t="inlineStr">
-        <is>
-          <t>预-1</t>
-        </is>
-      </c>
+      <c r="U22" s="2" t="inlineStr"/>
       <c r="V22" s="2" t="inlineStr"/>
       <c r="W22" s="2" t="inlineStr"/>
       <c r="X22" s="2" t="inlineStr"/>
       <c r="Y22" s="2" t="n">
-        <v>97.5</v>
+        <v>97.59999999999999</v>
       </c>
       <c r="Z22" s="2" t="n">
-        <v>22.44</v>
+        <v>22.65</v>
       </c>
       <c r="AA22" s="2" t="n"/>
       <c r="AB22" s="2" t="n">
-        <v>4.99</v>
+        <v>4.07</v>
       </c>
       <c r="AC22" s="2" t="n">
-        <v>-1.45</v>
+        <v>-2.43</v>
       </c>
       <c r="AD22" s="2" t="n">
         <v>-7.3</v>
@@ -3255,40 +3251,40 @@
         </is>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>9479.6</v>
+        <v>9485.6</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>9300.517</v>
+        <v>9303.517</v>
       </c>
       <c r="AM22" s="2" t="n">
-        <v>9202.915999999999</v>
+        <v>9204.415999999999</v>
       </c>
       <c r="AN22" s="2" t="n">
-        <v>9209.951999999999</v>
+        <v>9210.951999999999</v>
       </c>
       <c r="AO22" s="2" t="n">
-        <v>9738.620000000001</v>
+        <v>9739.219999999999</v>
       </c>
       <c r="AP22" s="2" t="n">
-        <v>12077.291</v>
+        <v>12077.591</v>
       </c>
       <c r="AQ22" s="2" t="n">
-        <v>8154.126</v>
+        <v>8154.276</v>
       </c>
       <c r="AR22" s="2" t="n">
-        <v>1.2177</v>
+        <v>1.2349</v>
       </c>
       <c r="AS22" s="2" t="n">
-        <v>0.5577</v>
+        <v>0.5662</v>
       </c>
       <c r="AT22" s="2" t="n">
-        <v>-1.2736</v>
+        <v>-1.2705</v>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>0.6603</v>
+        <v>0.6616</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>0.975</v>
+        <v>0.976</v>
       </c>
     </row>
     <row r="23">
@@ -3303,7 +3299,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>8458</v>
+        <v>8403</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -3311,13 +3307,13 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>9.07</v>
+        <v>9.06</v>
       </c>
       <c r="F23" s="2" t="n">
-        <v>22.4</v>
+        <v>21.6</v>
       </c>
       <c r="G23" s="2" t="n">
-        <v>103.73</v>
+        <v>101.38</v>
       </c>
       <c r="H23" s="2" t="inlineStr"/>
       <c r="I23" s="2" t="inlineStr"/>
@@ -3331,7 +3327,7 @@
         <v>-9</v>
       </c>
       <c r="Q23" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R23" s="2" t="inlineStr"/>
       <c r="S23" s="2" t="inlineStr"/>
@@ -3343,23 +3339,23 @@
       <c r="W23" s="2" t="inlineStr"/>
       <c r="X23" s="2" t="inlineStr"/>
       <c r="Y23" s="2" t="n">
-        <v>109.06</v>
+        <v>108.81</v>
       </c>
       <c r="Z23" s="2" t="n">
-        <v>39.36</v>
+        <v>38.23</v>
       </c>
       <c r="AA23" s="2" t="n"/>
       <c r="AB23" s="2" t="n">
-        <v>3.21</v>
+        <v>0.82</v>
       </c>
       <c r="AC23" s="2" t="n">
-        <v>10.68</v>
+        <v>7.94</v>
       </c>
       <c r="AD23" s="2" t="n">
-        <v>18.6</v>
+        <v>18.5</v>
       </c>
       <c r="AE23" s="2" t="n">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="AF23" s="2" t="inlineStr"/>
       <c r="AG23" s="2" t="n">
@@ -3373,40 +3369,40 @@
         </is>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>8176</v>
+        <v>8165</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>7938.289</v>
+        <v>7932.789</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>7564.653</v>
+        <v>7561.903</v>
       </c>
       <c r="AN23" s="2" t="n">
-        <v>7439.112</v>
+        <v>7437.279</v>
       </c>
       <c r="AO23" s="2" t="n">
-        <v>7499.334</v>
+        <v>7498.234</v>
       </c>
       <c r="AP23" s="2" t="n">
-        <v>8321.825999999999</v>
+        <v>8321.276</v>
       </c>
       <c r="AQ23" s="2" t="n">
-        <v>5996.193</v>
+        <v>5995.918</v>
       </c>
       <c r="AR23" s="2" t="n">
-        <v>3.102</v>
+        <v>3.0638</v>
       </c>
       <c r="AS23" s="2" t="n">
-        <v>1.6551</v>
+        <v>1.6356</v>
       </c>
       <c r="AT23" s="2" t="n">
-        <v>-0.3072</v>
+        <v>-0.3148</v>
       </c>
       <c r="AU23" s="2" t="n">
-        <v>0.9133</v>
+        <v>0.9098000000000001</v>
       </c>
       <c r="AV23" s="2" t="n">
-        <v>1.0906</v>
+        <v>1.0881</v>
       </c>
     </row>
     <row r="24">
@@ -3421,7 +3417,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>3488</v>
+        <v>3487</v>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
@@ -3465,17 +3461,17 @@
         <v>1</v>
       </c>
       <c r="Y24" s="2" t="n">
-        <v>-8.98</v>
+        <v>-8.99</v>
       </c>
       <c r="Z24" s="2" t="n">
-        <v>-15.17</v>
+        <v>-14.95</v>
       </c>
       <c r="AA24" s="2" t="n"/>
       <c r="AB24" s="2" t="n">
-        <v>-2.99</v>
+        <v>-2.65</v>
       </c>
       <c r="AC24" s="2" t="n">
-        <v>0.19</v>
+        <v>-1.47</v>
       </c>
       <c r="AD24" s="2" t="n">
         <v>78.59999999999999</v>
@@ -3493,40 +3489,40 @@
         </is>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>3485.4</v>
+        <v>3485.2</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>3445.186</v>
+        <v>3445.086</v>
       </c>
       <c r="AM24" s="2" t="n">
-        <v>3355.971</v>
+        <v>3355.921</v>
       </c>
       <c r="AN24" s="2" t="n">
-        <v>3372.635</v>
+        <v>3372.601</v>
       </c>
       <c r="AO24" s="2" t="n">
-        <v>3386.481</v>
+        <v>3386.461</v>
       </c>
       <c r="AP24" s="2" t="n">
-        <v>3238.205</v>
+        <v>3238.195</v>
       </c>
       <c r="AQ24" s="2" t="n">
-        <v>3319.008</v>
+        <v>3319.003</v>
       </c>
       <c r="AR24" s="2" t="n">
-        <v>2.4275</v>
+        <v>2.426</v>
       </c>
       <c r="AS24" s="2" t="n">
-        <v>0.1639</v>
+        <v>0.1631</v>
       </c>
       <c r="AT24" s="2" t="n">
-        <v>0.3627</v>
+        <v>0.3624</v>
       </c>
       <c r="AU24" s="2" t="n">
-        <v>0.3749</v>
+        <v>0.3747</v>
       </c>
       <c r="AV24" s="2" t="n">
-        <v>-0.0898</v>
+        <v>-0.08989999999999999</v>
       </c>
     </row>
     <row r="25">
@@ -3541,7 +3537,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>3843</v>
+        <v>3849</v>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
@@ -3552,7 +3548,7 @@
         <v>-2.92</v>
       </c>
       <c r="F25" s="2" t="n">
-        <v>-6.9</v>
+        <v>-6.8</v>
       </c>
       <c r="G25" s="2" t="n">
         <v>10.02</v>
@@ -3567,7 +3563,7 @@
       <c r="O25" s="2" t="inlineStr"/>
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R25" s="2" t="inlineStr"/>
       <c r="S25" s="2" t="inlineStr"/>
@@ -3579,23 +3575,23 @@
       </c>
       <c r="X25" s="2" t="inlineStr"/>
       <c r="Y25" s="2" t="n">
-        <v>-2.04</v>
+        <v>-2</v>
       </c>
       <c r="Z25" s="2" t="n">
-        <v>-23.84</v>
+        <v>-23.51</v>
       </c>
       <c r="AA25" s="2" t="n"/>
       <c r="AB25" s="2" t="n">
-        <v>-4.36</v>
+        <v>-2.46</v>
       </c>
       <c r="AC25" s="2" t="n">
-        <v>-0.83</v>
+        <v>-0.08</v>
       </c>
       <c r="AD25" s="2" t="n">
-        <v>43.2</v>
+        <v>43.4</v>
       </c>
       <c r="AE25" s="2" t="n">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="AF25" s="2" t="inlineStr"/>
       <c r="AG25" s="2" t="inlineStr"/>
@@ -3607,40 +3603,40 @@
         </is>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>3837.8</v>
+        <v>3839</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>3844.836</v>
+        <v>3845.436</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>3791.311</v>
+        <v>3791.611</v>
       </c>
       <c r="AN25" s="2" t="n">
-        <v>3844.745</v>
+        <v>3844.945</v>
       </c>
       <c r="AO25" s="2" t="n">
-        <v>3897.396</v>
+        <v>3897.516</v>
       </c>
       <c r="AP25" s="2" t="n">
-        <v>3860.306</v>
+        <v>3860.366</v>
       </c>
       <c r="AQ25" s="2" t="n">
-        <v>4195.74</v>
+        <v>4195.77</v>
       </c>
       <c r="AR25" s="2" t="n">
-        <v>0.7594</v>
+        <v>0.7675999999999999</v>
       </c>
       <c r="AS25" s="2" t="n">
-        <v>-0.2831</v>
+        <v>-0.279</v>
       </c>
       <c r="AT25" s="2" t="n">
-        <v>0.1125</v>
+        <v>0.1142</v>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>-0.502</v>
+        <v>-0.5012</v>
       </c>
       <c r="AV25" s="2" t="n">
-        <v>-0.0204</v>
+        <v>-0.02</v>
       </c>
     </row>
     <row r="26">
@@ -3655,7 +3651,7 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>15495</v>
+        <v>15505</v>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
@@ -3666,7 +3662,7 @@
         <v>3.52</v>
       </c>
       <c r="F26" s="2" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="G26" s="2" t="n">
         <v>3.1</v>
@@ -3697,17 +3693,17 @@
         <v>1</v>
       </c>
       <c r="Y26" s="2" t="n">
-        <v>93.06999999999999</v>
+        <v>93.09</v>
       </c>
       <c r="Z26" s="2" t="n">
-        <v>26.51</v>
+        <v>26.52</v>
       </c>
       <c r="AA26" s="2" t="n"/>
       <c r="AB26" s="2" t="n">
-        <v>12.44</v>
+        <v>10.39</v>
       </c>
       <c r="AC26" s="2" t="n">
-        <v>8.51</v>
+        <v>9.58</v>
       </c>
       <c r="AD26" s="2" t="n">
         <v>22.3</v>
@@ -3727,40 +3723,40 @@
         </is>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>14811</v>
+        <v>14813</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>13861.134</v>
+        <v>13862.134</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>13326.708</v>
+        <v>13327.208</v>
       </c>
       <c r="AN26" s="2" t="n">
-        <v>13306.219</v>
+        <v>13306.552</v>
       </c>
       <c r="AO26" s="2" t="n">
-        <v>13597.201</v>
+        <v>13597.401</v>
       </c>
       <c r="AP26" s="2" t="n">
-        <v>13993.394</v>
+        <v>13993.494</v>
       </c>
       <c r="AQ26" s="2" t="n">
-        <v>11647.467</v>
+        <v>11647.517</v>
       </c>
       <c r="AR26" s="2" t="n">
-        <v>4.8225</v>
+        <v>4.8266</v>
       </c>
       <c r="AS26" s="2" t="n">
-        <v>1.3625</v>
+        <v>1.3645</v>
       </c>
       <c r="AT26" s="2" t="n">
-        <v>-1.1725</v>
+        <v>-1.1717</v>
       </c>
       <c r="AU26" s="2" t="n">
-        <v>0.7747000000000001</v>
+        <v>0.7751</v>
       </c>
       <c r="AV26" s="2" t="n">
-        <v>0.9307</v>
+        <v>0.9308999999999999</v>
       </c>
     </row>
     <row r="27">
@@ -3775,7 +3771,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>23970</v>
+        <v>23990</v>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
@@ -3813,20 +3809,20 @@
       <c r="W27" s="2" t="inlineStr"/>
       <c r="X27" s="2" t="inlineStr"/>
       <c r="Y27" s="2" t="n">
-        <v>1.99</v>
+        <v>2.01</v>
       </c>
       <c r="Z27" s="2" t="n">
-        <v>-21.01</v>
+        <v>-20.76</v>
       </c>
       <c r="AA27" s="2" t="n"/>
       <c r="AB27" s="2" t="n">
-        <v>-0.31</v>
+        <v>-0.29</v>
       </c>
       <c r="AC27" s="2" t="n">
-        <v>-3.3</v>
+        <v>-4.19</v>
       </c>
       <c r="AD27" s="2" t="n">
-        <v>13.3</v>
+        <v>13.4</v>
       </c>
       <c r="AE27" s="2" t="n">
         <v>75</v>
@@ -3843,40 +3839,40 @@
         </is>
       </c>
       <c r="AK27" s="2" t="n">
-        <v>23751</v>
+        <v>23755</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>23303</v>
+        <v>23305</v>
       </c>
       <c r="AM27" s="2" t="n">
-        <v>23365.75</v>
+        <v>23366.75</v>
       </c>
       <c r="AN27" s="2" t="n">
-        <v>23869.333</v>
+        <v>23870</v>
       </c>
       <c r="AO27" s="2" t="n">
-        <v>24460.4</v>
+        <v>24460.8</v>
       </c>
       <c r="AP27" s="2" t="n">
-        <v>25393</v>
+        <v>25393.2</v>
       </c>
       <c r="AQ27" s="2" t="n">
-        <v>26005.612</v>
+        <v>26005.712</v>
       </c>
       <c r="AR27" s="2" t="n">
-        <v>1.1309</v>
+        <v>1.1354</v>
       </c>
       <c r="AS27" s="2" t="n">
-        <v>-0.5036</v>
+        <v>-0.5014</v>
       </c>
       <c r="AT27" s="2" t="n">
-        <v>-0.3333</v>
+        <v>-0.3325</v>
       </c>
       <c r="AU27" s="2" t="n">
-        <v>-0.4559</v>
+        <v>-0.4555</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>0.0199</v>
+        <v>0.0201</v>
       </c>
     </row>
     <row r="28">
@@ -3891,7 +3887,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>2365</v>
+        <v>2337.5</v>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
@@ -3899,10 +3895,10 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.32</v>
+        <v>0.4</v>
       </c>
       <c r="F28" s="2" t="n">
-        <v>-0.5</v>
+        <v>-1.5</v>
       </c>
       <c r="G28" s="2" t="n">
         <v>46.45</v>
@@ -3915,8 +3911,10 @@
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr"/>
       <c r="O28" s="2" t="inlineStr"/>
-      <c r="P28" s="2" t="n">
-        <v>-13</v>
+      <c r="P28" s="2" t="inlineStr">
+        <is>
+          <t>+13/-13</t>
+        </is>
       </c>
       <c r="Q28" s="2" t="n">
         <v>0</v>
@@ -3930,28 +3928,28 @@
         </is>
       </c>
       <c r="V28" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="W28" s="2" t="inlineStr"/>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="n">
-        <v>1.17</v>
+        <v>1.73</v>
       </c>
       <c r="Z28" s="2" t="n">
-        <v>-13.1</v>
+        <v>-13.6</v>
       </c>
       <c r="AA28" s="2" t="n"/>
       <c r="AB28" s="2" t="n">
-        <v>-6.08</v>
+        <v>-5.78</v>
       </c>
       <c r="AC28" s="2" t="n">
-        <v>-7.32</v>
+        <v>-5.66</v>
       </c>
       <c r="AD28" s="2" t="n">
-        <v>52</v>
+        <v>51.4</v>
       </c>
       <c r="AE28" s="2" t="n">
-        <v>49</v>
+        <v>35</v>
       </c>
       <c r="AF28" s="2" t="inlineStr"/>
       <c r="AG28" s="2" t="inlineStr"/>
@@ -3963,40 +3961,40 @@
         </is>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>2375.4</v>
+        <v>2369.9</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>2364.14</v>
+        <v>2361.39</v>
       </c>
       <c r="AM28" s="2" t="n">
-        <v>2404.305</v>
+        <v>2402.93</v>
       </c>
       <c r="AN28" s="2" t="n">
-        <v>2432.382</v>
+        <v>2431.465</v>
       </c>
       <c r="AO28" s="2" t="n">
-        <v>2405.176</v>
+        <v>2404.626</v>
       </c>
       <c r="AP28" s="2" t="n">
-        <v>2385.653</v>
+        <v>2385.378</v>
       </c>
       <c r="AQ28" s="2" t="n">
-        <v>2364.826</v>
+        <v>2358.868</v>
       </c>
       <c r="AR28" s="2" t="n">
-        <v>-0.1442</v>
+        <v>-0.2045</v>
       </c>
       <c r="AS28" s="2" t="n">
-        <v>-0.5597</v>
+        <v>-0.5891</v>
       </c>
       <c r="AT28" s="2" t="n">
-        <v>-0.0348</v>
+        <v>-0.0467</v>
       </c>
       <c r="AU28" s="2" t="n">
-        <v>-0.09039999999999999</v>
+        <v>-0.0964</v>
       </c>
       <c r="AV28" s="2" t="n">
-        <v>0.0117</v>
+        <v>0.0173</v>
       </c>
     </row>
     <row r="29">
@@ -4011,7 +4009,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>2199.5</v>
+        <v>2184</v>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
@@ -4019,10 +4017,10 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>1.36</v>
+        <v>1.35</v>
       </c>
       <c r="F29" s="2" t="n">
-        <v>9.9</v>
+        <v>9.1</v>
       </c>
       <c r="G29" s="2" t="n">
         <v>101.93</v>
@@ -4044,32 +4042,28 @@
       <c r="R29" s="2" t="inlineStr"/>
       <c r="S29" s="2" t="inlineStr"/>
       <c r="T29" s="2" t="inlineStr"/>
-      <c r="U29" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="U29" s="2" t="inlineStr"/>
       <c r="V29" s="2" t="inlineStr"/>
       <c r="W29" s="2" t="inlineStr"/>
       <c r="X29" s="2" t="inlineStr"/>
       <c r="Y29" s="2" t="n">
-        <v>25.22</v>
+        <v>25.02</v>
       </c>
       <c r="Z29" s="2" t="n">
-        <v>-5.32</v>
+        <v>-5.8</v>
       </c>
       <c r="AA29" s="2" t="n"/>
       <c r="AB29" s="2" t="n">
-        <v>-3.98</v>
+        <v>-2.84</v>
       </c>
       <c r="AC29" s="2" t="n">
-        <v>2.67</v>
+        <v>0.23</v>
       </c>
       <c r="AD29" s="2" t="n">
-        <v>90.09999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="AE29" s="2" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="AF29" s="2" t="inlineStr"/>
       <c r="AG29" s="2" t="inlineStr"/>
@@ -4087,40 +4081,40 @@
         </is>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>2194.3</v>
+        <v>2191.2</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>2228.903</v>
+        <v>2227.353</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>2235.858</v>
+        <v>2235.083</v>
       </c>
       <c r="AN29" s="2" t="n">
-        <v>2180.766</v>
+        <v>2180.249</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>2106.325</v>
+        <v>2106.015</v>
       </c>
       <c r="AP29" s="2" t="n">
-        <v>1994.477</v>
+        <v>1994.322</v>
       </c>
       <c r="AQ29" s="2" t="n">
-        <v>1993.762</v>
+        <v>1993.685</v>
       </c>
       <c r="AR29" s="2" t="n">
-        <v>-1.0335</v>
+        <v>-1.0689</v>
       </c>
       <c r="AS29" s="2" t="n">
-        <v>0.541</v>
+        <v>0.5228</v>
       </c>
       <c r="AT29" s="2" t="n">
-        <v>0.7647</v>
+        <v>0.7569</v>
       </c>
       <c r="AU29" s="2" t="n">
-        <v>0.306</v>
+        <v>0.302</v>
       </c>
       <c r="AV29" s="2" t="n">
-        <v>0.2522</v>
+        <v>0.2502</v>
       </c>
     </row>
     <row r="30">
@@ -4135,7 +4129,7 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>4770</v>
+        <v>4741</v>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
@@ -4146,10 +4140,10 @@
         <v>-1.13</v>
       </c>
       <c r="F30" s="2" t="n">
-        <v>-8.4</v>
+        <v>-9</v>
       </c>
       <c r="G30" s="2" t="n">
-        <v>13.06</v>
+        <v>9.41</v>
       </c>
       <c r="H30" s="2" t="inlineStr"/>
       <c r="I30" s="2" t="inlineStr"/>
@@ -4177,23 +4171,23 @@
       <c r="W30" s="2" t="inlineStr"/>
       <c r="X30" s="2" t="inlineStr"/>
       <c r="Y30" s="2" t="n">
-        <v>19.23</v>
+        <v>19.08</v>
       </c>
       <c r="Z30" s="2" t="n">
-        <v>-17.08</v>
+        <v>-17.45</v>
       </c>
       <c r="AA30" s="2" t="n"/>
       <c r="AB30" s="2" t="n">
-        <v>-4.57</v>
+        <v>-4.5</v>
       </c>
       <c r="AC30" s="2" t="n">
-        <v>-4.46</v>
+        <v>-8.380000000000001</v>
       </c>
       <c r="AD30" s="2" t="n">
-        <v>41.5</v>
+        <v>41</v>
       </c>
       <c r="AE30" s="2" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="inlineStr"/>
@@ -4205,40 +4199,40 @@
         </is>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>4785.3</v>
+        <v>4779.5</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>4841.007</v>
+        <v>4838.107</v>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>4932.594</v>
+        <v>4931.144</v>
       </c>
       <c r="AN30" s="2" t="n">
-        <v>4910.852</v>
+        <v>4909.885</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>4965.156</v>
+        <v>4964.576</v>
       </c>
       <c r="AP30" s="2" t="n">
-        <v>4982.97</v>
+        <v>4982.68</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>5116.038</v>
+        <v>5115.893</v>
       </c>
       <c r="AR30" s="2" t="n">
-        <v>-1.0827</v>
+        <v>-1.1132</v>
       </c>
       <c r="AS30" s="2" t="n">
-        <v>-0.2904</v>
+        <v>-0.3056</v>
       </c>
       <c r="AT30" s="2" t="n">
-        <v>-0.1547</v>
+        <v>-0.1608</v>
       </c>
       <c r="AU30" s="2" t="n">
-        <v>-0.471</v>
+        <v>-0.474</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>0.1923</v>
+        <v>0.1908</v>
       </c>
     </row>
     <row r="31">
@@ -4253,18 +4247,18 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>1158</v>
+        <v>1150</v>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>2B</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E31" s="2" t="n">
         <v>1.02</v>
       </c>
       <c r="F31" s="2" t="n">
-        <v>0.2</v>
+        <v>-0.5</v>
       </c>
       <c r="G31" s="2" t="n">
         <v>4.24</v>
@@ -4279,7 +4273,7 @@
       <c r="O31" s="2" t="inlineStr"/>
       <c r="P31" s="2" t="inlineStr"/>
       <c r="Q31" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R31" s="2" t="inlineStr"/>
       <c r="S31" s="2" t="inlineStr"/>
@@ -4287,27 +4281,31 @@
       <c r="U31" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="V31" s="2" t="inlineStr"/>
+      <c r="V31" s="2" t="inlineStr">
+        <is>
+          <t>预-1</t>
+        </is>
+      </c>
       <c r="W31" s="2" t="inlineStr"/>
       <c r="X31" s="2" t="inlineStr"/>
       <c r="Y31" s="2" t="n">
-        <v>31.79</v>
+        <v>31.61</v>
       </c>
       <c r="Z31" s="2" t="n">
-        <v>-7.49</v>
+        <v>-7.99</v>
       </c>
       <c r="AA31" s="2" t="n"/>
       <c r="AB31" s="2" t="n">
-        <v>-4.71</v>
+        <v>-4.51</v>
       </c>
       <c r="AC31" s="2" t="n">
-        <v>-3.13</v>
+        <v>-4.69</v>
       </c>
       <c r="AD31" s="2" t="n">
-        <v>31.8</v>
+        <v>31.3</v>
       </c>
       <c r="AE31" s="2" t="n">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="inlineStr"/>
@@ -4319,40 +4317,40 @@
         </is>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>1159.9</v>
+        <v>1158.3</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>1158.78</v>
+        <v>1157.98</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>1142.594</v>
+        <v>1142.194</v>
       </c>
       <c r="AN31" s="2" t="n">
-        <v>1152.742</v>
+        <v>1152.476</v>
       </c>
       <c r="AO31" s="2" t="n">
-        <v>1167.21</v>
+        <v>1167.05</v>
       </c>
       <c r="AP31" s="2" t="n">
-        <v>1154.988</v>
+        <v>1154.908</v>
       </c>
       <c r="AQ31" s="2" t="n">
-        <v>1115.557</v>
+        <v>1115.517</v>
       </c>
       <c r="AR31" s="2" t="n">
-        <v>0.8242</v>
+        <v>0.7877999999999999</v>
       </c>
       <c r="AS31" s="2" t="n">
-        <v>0.0525</v>
+        <v>0.0343</v>
       </c>
       <c r="AT31" s="2" t="n">
-        <v>0.0559</v>
+        <v>0.0487</v>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>-0.008500000000000001</v>
+        <v>-0.0121</v>
       </c>
       <c r="AV31" s="2" t="n">
-        <v>0.3179</v>
+        <v>0.3161</v>
       </c>
     </row>
     <row r="32">
@@ -4367,7 +4365,7 @@
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>7267</v>
+        <v>7181</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
@@ -4375,10 +4373,10 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>2.76</v>
+        <v>2.75</v>
       </c>
       <c r="F32" s="2" t="n">
-        <v>9.699999999999999</v>
+        <v>8.4</v>
       </c>
       <c r="G32" s="2" t="n">
         <v>101.67</v>
@@ -4401,29 +4399,29 @@
       <c r="S32" s="2" t="inlineStr"/>
       <c r="T32" s="2" t="inlineStr"/>
       <c r="U32" s="2" t="n">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="V32" s="2" t="inlineStr"/>
       <c r="W32" s="2" t="inlineStr"/>
       <c r="X32" s="2" t="inlineStr"/>
       <c r="Y32" s="2" t="n">
-        <v>48.41</v>
+        <v>48.06</v>
       </c>
       <c r="Z32" s="2" t="n">
-        <v>3.01</v>
+        <v>1.87</v>
       </c>
       <c r="AA32" s="2" t="n"/>
       <c r="AB32" s="2" t="n">
-        <v>-5.58</v>
+        <v>-6.52</v>
       </c>
       <c r="AC32" s="2" t="n">
-        <v>-7.68</v>
+        <v>-12.25</v>
       </c>
       <c r="AD32" s="2" t="n">
-        <v>89.5</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="AE32" s="2" t="n">
-        <v>48</v>
+        <v>34</v>
       </c>
       <c r="AF32" s="2" t="inlineStr"/>
       <c r="AG32" s="2" t="inlineStr"/>
@@ -4437,40 +4435,40 @@
         </is>
       </c>
       <c r="AK32" s="2" t="n">
-        <v>7235.6</v>
+        <v>7218.4</v>
       </c>
       <c r="AL32" s="2" t="n">
-        <v>7305.995</v>
+        <v>7297.395</v>
       </c>
       <c r="AM32" s="2" t="n">
-        <v>7386.262</v>
+        <v>7381.962</v>
       </c>
       <c r="AN32" s="2" t="n">
-        <v>7373.617</v>
+        <v>7370.75</v>
       </c>
       <c r="AO32" s="2" t="n">
-        <v>7168.571</v>
+        <v>7166.851</v>
       </c>
       <c r="AP32" s="2" t="n">
-        <v>6780.097</v>
+        <v>6779.237</v>
       </c>
       <c r="AQ32" s="2" t="n">
-        <v>6372.132</v>
+        <v>6371.702</v>
       </c>
       <c r="AR32" s="2" t="n">
-        <v>-0.5944</v>
+        <v>-0.6549</v>
       </c>
       <c r="AS32" s="2" t="n">
-        <v>-0.4786</v>
+        <v>-0.5086000000000001</v>
       </c>
       <c r="AT32" s="2" t="n">
-        <v>0.8565</v>
+        <v>0.8438</v>
       </c>
       <c r="AU32" s="2" t="n">
-        <v>0.2716</v>
+        <v>0.265</v>
       </c>
       <c r="AV32" s="2" t="n">
-        <v>0.4841</v>
+        <v>0.4806</v>
       </c>
     </row>
     <row r="33">
@@ -4485,7 +4483,7 @@
         </is>
       </c>
       <c r="C33" s="2" t="n">
-        <v>4892</v>
+        <v>4879</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
@@ -4496,7 +4494,7 @@
         <v>-0.35</v>
       </c>
       <c r="F33" s="2" t="n">
-        <v>-6.7</v>
+        <v>-7</v>
       </c>
       <c r="G33" s="2" t="n">
         <v>78.73999999999999</v>
@@ -4523,23 +4521,23 @@
       <c r="W33" s="2" t="inlineStr"/>
       <c r="X33" s="2" t="inlineStr"/>
       <c r="Y33" s="2" t="n">
-        <v>21.6</v>
+        <v>21.54</v>
       </c>
       <c r="Z33" s="2" t="n">
-        <v>-15.53</v>
+        <v>-15.61</v>
       </c>
       <c r="AA33" s="2" t="n"/>
       <c r="AB33" s="2" t="n">
-        <v>-4.99</v>
+        <v>-4.62</v>
       </c>
       <c r="AC33" s="2" t="n">
-        <v>-3.51</v>
+        <v>-7.02</v>
       </c>
       <c r="AD33" s="2" t="n">
-        <v>78.3</v>
+        <v>78.2</v>
       </c>
       <c r="AE33" s="2" t="n">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="AF33" s="2" t="inlineStr"/>
       <c r="AG33" s="2" t="inlineStr"/>
@@ -4551,40 +4549,40 @@
         </is>
       </c>
       <c r="AK33" s="2" t="n">
-        <v>4903.6</v>
+        <v>4901</v>
       </c>
       <c r="AL33" s="2" t="n">
-        <v>4982.322</v>
+        <v>4981.022</v>
       </c>
       <c r="AM33" s="2" t="n">
-        <v>5011.773</v>
+        <v>5011.123</v>
       </c>
       <c r="AN33" s="2" t="n">
-        <v>4963.643</v>
+        <v>4963.209</v>
       </c>
       <c r="AO33" s="2" t="n">
-        <v>4902.262</v>
+        <v>4902.002</v>
       </c>
       <c r="AP33" s="2" t="n">
-        <v>4927.469</v>
+        <v>4927.339</v>
       </c>
       <c r="AQ33" s="2" t="n">
-        <v>5134.674</v>
+        <v>5134.609</v>
       </c>
       <c r="AR33" s="2" t="n">
-        <v>-0.6879</v>
+        <v>-0.7013</v>
       </c>
       <c r="AS33" s="2" t="n">
-        <v>-0.0727</v>
+        <v>-0.0795</v>
       </c>
       <c r="AT33" s="2" t="n">
-        <v>0.2866</v>
+        <v>0.2838</v>
       </c>
       <c r="AU33" s="2" t="n">
-        <v>-0.3878</v>
+        <v>-0.3891</v>
       </c>
       <c r="AV33" s="2" t="n">
-        <v>0.216</v>
+        <v>0.2154</v>
       </c>
     </row>
     <row r="34">
@@ -4599,7 +4597,7 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>12175</v>
+        <v>12110</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
@@ -4607,13 +4605,13 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>3.5</v>
+        <v>3.93</v>
       </c>
       <c r="F34" s="2" t="n">
-        <v>16.6</v>
+        <v>16.5</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>1.98</v>
+        <v>1.96</v>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
       <c r="I34" s="2" t="inlineStr"/>
@@ -4641,23 +4639,23 @@
         <v>1</v>
       </c>
       <c r="Y34" s="2" t="n">
-        <v>76.76000000000001</v>
+        <v>80.66</v>
       </c>
       <c r="Z34" s="2" t="n">
-        <v>18.68</v>
+        <v>20.01</v>
       </c>
       <c r="AA34" s="2" t="n"/>
       <c r="AB34" s="2" t="n">
-        <v>11.42</v>
+        <v>7.18</v>
       </c>
       <c r="AC34" s="2" t="n">
-        <v>4.68</v>
+        <v>6.56</v>
       </c>
       <c r="AD34" s="2" t="n">
-        <v>14.7</v>
+        <v>14.4</v>
       </c>
       <c r="AE34" s="2" t="n">
-        <v>88</v>
+        <v>80</v>
       </c>
       <c r="AF34" s="2" t="inlineStr"/>
       <c r="AG34" s="2" t="n">
@@ -4671,40 +4669,40 @@
         </is>
       </c>
       <c r="AK34" s="2" t="n">
-        <v>11791</v>
+        <v>11778</v>
       </c>
       <c r="AL34" s="2" t="n">
-        <v>11038.193</v>
+        <v>11031.693</v>
       </c>
       <c r="AM34" s="2" t="n">
-        <v>10629.915</v>
+        <v>10626.665</v>
       </c>
       <c r="AN34" s="2" t="n">
-        <v>10645.534</v>
+        <v>10643.367</v>
       </c>
       <c r="AO34" s="2" t="n">
-        <v>10898.966</v>
+        <v>10897.666</v>
       </c>
       <c r="AP34" s="2" t="n">
-        <v>11587.294</v>
+        <v>11586.644</v>
       </c>
       <c r="AQ34" s="2" t="n">
-        <v>9650.967000000001</v>
+        <v>9547.254000000001</v>
       </c>
       <c r="AR34" s="2" t="n">
-        <v>4.5129</v>
+        <v>4.4796</v>
       </c>
       <c r="AS34" s="2" t="n">
-        <v>1.2597</v>
+        <v>1.2434</v>
       </c>
       <c r="AT34" s="2" t="n">
-        <v>-0.8608</v>
+        <v>-0.8669</v>
       </c>
       <c r="AU34" s="2" t="n">
-        <v>0.5610000000000001</v>
+        <v>0.5580000000000001</v>
       </c>
       <c r="AV34" s="2" t="n">
-        <v>0.7675999999999999</v>
+        <v>0.8066</v>
       </c>
     </row>
     <row r="35">
@@ -4719,7 +4717,7 @@
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>1752</v>
+        <v>1737</v>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
@@ -4730,7 +4728,7 @@
         <v>1.99</v>
       </c>
       <c r="F35" s="2" t="n">
-        <v>8.199999999999999</v>
+        <v>7.2</v>
       </c>
       <c r="G35" s="2" t="n">
         <v>96.56</v>
@@ -4759,23 +4757,23 @@
       <c r="W35" s="2" t="inlineStr"/>
       <c r="X35" s="2" t="inlineStr"/>
       <c r="Y35" s="2" t="n">
-        <v>47.03</v>
+        <v>46.78</v>
       </c>
       <c r="Z35" s="2" t="n">
-        <v>0.33</v>
+        <v>-0.43</v>
       </c>
       <c r="AA35" s="2" t="n"/>
       <c r="AB35" s="2" t="n">
-        <v>-4.59</v>
+        <v>-5.68</v>
       </c>
       <c r="AC35" s="2" t="n">
-        <v>-5.77</v>
+        <v>-10.04</v>
       </c>
       <c r="AD35" s="2" t="n">
-        <v>82.8</v>
+        <v>82.3</v>
       </c>
       <c r="AE35" s="2" t="n">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="AF35" s="2" t="inlineStr"/>
       <c r="AG35" s="2" t="inlineStr"/>
@@ -4789,40 +4787,40 @@
         </is>
       </c>
       <c r="AK35" s="2" t="n">
-        <v>1755.2</v>
+        <v>1752.2</v>
       </c>
       <c r="AL35" s="2" t="n">
-        <v>1766.841</v>
+        <v>1765.341</v>
       </c>
       <c r="AM35" s="2" t="n">
-        <v>1783.958</v>
+        <v>1783.208</v>
       </c>
       <c r="AN35" s="2" t="n">
-        <v>1767.993</v>
+        <v>1767.493</v>
       </c>
       <c r="AO35" s="2" t="n">
-        <v>1727.246</v>
+        <v>1726.946</v>
       </c>
       <c r="AP35" s="2" t="n">
-        <v>1688.06</v>
+        <v>1687.91</v>
       </c>
       <c r="AQ35" s="2" t="n">
-        <v>1573.151</v>
+        <v>1573.076</v>
       </c>
       <c r="AR35" s="2" t="n">
-        <v>-0.5164</v>
+        <v>-0.5601</v>
       </c>
       <c r="AS35" s="2" t="n">
-        <v>-0.0766</v>
+        <v>-0.0984</v>
       </c>
       <c r="AT35" s="2" t="n">
-        <v>0.6448</v>
+        <v>0.6357</v>
       </c>
       <c r="AU35" s="2" t="n">
-        <v>0.1865</v>
+        <v>0.1818</v>
       </c>
       <c r="AV35" s="2" t="n">
-        <v>0.4703</v>
+        <v>0.4678</v>
       </c>
     </row>
     <row r="36">
@@ -4837,7 +4835,7 @@
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>4695</v>
+        <v>4683</v>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
@@ -4848,7 +4846,7 @@
         <v>1.19</v>
       </c>
       <c r="F36" s="2" t="n">
-        <v>-4</v>
+        <v>-4.3</v>
       </c>
       <c r="G36" s="2" t="n">
         <v>91.69</v>
@@ -4875,20 +4873,20 @@
       <c r="W36" s="2" t="inlineStr"/>
       <c r="X36" s="2" t="inlineStr"/>
       <c r="Y36" s="2" t="n">
-        <v>30.51</v>
+        <v>30.44</v>
       </c>
       <c r="Z36" s="2" t="n">
-        <v>-10.78</v>
+        <v>-10.86</v>
       </c>
       <c r="AA36" s="2" t="n"/>
       <c r="AB36" s="2" t="n">
-        <v>-5.02</v>
+        <v>-4.84</v>
       </c>
       <c r="AC36" s="2" t="n">
-        <v>-3.8</v>
+        <v>-6.95</v>
       </c>
       <c r="AD36" s="2" t="n">
-        <v>75.40000000000001</v>
+        <v>75.2</v>
       </c>
       <c r="AE36" s="2" t="n">
         <v>38</v>
@@ -4903,40 +4901,40 @@
         </is>
       </c>
       <c r="AK36" s="2" t="n">
-        <v>4715.8</v>
+        <v>4713.4</v>
       </c>
       <c r="AL36" s="2" t="n">
-        <v>4780.321</v>
+        <v>4779.121</v>
       </c>
       <c r="AM36" s="2" t="n">
-        <v>4841.652</v>
+        <v>4841.052</v>
       </c>
       <c r="AN36" s="2" t="n">
-        <v>4797.209</v>
+        <v>4796.809</v>
       </c>
       <c r="AO36" s="2" t="n">
-        <v>4772.749</v>
+        <v>4772.509</v>
       </c>
       <c r="AP36" s="2" t="n">
-        <v>4773.358</v>
+        <v>4773.238</v>
       </c>
       <c r="AQ36" s="2" t="n">
-        <v>4662.452</v>
+        <v>4662.392</v>
       </c>
       <c r="AR36" s="2" t="n">
-        <v>-1.098</v>
+        <v>-1.1108</v>
       </c>
       <c r="AS36" s="2" t="n">
-        <v>-0.0607</v>
+        <v>-0.06710000000000001</v>
       </c>
       <c r="AT36" s="2" t="n">
-        <v>0.3004</v>
+        <v>0.2977</v>
       </c>
       <c r="AU36" s="2" t="n">
-        <v>-0.2017</v>
+        <v>-0.203</v>
       </c>
       <c r="AV36" s="2" t="n">
-        <v>0.3051</v>
+        <v>0.3044</v>
       </c>
     </row>
     <row r="37">
@@ -4951,7 +4949,7 @@
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>7200</v>
+        <v>7164</v>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
@@ -4959,10 +4957,10 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>5.48</v>
+        <v>5.47</v>
       </c>
       <c r="F37" s="2" t="n">
-        <v>22.8</v>
+        <v>22.2</v>
       </c>
       <c r="G37" s="2" t="n">
         <v>98.81999999999999</v>
@@ -4984,32 +4982,28 @@
       <c r="R37" s="2" t="inlineStr"/>
       <c r="S37" s="2" t="inlineStr"/>
       <c r="T37" s="2" t="inlineStr"/>
-      <c r="U37" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="U37" s="2" t="inlineStr"/>
       <c r="V37" s="2" t="inlineStr"/>
       <c r="W37" s="2" t="inlineStr"/>
       <c r="X37" s="2" t="inlineStr"/>
       <c r="Y37" s="2" t="n">
-        <v>56.82</v>
+        <v>56.65</v>
       </c>
       <c r="Z37" s="2" t="n">
-        <v>10.55</v>
+        <v>10.21</v>
       </c>
       <c r="AA37" s="2" t="n"/>
       <c r="AB37" s="2" t="n">
-        <v>-3.73</v>
+        <v>-4.37</v>
       </c>
       <c r="AC37" s="2" t="n">
-        <v>1.52</v>
+        <v>0.17</v>
       </c>
       <c r="AD37" s="2" t="n">
-        <v>101.4</v>
+        <v>101.2</v>
       </c>
       <c r="AE37" s="2" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="AF37" s="2" t="inlineStr"/>
       <c r="AG37" s="2" t="inlineStr"/>
@@ -5023,40 +5017,40 @@
         </is>
       </c>
       <c r="AK37" s="2" t="n">
-        <v>7162.4</v>
+        <v>7155.2</v>
       </c>
       <c r="AL37" s="2" t="n">
-        <v>7225.321</v>
+        <v>7221.721</v>
       </c>
       <c r="AM37" s="2" t="n">
-        <v>7177.358</v>
+        <v>7175.558</v>
       </c>
       <c r="AN37" s="2" t="n">
-        <v>7083.603</v>
+        <v>7082.403</v>
       </c>
       <c r="AO37" s="2" t="n">
-        <v>6647.118</v>
+        <v>6646.398</v>
       </c>
       <c r="AP37" s="2" t="n">
-        <v>5977.02</v>
+        <v>5976.66</v>
       </c>
       <c r="AQ37" s="2" t="n">
-        <v>5617.804</v>
+        <v>5617.624</v>
       </c>
       <c r="AR37" s="2" t="n">
-        <v>0.1265</v>
+        <v>0.1005</v>
       </c>
       <c r="AS37" s="2" t="n">
-        <v>0.4555</v>
+        <v>0.4423</v>
       </c>
       <c r="AT37" s="2" t="n">
-        <v>1.3783</v>
+        <v>1.3725</v>
       </c>
       <c r="AU37" s="2" t="n">
-        <v>0.713</v>
+        <v>0.7098</v>
       </c>
       <c r="AV37" s="2" t="n">
-        <v>0.5682</v>
+        <v>0.5665</v>
       </c>
     </row>
     <row r="38">
@@ -5071,7 +5065,7 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>7107</v>
+        <v>7097</v>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
@@ -5082,7 +5076,7 @@
         <v>5.04</v>
       </c>
       <c r="F38" s="2" t="n">
-        <v>17.5</v>
+        <v>17.3</v>
       </c>
       <c r="G38" s="2" t="n">
         <v>82.55</v>
@@ -5113,23 +5107,23 @@
       <c r="W38" s="2" t="inlineStr"/>
       <c r="X38" s="2" t="inlineStr"/>
       <c r="Y38" s="2" t="n">
-        <v>63.4</v>
+        <v>63.35</v>
       </c>
       <c r="Z38" s="2" t="n">
-        <v>10.76</v>
+        <v>10.75</v>
       </c>
       <c r="AA38" s="2" t="n"/>
       <c r="AB38" s="2" t="n">
-        <v>-3.38</v>
+        <v>-1.96</v>
       </c>
       <c r="AC38" s="2" t="n">
-        <v>-0.51</v>
+        <v>-1.34</v>
       </c>
       <c r="AD38" s="2" t="n">
         <v>97.8</v>
       </c>
       <c r="AE38" s="2" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="AF38" s="2" t="inlineStr"/>
       <c r="AG38" s="2" t="inlineStr"/>
@@ -5143,40 +5137,40 @@
         </is>
       </c>
       <c r="AK38" s="2" t="n">
-        <v>7034.2</v>
+        <v>7032.2</v>
       </c>
       <c r="AL38" s="2" t="n">
-        <v>7070.193</v>
+        <v>7069.193</v>
       </c>
       <c r="AM38" s="2" t="n">
-        <v>7019.173</v>
+        <v>7018.673</v>
       </c>
       <c r="AN38" s="2" t="n">
-        <v>7010.12</v>
+        <v>7009.786</v>
       </c>
       <c r="AO38" s="2" t="n">
-        <v>6600.015</v>
+        <v>6599.815</v>
       </c>
       <c r="AP38" s="2" t="n">
-        <v>6022.698</v>
+        <v>6022.598</v>
       </c>
       <c r="AQ38" s="2" t="n">
-        <v>5698.566</v>
+        <v>5698.516</v>
       </c>
       <c r="AR38" s="2" t="n">
-        <v>0.3452</v>
+        <v>0.3378</v>
       </c>
       <c r="AS38" s="2" t="n">
-        <v>0.1634</v>
+        <v>0.1597</v>
       </c>
       <c r="AT38" s="2" t="n">
-        <v>1.289</v>
+        <v>1.2874</v>
       </c>
       <c r="AU38" s="2" t="n">
-        <v>0.5342</v>
+        <v>0.5333</v>
       </c>
       <c r="AV38" s="2" t="n">
-        <v>0.634</v>
+        <v>0.6335</v>
       </c>
     </row>
     <row r="39">
@@ -5191,7 +5185,7 @@
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>3287</v>
+        <v>3273</v>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
@@ -5202,7 +5196,7 @@
         <v>5.94</v>
       </c>
       <c r="F39" s="2" t="n">
-        <v>20.7</v>
+        <v>20.2</v>
       </c>
       <c r="G39" s="2" t="n">
         <v>89.25</v>
@@ -5229,23 +5223,23 @@
       <c r="W39" s="2" t="inlineStr"/>
       <c r="X39" s="2" t="inlineStr"/>
       <c r="Y39" s="2" t="n">
-        <v>66.61</v>
+        <v>66.47</v>
       </c>
       <c r="Z39" s="2" t="n">
-        <v>12.68</v>
+        <v>12.37</v>
       </c>
       <c r="AA39" s="2" t="n"/>
       <c r="AB39" s="2" t="n">
-        <v>-7.27</v>
+        <v>-7.6</v>
       </c>
       <c r="AC39" s="2" t="n">
-        <v>-3.46</v>
+        <v>-5.77</v>
       </c>
       <c r="AD39" s="2" t="n">
-        <v>89.2</v>
+        <v>89.09999999999999</v>
       </c>
       <c r="AE39" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AF39" s="2" t="inlineStr"/>
       <c r="AG39" s="2" t="inlineStr"/>
@@ -5259,40 +5253,40 @@
         </is>
       </c>
       <c r="AK39" s="2" t="n">
-        <v>3301.4</v>
+        <v>3298.6</v>
       </c>
       <c r="AL39" s="2" t="n">
-        <v>3356.717</v>
+        <v>3355.317</v>
       </c>
       <c r="AM39" s="2" t="n">
-        <v>3338.793</v>
+        <v>3338.093</v>
       </c>
       <c r="AN39" s="2" t="n">
-        <v>3316.674</v>
+        <v>3316.207</v>
       </c>
       <c r="AO39" s="2" t="n">
-        <v>3116.333</v>
+        <v>3116.053</v>
       </c>
       <c r="AP39" s="2" t="n">
-        <v>2814.254</v>
+        <v>2814.114</v>
       </c>
       <c r="AQ39" s="2" t="n">
-        <v>2576.115</v>
+        <v>2576.045</v>
       </c>
       <c r="AR39" s="2" t="n">
-        <v>-0.0852</v>
+        <v>-0.1069</v>
       </c>
       <c r="AS39" s="2" t="n">
-        <v>0.0873</v>
+        <v>0.0764</v>
       </c>
       <c r="AT39" s="2" t="n">
-        <v>1.1958</v>
+        <v>1.191</v>
       </c>
       <c r="AU39" s="2" t="n">
-        <v>0.7687</v>
+        <v>0.766</v>
       </c>
       <c r="AV39" s="2" t="n">
-        <v>0.6661</v>
+        <v>0.6647</v>
       </c>
     </row>
     <row r="40">
@@ -5307,7 +5301,7 @@
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>71460</v>
+        <v>71470</v>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
@@ -5351,17 +5345,17 @@
       <c r="W40" s="2" t="inlineStr"/>
       <c r="X40" s="2" t="inlineStr"/>
       <c r="Y40" s="2" t="n">
-        <v>25.99</v>
+        <v>26</v>
       </c>
       <c r="Z40" s="2" t="n">
-        <v>-8.550000000000001</v>
+        <v>-8.41</v>
       </c>
       <c r="AA40" s="2" t="n"/>
       <c r="AB40" s="2" t="n">
-        <v>0.64</v>
+        <v>0.99</v>
       </c>
       <c r="AC40" s="2" t="n">
-        <v>-3.97</v>
+        <v>-2.42</v>
       </c>
       <c r="AD40" s="2" t="n">
         <v>0.1</v>
@@ -5381,40 +5375,40 @@
         </is>
       </c>
       <c r="AK40" s="2" t="n">
-        <v>70326</v>
+        <v>70328</v>
       </c>
       <c r="AL40" s="2" t="n">
-        <v>69058</v>
+        <v>69059</v>
       </c>
       <c r="AM40" s="2" t="n">
-        <v>68475</v>
+        <v>68475.5</v>
       </c>
       <c r="AN40" s="2" t="n">
-        <v>69864.398</v>
+        <v>69864.731</v>
       </c>
       <c r="AO40" s="2" t="n">
-        <v>73050.36</v>
+        <v>73050.56</v>
       </c>
       <c r="AP40" s="2" t="n">
-        <v>76153.624</v>
+        <v>76153.724</v>
       </c>
       <c r="AQ40" s="2" t="n">
-        <v>69894.004</v>
+        <v>69894.054</v>
       </c>
       <c r="AR40" s="2" t="n">
-        <v>1.3996</v>
+        <v>1.4004</v>
       </c>
       <c r="AS40" s="2" t="n">
-        <v>-0.2403</v>
+        <v>-0.2399</v>
       </c>
       <c r="AT40" s="2" t="n">
-        <v>-0.6207</v>
+        <v>-0.6205000000000001</v>
       </c>
       <c r="AU40" s="2" t="n">
-        <v>-0.1167</v>
+        <v>-0.1166</v>
       </c>
       <c r="AV40" s="2" t="n">
-        <v>0.2599</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="41">
@@ -8041,7 +8035,7 @@
         <v>16.1</v>
       </c>
       <c r="AE62" s="2" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AF62" s="2" t="inlineStr"/>
       <c r="AG62" s="2" t="inlineStr"/>
@@ -15875,7 +15869,7 @@
       <c r="O126" s="2" t="inlineStr"/>
       <c r="P126" s="2" t="inlineStr"/>
       <c r="Q126" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R126" s="2" t="inlineStr"/>
       <c r="S126" s="2" t="inlineStr"/>
@@ -20571,7 +20565,7 @@
         </is>
       </c>
       <c r="C165" s="2" t="n">
-        <v>148.07</v>
+        <v>151.06</v>
       </c>
       <c r="D165" s="2" t="n"/>
       <c r="E165" s="2" t="n"/>
@@ -20596,7 +20590,11 @@
       <c r="R165" s="2" t="inlineStr"/>
       <c r="S165" s="2" t="inlineStr"/>
       <c r="T165" s="2" t="inlineStr"/>
-      <c r="U165" s="2" t="inlineStr"/>
+      <c r="U165" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="V165" s="2" t="inlineStr"/>
       <c r="W165" s="2" t="inlineStr"/>
       <c r="X165" s="2" t="inlineStr"/>
@@ -20613,30 +20611,30 @@
       <c r="AI165" s="2" t="inlineStr"/>
       <c r="AJ165" s="2" t="inlineStr"/>
       <c r="AK165" s="2" t="n">
-        <v>148.464</v>
+        <v>149.062</v>
       </c>
       <c r="AL165" s="2" t="n">
-        <v>149.799</v>
+        <v>150.098</v>
       </c>
       <c r="AM165" s="2" t="n">
-        <v>149.671</v>
+        <v>149.82</v>
       </c>
       <c r="AN165" s="2" t="n">
-        <v>146.199</v>
+        <v>146.299</v>
       </c>
       <c r="AO165" s="2" t="n">
-        <v>138.143</v>
+        <v>138.203</v>
       </c>
       <c r="AP165" s="2" t="n"/>
       <c r="AQ165" s="2" t="n"/>
       <c r="AR165" s="2" t="n">
-        <v>-0.215</v>
+        <v>-0.1117</v>
       </c>
       <c r="AS165" s="2" t="n">
-        <v>0.5853</v>
+        <v>0.6379</v>
       </c>
       <c r="AT165" s="2" t="n">
-        <v>0.9863</v>
+        <v>1.0092</v>
       </c>
       <c r="AU165" s="2" t="n"/>
       <c r="AV165" s="2" t="n"/>
@@ -21720,7 +21718,7 @@
         <v>-16.55</v>
       </c>
       <c r="AD174" s="2" t="n">
-        <v>17.5</v>
+        <v>17.6</v>
       </c>
       <c r="AE174" s="2" t="n">
         <v>31</v>
@@ -22107,7 +22105,7 @@
         <v>72</v>
       </c>
       <c r="AE177" s="2" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="AF177" s="2" t="inlineStr"/>
       <c r="AG177" s="2" t="inlineStr"/>
@@ -22661,7 +22659,7 @@
         </is>
       </c>
       <c r="C182" s="2" t="n">
-        <v>6008</v>
+        <v>5984</v>
       </c>
       <c r="D182" s="2" t="inlineStr">
         <is>
@@ -22672,10 +22670,10 @@
         <v>-3.87</v>
       </c>
       <c r="F182" s="2" t="n">
-        <v>-22.4</v>
+        <v>-22.7</v>
       </c>
       <c r="G182" s="2" t="n">
-        <v>11.56</v>
+        <v>10.56</v>
       </c>
       <c r="H182" s="2" t="inlineStr"/>
       <c r="I182" s="2" t="inlineStr"/>
@@ -22697,23 +22695,23 @@
       <c r="W182" s="2" t="inlineStr"/>
       <c r="X182" s="2" t="inlineStr"/>
       <c r="Y182" s="2" t="n">
-        <v>-30.48</v>
+        <v>-30.56</v>
       </c>
       <c r="Z182" s="2" t="n">
-        <v>-35.91</v>
+        <v>-35.98</v>
       </c>
       <c r="AA182" s="2" t="n"/>
       <c r="AB182" s="2" t="n">
-        <v>-9.5</v>
+        <v>-8.35</v>
       </c>
       <c r="AC182" s="2" t="n">
-        <v>-10.06</v>
+        <v>-10.55</v>
       </c>
       <c r="AD182" s="2" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="AE182" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AF182" s="2" t="inlineStr"/>
       <c r="AG182" s="2" t="n">
@@ -22727,40 +22725,40 @@
         </is>
       </c>
       <c r="AK182" s="2" t="n">
-        <v>6173.2</v>
+        <v>6168.4</v>
       </c>
       <c r="AL182" s="2" t="n">
-        <v>6400.8</v>
+        <v>6398.4</v>
       </c>
       <c r="AM182" s="2" t="n">
-        <v>6491.95</v>
+        <v>6490.75</v>
       </c>
       <c r="AN182" s="2" t="n">
-        <v>6655.033</v>
+        <v>6654.233</v>
       </c>
       <c r="AO182" s="2" t="n">
-        <v>6793.84</v>
+        <v>6793.36</v>
       </c>
       <c r="AP182" s="2" t="n">
-        <v>7168.705</v>
+        <v>7168.465</v>
       </c>
       <c r="AQ182" s="2" t="n">
-        <v>7914.437</v>
+        <v>7914.317</v>
       </c>
       <c r="AR182" s="2" t="n">
-        <v>-1.085</v>
+        <v>-1.1041</v>
       </c>
       <c r="AS182" s="2" t="n">
-        <v>-1.5586</v>
+        <v>-1.568</v>
       </c>
       <c r="AT182" s="2" t="n">
-        <v>-0.7987</v>
+        <v>-0.8023</v>
       </c>
       <c r="AU182" s="2" t="n">
-        <v>-0.6499</v>
+        <v>-0.6516</v>
       </c>
       <c r="AV182" s="2" t="n">
-        <v>-0.3048</v>
+        <v>-0.3056</v>
       </c>
     </row>
     <row r="183">
@@ -22775,7 +22773,7 @@
         </is>
       </c>
       <c r="C183" s="2" t="n">
-        <v>1358.5</v>
+        <v>1360</v>
       </c>
       <c r="D183" s="2" t="inlineStr">
         <is>
@@ -22786,7 +22784,7 @@
         <v>0.77</v>
       </c>
       <c r="F183" s="2" t="n">
-        <v>3.1</v>
+        <v>3.2</v>
       </c>
       <c r="G183" s="2" t="n">
         <v>83.7</v>
@@ -22811,23 +22809,23 @@
       <c r="W183" s="2" t="inlineStr"/>
       <c r="X183" s="2" t="inlineStr"/>
       <c r="Y183" s="2" t="n">
-        <v>36.21</v>
+        <v>36.24</v>
       </c>
       <c r="Z183" s="2" t="n">
-        <v>-6.08</v>
+        <v>-5.84</v>
       </c>
       <c r="AA183" s="2" t="n"/>
       <c r="AB183" s="2" t="n">
-        <v>-7.75</v>
+        <v>-7.17</v>
       </c>
       <c r="AC183" s="2" t="n">
-        <v>-1.15</v>
+        <v>-4.58</v>
       </c>
       <c r="AD183" s="2" t="n">
-        <v>87.5</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="AE183" s="2" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="AF183" s="2" t="inlineStr"/>
       <c r="AG183" s="2" t="inlineStr"/>
@@ -22841,40 +22839,40 @@
         </is>
       </c>
       <c r="AK183" s="2" t="n">
-        <v>1375.3</v>
+        <v>1375.6</v>
       </c>
       <c r="AL183" s="2" t="n">
-        <v>1401.354</v>
+        <v>1401.504</v>
       </c>
       <c r="AM183" s="2" t="n">
-        <v>1394.273</v>
+        <v>1394.348</v>
       </c>
       <c r="AN183" s="2" t="n">
-        <v>1367.211</v>
+        <v>1367.261</v>
       </c>
       <c r="AO183" s="2" t="n">
-        <v>1335.769</v>
+        <v>1335.799</v>
       </c>
       <c r="AP183" s="2" t="n">
-        <v>1294.082</v>
+        <v>1294.097</v>
       </c>
       <c r="AQ183" s="2" t="n">
-        <v>1286.442</v>
+        <v>1286.449</v>
       </c>
       <c r="AR183" s="2" t="n">
-        <v>-0.9173</v>
+        <v>-0.9119</v>
       </c>
       <c r="AS183" s="2" t="n">
-        <v>0.4898</v>
+        <v>0.4926</v>
       </c>
       <c r="AT183" s="2" t="n">
-        <v>0.4969</v>
+        <v>0.4981</v>
       </c>
       <c r="AU183" s="2" t="n">
-        <v>0.1642</v>
+        <v>0.1648</v>
       </c>
       <c r="AV183" s="2" t="n">
-        <v>0.3621</v>
+        <v>0.3624</v>
       </c>
     </row>
     <row r="184">
@@ -22889,7 +22887,7 @@
         </is>
       </c>
       <c r="C184" s="2" t="n">
-        <v>5294</v>
+        <v>5310</v>
       </c>
       <c r="D184" s="2" t="inlineStr">
         <is>
@@ -22900,7 +22898,7 @@
         <v>-0.1</v>
       </c>
       <c r="F184" s="2" t="n">
-        <v>-6.9</v>
+        <v>-6.6</v>
       </c>
       <c r="G184" s="2" t="n">
         <v>1.22</v>
@@ -22925,23 +22923,23 @@
       <c r="W184" s="2" t="inlineStr"/>
       <c r="X184" s="2" t="inlineStr"/>
       <c r="Y184" s="2" t="n">
-        <v>22.7</v>
+        <v>22.78</v>
       </c>
       <c r="Z184" s="2" t="n">
-        <v>-13.8</v>
+        <v>-13.4</v>
       </c>
       <c r="AA184" s="2" t="n"/>
       <c r="AB184" s="2" t="n">
-        <v>-2.95</v>
+        <v>-0.84</v>
       </c>
       <c r="AC184" s="2" t="n">
-        <v>-6.86</v>
+        <v>-5.54</v>
       </c>
       <c r="AD184" s="2" t="n">
-        <v>10</v>
+        <v>10.2</v>
       </c>
       <c r="AE184" s="2" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="AF184" s="2" t="inlineStr"/>
       <c r="AG184" s="2" t="n">
@@ -22955,40 +22953,40 @@
         </is>
       </c>
       <c r="AK184" s="2" t="n">
-        <v>5225</v>
+        <v>5228.2</v>
       </c>
       <c r="AL184" s="2" t="n">
-        <v>5193.859</v>
+        <v>5195.459</v>
       </c>
       <c r="AM184" s="2" t="n">
-        <v>5171.875</v>
+        <v>5172.675</v>
       </c>
       <c r="AN184" s="2" t="n">
-        <v>5304.371</v>
+        <v>5304.905</v>
       </c>
       <c r="AO184" s="2" t="n">
-        <v>5465.43</v>
+        <v>5465.75</v>
       </c>
       <c r="AP184" s="2" t="n">
-        <v>5718.523</v>
+        <v>5718.683</v>
       </c>
       <c r="AQ184" s="2" t="n">
-        <v>5492.156</v>
+        <v>5492.236</v>
       </c>
       <c r="AR184" s="2" t="n">
-        <v>0.772</v>
+        <v>0.7883</v>
       </c>
       <c r="AS184" s="2" t="n">
-        <v>-0.8166</v>
+        <v>-0.8087</v>
       </c>
       <c r="AT184" s="2" t="n">
-        <v>-0.3314</v>
+        <v>-0.3284</v>
       </c>
       <c r="AU184" s="2" t="n">
-        <v>-0.4492</v>
+        <v>-0.4478</v>
       </c>
       <c r="AV184" s="2" t="n">
-        <v>0.227</v>
+        <v>0.2278</v>
       </c>
     </row>
     <row r="185">
@@ -23003,7 +23001,7 @@
         </is>
       </c>
       <c r="C185" s="2" t="n">
-        <v>4750</v>
+        <v>4751</v>
       </c>
       <c r="D185" s="2" t="inlineStr">
         <is>
@@ -23042,14 +23040,14 @@
         <v>10.31</v>
       </c>
       <c r="Z185" s="2" t="n">
-        <v>-19.83</v>
+        <v>-19.71</v>
       </c>
       <c r="AA185" s="2" t="n"/>
       <c r="AB185" s="2" t="n">
-        <v>0.63</v>
+        <v>2.23</v>
       </c>
       <c r="AC185" s="2" t="n">
-        <v>-3.19</v>
+        <v>-1.79</v>
       </c>
       <c r="AD185" s="2" t="n">
         <v>-3.5</v>
@@ -23069,37 +23067,37 @@
         </is>
       </c>
       <c r="AK185" s="2" t="n">
-        <v>4628.6</v>
+        <v>4628.8</v>
       </c>
       <c r="AL185" s="2" t="n">
-        <v>4517.2</v>
+        <v>4517.3</v>
       </c>
       <c r="AM185" s="2" t="n">
-        <v>4483.25</v>
+        <v>4483.3</v>
       </c>
       <c r="AN185" s="2" t="n">
-        <v>4612.644</v>
+        <v>4612.678</v>
       </c>
       <c r="AO185" s="2" t="n">
-        <v>4815.993</v>
+        <v>4816.013</v>
       </c>
       <c r="AP185" s="2" t="n">
-        <v>5765.46</v>
+        <v>5765.47</v>
       </c>
       <c r="AQ185" s="2" t="n">
-        <v>5326.775</v>
+        <v>5326.78</v>
       </c>
       <c r="AR185" s="2" t="n">
-        <v>1.5555</v>
+        <v>1.5567</v>
       </c>
       <c r="AS185" s="2" t="n">
-        <v>-0.521</v>
+        <v>-0.5205</v>
       </c>
       <c r="AT185" s="2" t="n">
-        <v>-0.8835</v>
+        <v>-0.8833</v>
       </c>
       <c r="AU185" s="2" t="n">
-        <v>-0.4831</v>
+        <v>-0.483</v>
       </c>
       <c r="AV185" s="2" t="n">
         <v>0.1031</v>
@@ -23519,7 +23517,7 @@
         <v>19.3</v>
       </c>
       <c r="AE189" s="2" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="AF189" s="2" t="inlineStr"/>
       <c r="AG189" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-04
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -928,7 +928,9 @@
         <v>0</v>
       </c>
       <c r="R3" s="2" t="inlineStr"/>
-      <c r="S3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T3" s="2" t="inlineStr"/>
       <c r="U3" s="2" t="inlineStr"/>
       <c r="V3" s="2" t="n">
@@ -2014,7 +2016,9 @@
         <v>0</v>
       </c>
       <c r="R12" s="2" t="inlineStr"/>
-      <c r="S12" s="2" t="inlineStr"/>
+      <c r="S12" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="T12" s="2" t="inlineStr"/>
       <c r="U12" s="2" t="n">
         <v>1</v>
@@ -2135,7 +2139,9 @@
         <v>1</v>
       </c>
       <c r="S13" s="2" t="inlineStr"/>
-      <c r="T13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U13" s="2" t="inlineStr"/>
       <c r="V13" s="2" t="inlineStr"/>
       <c r="W13" s="2" t="inlineStr"/>
@@ -2253,7 +2259,9 @@
       </c>
       <c r="R14" s="2" t="inlineStr"/>
       <c r="S14" s="2" t="inlineStr"/>
-      <c r="T14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U14" s="2" t="inlineStr"/>
       <c r="V14" s="2" t="inlineStr"/>
       <c r="W14" s="2" t="inlineStr"/>
@@ -2853,7 +2861,9 @@
       </c>
       <c r="R19" s="2" t="inlineStr"/>
       <c r="S19" s="2" t="inlineStr"/>
-      <c r="T19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U19" s="2" t="inlineStr"/>
       <c r="V19" s="2" t="inlineStr"/>
       <c r="W19" s="2" t="inlineStr"/>
@@ -2979,7 +2989,9 @@
       </c>
       <c r="R20" s="2" t="inlineStr"/>
       <c r="S20" s="2" t="inlineStr"/>
-      <c r="T20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U20" s="2" t="inlineStr"/>
       <c r="V20" s="2" t="inlineStr"/>
       <c r="W20" s="2" t="inlineStr"/>
@@ -9701,7 +9713,9 @@
       </c>
       <c r="R76" s="2" t="inlineStr"/>
       <c r="S76" s="2" t="inlineStr"/>
-      <c r="T76" s="2" t="inlineStr"/>
+      <c r="T76" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U76" s="2" t="n">
         <v>1</v>
       </c>
@@ -14765,7 +14779,9 @@
       </c>
       <c r="R117" s="2" t="inlineStr"/>
       <c r="S117" s="2" t="inlineStr"/>
-      <c r="T117" s="2" t="inlineStr"/>
+      <c r="T117" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U117" s="2" t="inlineStr"/>
       <c r="V117" s="2" t="inlineStr"/>
       <c r="W117" s="2" t="inlineStr"/>
@@ -16725,7 +16741,9 @@
       </c>
       <c r="R133" s="2" t="inlineStr"/>
       <c r="S133" s="2" t="inlineStr"/>
-      <c r="T133" s="2" t="inlineStr"/>
+      <c r="T133" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="U133" s="2" t="n">
         <v>-1</v>
       </c>
@@ -20209,7 +20227,7 @@
         <v>35</v>
       </c>
       <c r="G162" s="2" t="n">
-        <v>108.31</v>
+        <v>108.29</v>
       </c>
       <c r="H162" s="2" t="inlineStr"/>
       <c r="I162" s="2" t="inlineStr"/>
@@ -21799,7 +21817,7 @@
         <v>48</v>
       </c>
       <c r="G175" s="2" t="n">
-        <v>114.08</v>
+        <v>114.03</v>
       </c>
       <c r="H175" s="2" t="inlineStr"/>
       <c r="I175" s="2" t="inlineStr">
@@ -24673,7 +24691,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-03 | 197 只</t>
+          <t>截至: 2026-10-04 | 197 只</t>
         </is>
       </c>
     </row>
@@ -24867,14 +24885,14 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置(位置门前): {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。位置门 = A OR B。A: 200日pos&lt;=0.80(200日数据不足回退3个月); B: 近3日 4均线(5/10/15/20)纠缠 max/min-1&lt;5% 且距250日收盘高点回落≥5%(创新高处的平台突破归新高, 不算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发。强度: 放量+RS超额+阳线。捕获纠缠平台突破、次新股底部反强</t>
+          <t xml:space="preserve">  SOS (Sign of Strength, Wyckoff): P1前置: {C&gt;MA5, C&gt;MA10, MA5&gt;MA10}三项比较至少2项为正(排除股价在短期均线下方/空头排列)。强度路径: 放量+RS超额+阳线。无位置门(2026-10-02取消: 原A门200日pos&lt;=0.80/B门均线纠缠+距250日高点回落≥5%/门E Stage 1B-2B 全部移除, 高位/新高处的放量突破同样算SOS)。仙股过滤: 信号K线收盘&lt;0.5(本币)不触发</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
+          <t xml:space="preserve">    阳线path: 中大阳(实体&gt;3% ∨ 收盘较昨收&gt;3%, 覆盖大幅低开高走) + 收盘位于日内上1/3 + 放量(&gt;=2x 20日均量; 海外大盘股池放宽至1.5x) + 当日涨幅较指数超额&gt;=2%(A股沪深300指数000300.SH/HK恒指HSI.HI/美股标普500指数^GSPC, 均首选jianxin真实指数, ETF兜底; 基准缺失时跳过此门)</t>
         </is>
       </c>
     </row>
@@ -24995,42 +25013,42 @@
     <row r="52">
       <c r="A52" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stage (Weinstein Stage Analysis, MA150=30周线为锚):</t>
+          <t xml:space="preserve">  ★ 海外SOS放量门放宽: 大盘股量能结构性平缓, 2×20日均量几乎不可触发(250日统计37%空榜日) → 海外池(US+JP)降为1.5×, HK/A/ETF维持2× (2026-10-03)</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    1=筑底(均线走平,价在其下方/附近徘徊) 1B=筑底末期(价已回均线上方但均线未上弯)</t>
+          <t xml:space="preserve">  Stage (Weinstein Stage Analysis, MA150=30周线为锚):</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    2A=Stage1→2过渡(近20日收盘创60日新高但均线尚未上弯) 2B=趋势运行中(MA150上行)</t>
+          <t xml:space="preserve">    1=筑底(均线走平,价在其下方/附近徘徊) 1B=筑底末期(价已回均线上方但均线未上弯)</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">    3=顶部(此前3月均线上行后走平, 价在其上方震荡) 4=下行(价在下行均线下方)</t>
+          <t xml:space="preserve">    2A=Stage1→2过渡(近20日收盘创60日新高但均线尚未上弯) 2B=趋势运行中(MA150上行)</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  MA150斜率20d%: MA150近20日(约1个月)变化%; 距MA150%: 收盘距MA150百分比(&gt;0=上方)</t>
+          <t xml:space="preserve">    3=顶部(此前3月均线上行后走平, 价在其上方震荡) 4=下行(价在下行均线下方)</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  ★ 美股SOS位置门扩展: A∨B∨(Stage 1B/2A/2B) — 信号K线当日处于筑底末期/Stage1→2过渡/Stage2上行趋势的突破也放行 (门E)</t>
+          <t xml:space="preserve">  MA150斜率20d%: MA150近20日(约1个月)变化%; 距MA150%: 收盘距MA150百分比(&gt;0=上方)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-11
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -1353,7 +1353,7 @@
         <v>9628.039000000001</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>8766.894</v>
+        <v>8766.893</v>
       </c>
       <c r="AR6" s="2" t="n">
         <v>3.5955</v>
@@ -6031,10 +6031,10 @@
         </is>
       </c>
       <c r="AK45" s="2" t="n">
-        <v>238.599</v>
+        <v>238.6</v>
       </c>
       <c r="AL45" s="2" t="n">
-        <v>237.608</v>
+        <v>237.609</v>
       </c>
       <c r="AM45" s="2" t="n">
         <v>242.72</v>
@@ -6052,10 +6052,10 @@
         <v>256.978</v>
       </c>
       <c r="AR45" s="2" t="n">
-        <v>-0.215</v>
+        <v>-0.2149</v>
       </c>
       <c r="AS45" s="2" t="n">
-        <v>-0.9124</v>
+        <v>-0.9123</v>
       </c>
       <c r="AT45" s="2" t="n">
         <v>-0.1222</v>
@@ -9537,7 +9537,7 @@
         <v>-7.3</v>
       </c>
       <c r="G74" s="2" t="n">
-        <v>-9.039999999999999</v>
+        <v>-9.050000000000001</v>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr"/>
@@ -12375,7 +12375,7 @@
       <c r="O97" s="2" t="inlineStr"/>
       <c r="P97" s="2" t="inlineStr"/>
       <c r="Q97" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="R97" s="2" t="inlineStr"/>
       <c r="S97" s="2" t="inlineStr"/>
@@ -12839,7 +12839,7 @@
         <v>-9.6</v>
       </c>
       <c r="G101" s="2" t="n">
-        <v>0.32</v>
+        <v>0.27</v>
       </c>
       <c r="H101" s="2" t="inlineStr">
         <is>
@@ -14239,7 +14239,7 @@
         <v>4.6</v>
       </c>
       <c r="AE112" s="2" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="AF112" s="2" t="inlineStr"/>
       <c r="AG112" s="2" t="inlineStr"/>
@@ -14439,7 +14439,7 @@
         <v>-27.3</v>
       </c>
       <c r="G114" s="2" t="n">
-        <v>-5.2</v>
+        <v>-5.22</v>
       </c>
       <c r="H114" s="2" t="inlineStr"/>
       <c r="I114" s="2" t="inlineStr">
@@ -14914,7 +14914,7 @@
         <v>764.194</v>
       </c>
       <c r="AR117" s="2" t="n">
-        <v>4.1806</v>
+        <v>4.1805</v>
       </c>
       <c r="AS117" s="2" t="n">
         <v>2.1441</v>
@@ -20827,7 +20827,7 @@
         </is>
       </c>
       <c r="C166" s="2" t="n">
-        <v>41.855</v>
+        <v>41.86</v>
       </c>
       <c r="D166" s="2" t="inlineStr">
         <is>
@@ -20872,16 +20872,16 @@
         <v>51.32</v>
       </c>
       <c r="Z166" s="2" t="n">
-        <v>12.2</v>
+        <v>12.22</v>
       </c>
       <c r="AA166" s="2" t="n">
-        <v>-1.48</v>
+        <v>-1.47</v>
       </c>
       <c r="AB166" s="2" t="n">
-        <v>-5.02</v>
+        <v>-5.01</v>
       </c>
       <c r="AC166" s="2" t="n">
-        <v>5.92</v>
+        <v>5.94</v>
       </c>
       <c r="AD166" s="2" t="n">
         <v>99.2</v>
@@ -20905,10 +20905,10 @@
         </is>
       </c>
       <c r="AK166" s="2" t="n">
-        <v>43.243</v>
+        <v>43.244</v>
       </c>
       <c r="AL166" s="2" t="n">
-        <v>42.569</v>
+        <v>42.57</v>
       </c>
       <c r="AM166" s="2" t="n">
         <v>41.166</v>
@@ -20926,16 +20926,16 @@
         <v>32.319</v>
       </c>
       <c r="AR166" s="2" t="n">
-        <v>0.9029</v>
+        <v>0.9035</v>
       </c>
       <c r="AS166" s="2" t="n">
-        <v>1.2917</v>
+        <v>1.292</v>
       </c>
       <c r="AT166" s="2" t="n">
-        <v>2.1197</v>
+        <v>2.1198</v>
       </c>
       <c r="AU166" s="2" t="n">
-        <v>0.8479</v>
+        <v>0.848</v>
       </c>
       <c r="AV166" s="2" t="n">
         <v>0.5132</v>
@@ -24837,7 +24837,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-10 | 197 只</t>
+          <t>截至: 2026-10-11 | 197 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-12
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -1353,7 +1353,7 @@
         <v>9628.039000000001</v>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>8766.893</v>
+        <v>8766.894</v>
       </c>
       <c r="AR6" s="2" t="n">
         <v>3.5955</v>
@@ -4259,7 +4259,7 @@
         <v>2377.445</v>
       </c>
       <c r="AQ30" s="2" t="n">
-        <v>2366.394</v>
+        <v>2366.395</v>
       </c>
       <c r="AR30" s="2" t="n">
         <v>0.709</v>
@@ -5801,7 +5801,7 @@
         <v>42.44</v>
       </c>
       <c r="AM43" s="2" t="n">
-        <v>43.721</v>
+        <v>43.722</v>
       </c>
       <c r="AN43" s="2" t="n">
         <v>45.89</v>
@@ -7547,7 +7547,7 @@
         <v>60.022</v>
       </c>
       <c r="AO57" s="2" t="n">
-        <v>62.848</v>
+        <v>62.847</v>
       </c>
       <c r="AP57" s="2" t="n">
         <v>72.49299999999999</v>
@@ -9605,7 +9605,7 @@
         <v>114.757</v>
       </c>
       <c r="AM74" s="2" t="n">
-        <v>120.274</v>
+        <v>120.273</v>
       </c>
       <c r="AN74" s="2" t="n">
         <v>124.931</v>
@@ -10347,7 +10347,7 @@
         <v>190.052</v>
       </c>
       <c r="AO80" s="2" t="n">
-        <v>209.856</v>
+        <v>209.857</v>
       </c>
       <c r="AP80" s="2" t="n">
         <v>221.47</v>
@@ -10592,7 +10592,7 @@
         <v>54.985</v>
       </c>
       <c r="AP82" s="2" t="n">
-        <v>53.594</v>
+        <v>53.593</v>
       </c>
       <c r="AQ82" s="2" t="n">
         <v>53.226</v>
@@ -12307,7 +12307,7 @@
         <v>147.876</v>
       </c>
       <c r="AM96" s="2" t="n">
-        <v>148.728</v>
+        <v>148.727</v>
       </c>
       <c r="AN96" s="2" t="n">
         <v>148.029</v>
@@ -12423,7 +12423,7 @@
         <v>14.901</v>
       </c>
       <c r="AM97" s="2" t="n">
-        <v>14.968</v>
+        <v>14.967</v>
       </c>
       <c r="AN97" s="2" t="n">
         <v>15.408</v>
@@ -14019,7 +14019,7 @@
         <v>260.303</v>
       </c>
       <c r="AM110" s="2" t="n">
-        <v>264.688</v>
+        <v>264.689</v>
       </c>
       <c r="AN110" s="2" t="n">
         <v>266.528</v>
@@ -14645,7 +14645,7 @@
         <v>119.758</v>
       </c>
       <c r="AM115" s="2" t="n">
-        <v>123.521</v>
+        <v>123.52</v>
       </c>
       <c r="AN115" s="2" t="n">
         <v>126.704</v>
@@ -16251,7 +16251,7 @@
         <v>144.364</v>
       </c>
       <c r="AM128" s="2" t="n">
-        <v>145.781</v>
+        <v>145.78</v>
       </c>
       <c r="AN128" s="2" t="n">
         <v>146.394</v>
@@ -17871,7 +17871,7 @@
         <v>37.98</v>
       </c>
       <c r="AM141" s="2" t="n">
-        <v>39.435</v>
+        <v>39.436</v>
       </c>
       <c r="AN141" s="2" t="n">
         <v>41.415</v>
@@ -20581,7 +20581,7 @@
         <v>29.411</v>
       </c>
       <c r="AM163" s="2" t="n">
-        <v>28.488</v>
+        <v>28.489</v>
       </c>
       <c r="AN163" s="2" t="n">
         <v>25.618</v>
@@ -20712,7 +20712,7 @@
         <v>144.815</v>
       </c>
       <c r="AP164" s="2" t="n">
-        <v>130.28</v>
+        <v>130.281</v>
       </c>
       <c r="AQ164" s="2" t="n">
         <v>129.524</v>
@@ -23857,7 +23857,7 @@
         <v>252.582</v>
       </c>
       <c r="AM190" s="2" t="n">
-        <v>252.02</v>
+        <v>252.019</v>
       </c>
       <c r="AN190" s="2" t="n">
         <v>253.731</v>
@@ -24779,7 +24779,7 @@
         <v>187.529</v>
       </c>
       <c r="AM198" s="2" t="n">
-        <v>189.703</v>
+        <v>189.702</v>
       </c>
       <c r="AN198" s="2" t="n">
         <v>191.377</v>
@@ -24837,7 +24837,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-11 | 197 只</t>
+          <t>截至: 2026-10-12 | 197 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-13
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -845,17 +845,13 @@
       </c>
       <c r="V2" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="X2" s="2" t="inlineStr">
-        <is>
-          <t>9d</t>
-        </is>
-      </c>
+        <v>14</v>
+      </c>
+      <c r="X2" s="2" t="inlineStr"/>
       <c r="Y2" s="2" t="inlineStr"/>
       <c r="Z2" s="2" t="n">
         <v>-1</v>
@@ -1266,11 +1262,11 @@
       </c>
       <c r="V5" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W5" s="2" t="n">
-        <v>2</v>
+        <v>52</v>
       </c>
       <c r="X5" s="2" t="inlineStr"/>
       <c r="Y5" s="2" t="inlineStr"/>
@@ -1546,7 +1542,7 @@
         </is>
       </c>
       <c r="W7" s="2" t="n">
-        <v>44</v>
+        <v>68</v>
       </c>
       <c r="X7" s="2" t="inlineStr"/>
       <c r="Y7" s="2" t="inlineStr"/>
@@ -2219,7 +2215,7 @@
         </is>
       </c>
       <c r="W12" s="2" t="n">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="X12" s="2" t="inlineStr"/>
       <c r="Y12" s="2" t="inlineStr"/>
@@ -2356,11 +2352,11 @@
       </c>
       <c r="V13" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W13" s="2" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="X13" s="2" t="inlineStr">
         <is>
@@ -2507,11 +2503,7 @@
       <c r="W14" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="X14" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
+      <c r="X14" s="2" t="inlineStr"/>
       <c r="Y14" s="2" t="inlineStr"/>
       <c r="Z14" s="2" t="n">
         <v>-1</v>
@@ -3611,7 +3603,7 @@
         </is>
       </c>
       <c r="W22" s="2" t="n">
-        <v>49</v>
+        <v>323</v>
       </c>
       <c r="X22" s="2" t="inlineStr"/>
       <c r="Y22" s="2" t="inlineStr"/>
@@ -4429,7 +4421,7 @@
         </is>
       </c>
       <c r="W28" s="2" t="n">
-        <v>36</v>
+        <v>53</v>
       </c>
       <c r="X28" s="2" t="inlineStr"/>
       <c r="Y28" s="2" t="inlineStr"/>
@@ -4971,7 +4963,7 @@
         </is>
       </c>
       <c r="W32" s="2" t="n">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="X32" s="2" t="inlineStr"/>
       <c r="Y32" s="2" t="inlineStr"/>
@@ -5644,7 +5636,7 @@
         </is>
       </c>
       <c r="W37" s="2" t="n">
-        <v>56</v>
+        <v>342</v>
       </c>
       <c r="X37" s="2" t="inlineStr"/>
       <c r="Y37" s="2" t="inlineStr"/>
@@ -6327,11 +6319,11 @@
       </c>
       <c r="V42" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W42" s="2" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="X42" s="2" t="inlineStr">
         <is>
@@ -7445,7 +7437,7 @@
         </is>
       </c>
       <c r="W50" s="2" t="n">
-        <v>79</v>
+        <v>90</v>
       </c>
       <c r="X50" s="2" t="inlineStr"/>
       <c r="Y50" s="2" t="inlineStr"/>
@@ -8134,11 +8126,11 @@
       </c>
       <c r="V55" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W55" s="2" t="n">
-        <v>1</v>
+        <v>134</v>
       </c>
       <c r="X55" s="2" t="inlineStr"/>
       <c r="Y55" s="2" t="inlineStr"/>
@@ -8273,7 +8265,7 @@
         </is>
       </c>
       <c r="W56" s="2" t="n">
-        <v>19</v>
+        <v>271</v>
       </c>
       <c r="X56" s="2" t="inlineStr"/>
       <c r="Y56" s="2" t="inlineStr"/>
@@ -8692,11 +8684,11 @@
       </c>
       <c r="V59" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W59" s="2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="X59" s="2" t="inlineStr"/>
       <c r="Y59" s="2" t="inlineStr"/>
@@ -8978,7 +8970,7 @@
         </is>
       </c>
       <c r="W61" s="2" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="X61" s="2" t="inlineStr"/>
       <c r="Y61" s="2" t="inlineStr"/>
@@ -9929,7 +9921,7 @@
         </is>
       </c>
       <c r="W68" s="2" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="X68" s="2" t="inlineStr"/>
       <c r="Y68" s="2" t="inlineStr"/>
@@ -10056,17 +10048,13 @@
       </c>
       <c r="V69" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W69" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="X69" s="2" t="inlineStr">
-        <is>
-          <t>2d</t>
-        </is>
-      </c>
+        <v>5</v>
+      </c>
+      <c r="X69" s="2" t="inlineStr"/>
       <c r="Y69" s="2" t="inlineStr"/>
       <c r="Z69" s="2" t="inlineStr"/>
       <c r="AA69" s="2" t="n">
@@ -10203,11 +10191,7 @@
       <c r="W70" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="X70" s="2" t="inlineStr">
-        <is>
-          <t>7d</t>
-        </is>
-      </c>
+      <c r="X70" s="2" t="inlineStr"/>
       <c r="Y70" s="2" t="inlineStr"/>
       <c r="Z70" s="2" t="inlineStr"/>
       <c r="AA70" s="2" t="n">
@@ -10892,11 +10876,7 @@
       <c r="W75" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="X75" s="2" t="inlineStr">
-        <is>
-          <t>8d</t>
-        </is>
-      </c>
+      <c r="X75" s="2" t="inlineStr"/>
       <c r="Y75" s="2" t="inlineStr"/>
       <c r="Z75" s="2" t="n">
         <v>-1</v>
@@ -11029,7 +11009,7 @@
         </is>
       </c>
       <c r="W76" s="2" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="X76" s="2" t="inlineStr"/>
       <c r="Y76" s="2" t="inlineStr"/>
@@ -12288,7 +12268,7 @@
         </is>
       </c>
       <c r="W85" s="2" t="n">
-        <v>193</v>
+        <v>356</v>
       </c>
       <c r="X85" s="2" t="inlineStr"/>
       <c r="Y85" s="2" t="inlineStr"/>
@@ -12562,7 +12542,7 @@
         </is>
       </c>
       <c r="W87" s="2" t="n">
-        <v>19</v>
+        <v>80</v>
       </c>
       <c r="X87" s="2" t="inlineStr"/>
       <c r="Y87" s="2" t="inlineStr"/>
@@ -12693,7 +12673,7 @@
         </is>
       </c>
       <c r="W88" s="2" t="n">
-        <v>52</v>
+        <v>59</v>
       </c>
       <c r="X88" s="2" t="inlineStr"/>
       <c r="Y88" s="2" t="inlineStr"/>
@@ -12969,7 +12949,7 @@
         </is>
       </c>
       <c r="W90" s="2" t="n">
-        <v>193</v>
+        <v>308</v>
       </c>
       <c r="X90" s="2" t="inlineStr"/>
       <c r="Y90" s="2" t="inlineStr"/>
@@ -13787,13 +13767,9 @@
         </is>
       </c>
       <c r="W96" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="X96" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
+        <v>21</v>
+      </c>
+      <c r="X96" s="2" t="inlineStr"/>
       <c r="Y96" s="2" t="inlineStr"/>
       <c r="Z96" s="2" t="n">
         <v>-1</v>
@@ -14496,7 +14472,7 @@
         </is>
       </c>
       <c r="W101" s="2" t="n">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="X101" s="2" t="inlineStr"/>
       <c r="Y101" s="2" t="inlineStr"/>
@@ -15322,11 +15298,11 @@
       </c>
       <c r="V107" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W107" s="2" t="n">
-        <v>2</v>
+        <v>90</v>
       </c>
       <c r="X107" s="2" t="inlineStr"/>
       <c r="Y107" s="2" t="inlineStr"/>
@@ -15866,11 +15842,11 @@
       </c>
       <c r="V111" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W111" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="X111" s="2" t="inlineStr"/>
       <c r="Y111" s="2" t="inlineStr"/>
@@ -16168,7 +16144,7 @@
         </is>
       </c>
       <c r="W113" s="2" t="n">
-        <v>37</v>
+        <v>130</v>
       </c>
       <c r="X113" s="2" t="inlineStr"/>
       <c r="Y113" s="2" t="inlineStr"/>
@@ -16593,7 +16569,7 @@
         </is>
       </c>
       <c r="W116" s="2" t="n">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="X116" s="2" t="inlineStr"/>
       <c r="Y116" s="2" t="inlineStr"/>
@@ -17701,11 +17677,11 @@
       </c>
       <c r="V124" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="W124" s="2" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="X124" s="2" t="inlineStr"/>
       <c r="Y124" s="2" t="inlineStr"/>
@@ -18815,7 +18791,7 @@
         </is>
       </c>
       <c r="W132" s="2" t="n">
-        <v>52</v>
+        <v>151</v>
       </c>
       <c r="X132" s="2" t="inlineStr"/>
       <c r="Y132" s="2" t="inlineStr"/>
@@ -19526,7 +19502,7 @@
         </is>
       </c>
       <c r="W137" s="2" t="n">
-        <v>51</v>
+        <v>66</v>
       </c>
       <c r="X137" s="2" t="inlineStr"/>
       <c r="Y137" s="2" t="inlineStr"/>
@@ -19955,7 +19931,7 @@
         </is>
       </c>
       <c r="W140" s="2" t="n">
-        <v>52</v>
+        <v>326</v>
       </c>
       <c r="X140" s="2" t="inlineStr"/>
       <c r="Y140" s="2" t="inlineStr"/>
@@ -20243,7 +20219,7 @@
         </is>
       </c>
       <c r="W142" s="2" t="n">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="X142" s="2" t="inlineStr"/>
       <c r="Y142" s="2" t="inlineStr"/>
@@ -21339,7 +21315,7 @@
         </is>
       </c>
       <c r="W150" s="2" t="n">
-        <v>198</v>
+        <v>237</v>
       </c>
       <c r="X150" s="2" t="inlineStr"/>
       <c r="Y150" s="2" t="inlineStr"/>
@@ -21754,7 +21730,7 @@
         </is>
       </c>
       <c r="W153" s="2" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="X153" s="2" t="inlineStr"/>
       <c r="Y153" s="2" t="inlineStr"/>
@@ -22443,7 +22419,7 @@
         </is>
       </c>
       <c r="W158" s="2" t="n">
-        <v>203</v>
+        <v>316</v>
       </c>
       <c r="X158" s="2" t="inlineStr"/>
       <c r="Y158" s="2" t="inlineStr"/>
@@ -23132,7 +23108,7 @@
         </is>
       </c>
       <c r="W163" s="2" t="n">
-        <v>24</v>
+        <v>197</v>
       </c>
       <c r="X163" s="2" t="inlineStr"/>
       <c r="Y163" s="2" t="inlineStr"/>
@@ -24355,11 +24331,11 @@
       </c>
       <c r="V172" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W172" s="2" t="n">
-        <v>2</v>
+        <v>81</v>
       </c>
       <c r="X172" s="2" t="inlineStr"/>
       <c r="Y172" s="2" t="inlineStr"/>
@@ -24506,7 +24482,7 @@
         </is>
       </c>
       <c r="W173" s="2" t="n">
-        <v>52</v>
+        <v>349</v>
       </c>
       <c r="X173" s="2" t="inlineStr"/>
       <c r="Y173" s="2" t="inlineStr"/>
@@ -25890,11 +25866,11 @@
       </c>
       <c r="V183" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="W183" s="2" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="X183" s="2" t="inlineStr"/>
       <c r="Y183" s="2" t="inlineStr"/>
@@ -26307,13 +26283,9 @@
         </is>
       </c>
       <c r="W186" s="2" t="n">
-        <v>10</v>
-      </c>
-      <c r="X186" s="2" t="inlineStr">
-        <is>
-          <t>10d</t>
-        </is>
-      </c>
+        <v>273</v>
+      </c>
+      <c r="X186" s="2" t="inlineStr"/>
       <c r="Y186" s="2" t="inlineStr"/>
       <c r="Z186" s="2" t="inlineStr"/>
       <c r="AA186" s="2" t="inlineStr"/>
@@ -26440,11 +26412,7 @@
       <c r="W187" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="X187" s="2" t="inlineStr">
-        <is>
-          <t>9d</t>
-        </is>
-      </c>
+      <c r="X187" s="2" t="inlineStr"/>
       <c r="Y187" s="2" t="inlineStr"/>
       <c r="Z187" s="2" t="inlineStr"/>
       <c r="AA187" s="2" t="inlineStr"/>
@@ -26569,7 +26537,7 @@
         </is>
       </c>
       <c r="W188" s="2" t="n">
-        <v>79</v>
+        <v>89</v>
       </c>
       <c r="X188" s="2" t="inlineStr"/>
       <c r="Y188" s="2" t="inlineStr"/>
@@ -26956,11 +26924,11 @@
       </c>
       <c r="V191" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="W191" s="2" t="n">
-        <v>1</v>
+        <v>46</v>
       </c>
       <c r="X191" s="2" t="inlineStr"/>
       <c r="Y191" s="2" t="inlineStr"/>
@@ -27349,13 +27317,9 @@
         </is>
       </c>
       <c r="W194" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="X194" s="2" t="inlineStr">
-        <is>
-          <t>5d</t>
-        </is>
-      </c>
+        <v>12</v>
+      </c>
+      <c r="X194" s="2" t="inlineStr"/>
       <c r="Y194" s="2" t="inlineStr"/>
       <c r="Z194" s="2" t="inlineStr"/>
       <c r="AA194" s="2" t="inlineStr"/>
@@ -27484,13 +27448,9 @@
         </is>
       </c>
       <c r="W195" s="2" t="n">
-        <v>7</v>
-      </c>
-      <c r="X195" s="2" t="inlineStr">
-        <is>
-          <t>7d</t>
-        </is>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="X195" s="2" t="inlineStr"/>
       <c r="Y195" s="2" t="inlineStr"/>
       <c r="Z195" s="2" t="inlineStr"/>
       <c r="AA195" s="2" t="inlineStr"/>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-16
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -823,7 +823,7 @@
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>2722.5</v>
+        <v>2667.5</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>14.39</v>
@@ -889,20 +889,20 @@
       <c r="AE2" s="2" t="inlineStr"/>
       <c r="AF2" s="2" t="inlineStr"/>
       <c r="AG2" s="2" t="n">
-        <v>80.36</v>
+        <v>79.84</v>
       </c>
       <c r="AH2" s="2" t="n">
-        <v>0.72</v>
+        <v>-1.29</v>
       </c>
       <c r="AI2" s="2" t="n"/>
       <c r="AJ2" s="2" t="n">
-        <v>-21.97</v>
+        <v>-23.98</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>-12.39</v>
+        <v>-14.39</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>2.5</v>
+        <v>2.3</v>
       </c>
       <c r="AM2" s="2" t="n">
         <v>11</v>
@@ -923,40 +923,40 @@
         </is>
       </c>
       <c r="AS2" s="2" t="n">
-        <v>3002</v>
+        <v>2991</v>
       </c>
       <c r="AT2" s="2" t="n">
-        <v>3312.6</v>
+        <v>3307.1</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>3198.925</v>
+        <v>3196.175</v>
       </c>
       <c r="AV2" s="2" t="n">
-        <v>3173.317</v>
+        <v>3171.483</v>
       </c>
       <c r="AW2" s="2" t="n">
-        <v>3334.87</v>
+        <v>3333.77</v>
       </c>
       <c r="AX2" s="2" t="n">
-        <v>3678.957</v>
+        <v>3678.407</v>
       </c>
       <c r="AY2" s="2" t="n">
-        <v>2784.444</v>
+        <v>2784.169</v>
       </c>
       <c r="AZ2" s="2" t="n">
-        <v>-1.4571</v>
+        <v>-1.541</v>
       </c>
       <c r="BA2" s="2" t="n">
-        <v>-0.0633</v>
+        <v>-0.108</v>
       </c>
       <c r="BB2" s="2" t="n">
-        <v>-0.3266</v>
+        <v>-0.3437</v>
       </c>
       <c r="BC2" s="2" t="n">
-        <v>-0.0128</v>
+        <v>-0.0205</v>
       </c>
       <c r="BD2" s="2" t="n">
-        <v>0.8036</v>
+        <v>0.7984</v>
       </c>
     </row>
     <row r="3">
@@ -971,7 +971,7 @@
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>15465</v>
+        <v>15205</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>89.05</v>
@@ -994,20 +994,20 @@
         <v>-9</v>
       </c>
       <c r="N3" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O3" s="2" t="inlineStr"/>
       <c r="P3" s="2" t="inlineStr"/>
       <c r="Q3" s="2" t="inlineStr"/>
       <c r="R3" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S3" s="2" t="n">
         <v>4</v>
       </c>
       <c r="T3" s="2" t="inlineStr">
         <is>
-          <t>0110111100</t>
+          <t>0110011100</t>
         </is>
       </c>
       <c r="U3" s="2" t="inlineStr">
@@ -1045,23 +1045,23 @@
       </c>
       <c r="AF3" s="2" t="inlineStr"/>
       <c r="AG3" s="2" t="n">
-        <v>97.34</v>
+        <v>96.84</v>
       </c>
       <c r="AH3" s="2" t="n">
-        <v>18.79</v>
+        <v>16.83</v>
       </c>
       <c r="AI3" s="2" t="n"/>
       <c r="AJ3" s="2" t="n">
-        <v>-10.06</v>
+        <v>-12.02</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>6.3</v>
+        <v>4.34</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>56.5</v>
+        <v>55.9</v>
       </c>
       <c r="AM3" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AN3" s="2" t="inlineStr"/>
       <c r="AO3" s="2" t="inlineStr"/>
@@ -1073,40 +1073,40 @@
         </is>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>16161</v>
+        <v>16109</v>
       </c>
       <c r="AT3" s="2" t="n">
-        <v>16953.5</v>
+        <v>16927.5</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>15668.612</v>
+        <v>15655.612</v>
       </c>
       <c r="AV3" s="2" t="n">
-        <v>15595.575</v>
+        <v>15586.908</v>
       </c>
       <c r="AW3" s="2" t="n">
-        <v>15799.745</v>
+        <v>15794.545</v>
       </c>
       <c r="AX3" s="2" t="n">
-        <v>16256.572</v>
+        <v>16253.972</v>
       </c>
       <c r="AY3" s="2" t="n">
-        <v>13604.666</v>
+        <v>13603.366</v>
       </c>
       <c r="AZ3" s="2" t="n">
-        <v>2.195</v>
+        <v>2.1119</v>
       </c>
       <c r="BA3" s="2" t="n">
-        <v>0.898</v>
+        <v>0.8541</v>
       </c>
       <c r="BB3" s="2" t="n">
-        <v>1.1007</v>
+        <v>1.0832</v>
       </c>
       <c r="BC3" s="2" t="n">
-        <v>-0.0832</v>
+        <v>-0.0915</v>
       </c>
       <c r="BD3" s="2" t="n">
-        <v>0.9734</v>
+        <v>0.9684</v>
       </c>
     </row>
     <row r="4">
@@ -1121,7 +1121,7 @@
         </is>
       </c>
       <c r="C4" s="2" t="n">
-        <v>9627</v>
+        <v>9607</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>107.99</v>
@@ -1191,20 +1191,20 @@
       <c r="AE4" s="2" t="inlineStr"/>
       <c r="AF4" s="2" t="inlineStr"/>
       <c r="AG4" s="2" t="n">
-        <v>130.25</v>
+        <v>130.18</v>
       </c>
       <c r="AH4" s="2" t="n">
-        <v>38.79</v>
+        <v>38.53</v>
       </c>
       <c r="AI4" s="2" t="n"/>
       <c r="AJ4" s="2" t="n">
-        <v>-26.11</v>
+        <v>-26.37</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>-17.21</v>
+        <v>-17.47</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>61.1</v>
+        <v>61</v>
       </c>
       <c r="AM4" s="2" t="n">
         <v>12</v>
@@ -1223,40 +1223,40 @@
         </is>
       </c>
       <c r="AS4" s="2" t="n">
-        <v>10294</v>
+        <v>10290</v>
       </c>
       <c r="AT4" s="2" t="n">
-        <v>11231.5</v>
+        <v>11229.5</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>10917.029</v>
+        <v>10916.029</v>
       </c>
       <c r="AV4" s="2" t="n">
-        <v>10686.014</v>
+        <v>10685.347</v>
       </c>
       <c r="AW4" s="2" t="n">
-        <v>10341.916</v>
+        <v>10341.516</v>
       </c>
       <c r="AX4" s="2" t="n">
-        <v>10262.627</v>
+        <v>10262.427</v>
       </c>
       <c r="AY4" s="2" t="n">
-        <v>7453.667</v>
+        <v>7453.567</v>
       </c>
       <c r="AZ4" s="2" t="n">
-        <v>-2.3735</v>
+        <v>-2.3824</v>
       </c>
       <c r="BA4" s="2" t="n">
-        <v>0.1752</v>
+        <v>0.1705</v>
       </c>
       <c r="BB4" s="2" t="n">
-        <v>1.432</v>
+        <v>1.4299</v>
       </c>
       <c r="BC4" s="2" t="n">
-        <v>0.5872000000000001</v>
+        <v>0.5861</v>
       </c>
       <c r="BD4" s="2" t="n">
-        <v>1.3025</v>
+        <v>1.3018</v>
       </c>
     </row>
     <row r="5">
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="C5" s="2" t="n">
-        <v>6046</v>
+        <v>6026</v>
       </c>
       <c r="D5" s="2" t="n">
         <v>18.68</v>
@@ -1323,7 +1323,7 @@
       <c r="Y5" s="2" t="inlineStr"/>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>3→4·5d ← 1→3·8d</t>
+          <t>4+→4·2d ← 4→4+·3d ← 3→4·5d</t>
         </is>
       </c>
       <c r="AA5" s="2" t="inlineStr"/>
@@ -1339,23 +1339,23 @@
       </c>
       <c r="AF5" s="2" t="inlineStr"/>
       <c r="AG5" s="2" t="n">
-        <v>27.81</v>
+        <v>27.73</v>
       </c>
       <c r="AH5" s="2" t="n">
-        <v>-8.85</v>
+        <v>-9.130000000000001</v>
       </c>
       <c r="AI5" s="2" t="n"/>
       <c r="AJ5" s="2" t="n">
-        <v>3.75</v>
+        <v>3.48</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>2.76</v>
+        <v>2.48</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>14.2</v>
+        <v>14.1</v>
       </c>
       <c r="AM5" s="2" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="AN5" s="2" t="inlineStr"/>
       <c r="AO5" s="2" t="n">
@@ -1373,40 +1373,40 @@
         </is>
       </c>
       <c r="AS5" s="2" t="n">
-        <v>6068.2</v>
+        <v>6064.2</v>
       </c>
       <c r="AT5" s="2" t="n">
-        <v>6126.5</v>
+        <v>6124.5</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>5978.545</v>
+        <v>5977.545</v>
       </c>
       <c r="AV5" s="2" t="n">
-        <v>5911.45</v>
+        <v>5910.783</v>
       </c>
       <c r="AW5" s="2" t="n">
-        <v>5992.289</v>
+        <v>5991.889</v>
       </c>
       <c r="AX5" s="2" t="n">
-        <v>6527.814</v>
+        <v>6527.614</v>
       </c>
       <c r="AY5" s="2" t="n">
-        <v>6261.537</v>
+        <v>6261.437</v>
       </c>
       <c r="AZ5" s="2" t="n">
-        <v>0.8254</v>
+        <v>0.8081</v>
       </c>
       <c r="BA5" s="2" t="n">
-        <v>0.7806999999999999</v>
+        <v>0.7719</v>
       </c>
       <c r="BB5" s="2" t="n">
-        <v>0.2052</v>
+        <v>0.2017</v>
       </c>
       <c r="BC5" s="2" t="n">
-        <v>-0.3475</v>
+        <v>-0.349</v>
       </c>
       <c r="BD5" s="2" t="n">
-        <v>0.2781</v>
+        <v>0.2773</v>
       </c>
     </row>
     <row r="6">
@@ -1421,7 +1421,7 @@
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>8356</v>
+        <v>8326</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>70.48999999999999</v>
@@ -1447,7 +1447,7 @@
         <v>0</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T6" s="2" t="inlineStr">
         <is>
@@ -1456,7 +1456,7 @@
       </c>
       <c r="U6" s="2" t="inlineStr">
         <is>
-          <t>0010000000</t>
+          <t>0010000010</t>
         </is>
       </c>
       <c r="V6" s="2" t="inlineStr">
@@ -1485,20 +1485,20 @@
       </c>
       <c r="AF6" s="2" t="inlineStr"/>
       <c r="AG6" s="2" t="n">
-        <v>45.18</v>
+        <v>45.09</v>
       </c>
       <c r="AH6" s="2" t="n">
-        <v>-7.16</v>
+        <v>-7.47</v>
       </c>
       <c r="AI6" s="2" t="n"/>
       <c r="AJ6" s="2" t="n">
-        <v>-6.07</v>
+        <v>-6.38</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>0.98</v>
+        <v>0.67</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>22.6</v>
+        <v>22.5</v>
       </c>
       <c r="AM6" s="2" t="n">
         <v>15</v>
@@ -1519,40 +1519,40 @@
         </is>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>8762</v>
+        <v>8756</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>8992.9</v>
+        <v>8989.9</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8640.85</v>
+        <v>8639.35</v>
       </c>
       <c r="AV6" s="2" t="n">
-        <v>8505.433000000001</v>
+        <v>8504.433000000001</v>
       </c>
       <c r="AW6" s="2" t="n">
-        <v>8704.959999999999</v>
+        <v>8704.360000000001</v>
       </c>
       <c r="AX6" s="2" t="n">
-        <v>9564.022999999999</v>
+        <v>9563.723</v>
       </c>
       <c r="AY6" s="2" t="n">
-        <v>8825.906999999999</v>
+        <v>8825.757</v>
       </c>
       <c r="AZ6" s="2" t="n">
-        <v>0.7812</v>
+        <v>0.7635999999999999</v>
       </c>
       <c r="BA6" s="2" t="n">
-        <v>0.9348</v>
+        <v>0.9257</v>
       </c>
       <c r="BB6" s="2" t="n">
-        <v>-0.0911</v>
+        <v>-0.09470000000000001</v>
       </c>
       <c r="BC6" s="2" t="n">
-        <v>-0.4201</v>
+        <v>-0.4217</v>
       </c>
       <c r="BD6" s="2" t="n">
-        <v>0.4518</v>
+        <v>0.4509</v>
       </c>
     </row>
     <row r="7">
@@ -1567,7 +1567,7 @@
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>6242</v>
+        <v>6279</v>
       </c>
       <c r="D7" s="2" t="n">
         <v>75.40000000000001</v>
@@ -1592,7 +1592,7 @@
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="2" t="inlineStr"/>
       <c r="N7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O7" s="2" t="inlineStr"/>
       <c r="P7" s="2" t="inlineStr"/>
@@ -1645,20 +1645,20 @@
       <c r="AE7" s="2" t="inlineStr"/>
       <c r="AF7" s="2" t="inlineStr"/>
       <c r="AG7" s="2" t="n">
-        <v>41.65</v>
+        <v>41.84</v>
       </c>
       <c r="AH7" s="2" t="n">
-        <v>8.93</v>
+        <v>9.6</v>
       </c>
       <c r="AI7" s="2" t="n"/>
       <c r="AJ7" s="2" t="n">
-        <v>12.59</v>
+        <v>13.26</v>
       </c>
       <c r="AK7" s="2" t="n">
-        <v>8.07</v>
+        <v>8.74</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>98.7</v>
+        <v>99</v>
       </c>
       <c r="AM7" s="2" t="n">
         <v>89</v>
@@ -1675,40 +1675,40 @@
         </is>
       </c>
       <c r="AS7" s="2" t="n">
-        <v>6024</v>
+        <v>6031.4</v>
       </c>
       <c r="AT7" s="2" t="n">
-        <v>5870.3</v>
+        <v>5874</v>
       </c>
       <c r="AU7" s="2" t="n">
-        <v>5831.652</v>
+        <v>5833.502</v>
       </c>
       <c r="AV7" s="2" t="n">
-        <v>5772.842</v>
+        <v>5774.076</v>
       </c>
       <c r="AW7" s="2" t="n">
-        <v>5678.129</v>
+        <v>5678.869</v>
       </c>
       <c r="AX7" s="2" t="n">
-        <v>5406.608</v>
+        <v>5406.978</v>
       </c>
       <c r="AY7" s="2" t="n">
-        <v>5332.04</v>
+        <v>5332.225</v>
       </c>
       <c r="AZ7" s="2" t="n">
-        <v>1.0627</v>
+        <v>1.0962</v>
       </c>
       <c r="BA7" s="2" t="n">
-        <v>0.9877</v>
+        <v>1.0045</v>
       </c>
       <c r="BB7" s="2" t="n">
-        <v>0.3728</v>
+        <v>0.3796</v>
       </c>
       <c r="BC7" s="2" t="n">
-        <v>0.4223</v>
+        <v>0.4258</v>
       </c>
       <c r="BD7" s="2" t="n">
-        <v>0.4165</v>
+        <v>0.4184</v>
       </c>
     </row>
     <row r="8">
@@ -1723,7 +1723,7 @@
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>2402.5</v>
+        <v>2428</v>
       </c>
       <c r="D8" s="2" t="n">
         <v>39.9</v>
@@ -1746,19 +1746,19 @@
         <v>1</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T8" s="2" t="inlineStr">
         <is>
-          <t>1111101101</t>
+          <t>1111111101</t>
         </is>
       </c>
       <c r="U8" s="2" t="inlineStr">
         <is>
-          <t>1111101101</t>
+          <t>1111111101</t>
         </is>
       </c>
       <c r="V8" s="2" t="inlineStr">
@@ -1793,25 +1793,29 @@
       <c r="AE8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AF8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
+      </c>
       <c r="AG8" s="2" t="n">
-        <v>16.76</v>
+        <v>17.05</v>
       </c>
       <c r="AH8" s="2" t="n">
-        <v>-0.99</v>
+        <v>0.08</v>
       </c>
       <c r="AI8" s="2" t="n"/>
       <c r="AJ8" s="2" t="n">
-        <v>11.02</v>
+        <v>12.1</v>
       </c>
       <c r="AK8" s="2" t="n">
-        <v>3.36</v>
+        <v>4.43</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>74.8</v>
+        <v>75.3</v>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="AN8" s="2" t="inlineStr"/>
       <c r="AO8" s="2" t="inlineStr"/>
@@ -1825,40 +1829,40 @@
         </is>
       </c>
       <c r="AS8" s="2" t="n">
-        <v>2313.9</v>
+        <v>2319</v>
       </c>
       <c r="AT8" s="2" t="n">
-        <v>2279.65</v>
+        <v>2282.2</v>
       </c>
       <c r="AU8" s="2" t="n">
-        <v>2296.516</v>
+        <v>2297.791</v>
       </c>
       <c r="AV8" s="2" t="n">
-        <v>2289.794</v>
+        <v>2290.644</v>
       </c>
       <c r="AW8" s="2" t="n">
-        <v>2290.679</v>
+        <v>2291.189</v>
       </c>
       <c r="AX8" s="2" t="n">
-        <v>2212.094</v>
+        <v>2212.349</v>
       </c>
       <c r="AY8" s="2" t="n">
-        <v>2260.002</v>
+        <v>2260.129</v>
       </c>
       <c r="AZ8" s="2" t="n">
-        <v>-0.06320000000000001</v>
+        <v>-0.0051</v>
       </c>
       <c r="BA8" s="2" t="n">
-        <v>0.5534</v>
+        <v>0.5825</v>
       </c>
       <c r="BB8" s="2" t="n">
-        <v>0.2428</v>
+        <v>0.2544</v>
       </c>
       <c r="BC8" s="2" t="n">
-        <v>0.059</v>
+        <v>0.065</v>
       </c>
       <c r="BD8" s="2" t="n">
-        <v>0.1676</v>
+        <v>0.1705</v>
       </c>
     </row>
     <row r="9">
@@ -1873,7 +1877,7 @@
         </is>
       </c>
       <c r="C9" s="2" t="n">
-        <v>6357</v>
+        <v>6404</v>
       </c>
       <c r="D9" s="2" t="n">
         <v>2.93</v>
@@ -1888,7 +1892,7 @@
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O9" s="2" t="inlineStr"/>
       <c r="P9" s="2" t="inlineStr"/>
@@ -1921,13 +1925,17 @@
       </c>
       <c r="X9" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y9" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y9" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z9" s="2" t="inlineStr">
         <is>
-          <t>4+→4·1d ← 4→4+·2d</t>
+          <t>4→4+·2d ← 4+→4·16d ← 4→4+·17d</t>
         </is>
       </c>
       <c r="AA9" s="2" t="inlineStr"/>
@@ -1941,23 +1949,23 @@
       </c>
       <c r="AF9" s="2" t="inlineStr"/>
       <c r="AG9" s="2" t="n">
-        <v>-32.77</v>
+        <v>-32.62</v>
       </c>
       <c r="AH9" s="2" t="n">
-        <v>-28.08</v>
+        <v>-27.53</v>
       </c>
       <c r="AI9" s="2" t="n"/>
       <c r="AJ9" s="2" t="n">
-        <v>6.76</v>
+        <v>7.31</v>
       </c>
       <c r="AK9" s="2" t="n">
-        <v>-0.82</v>
+        <v>-0.27</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>8.5</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AM9" s="2" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="AN9" s="2" t="inlineStr">
         <is>
@@ -1975,40 +1983,40 @@
         </is>
       </c>
       <c r="AS9" s="2" t="n">
-        <v>6170.6</v>
+        <v>6180</v>
       </c>
       <c r="AT9" s="2" t="n">
-        <v>6130.2</v>
+        <v>6134.9</v>
       </c>
       <c r="AU9" s="2" t="n">
-        <v>6290.1</v>
+        <v>6292.45</v>
       </c>
       <c r="AV9" s="2" t="n">
-        <v>6402.233</v>
+        <v>6403.8</v>
       </c>
       <c r="AW9" s="2" t="n">
-        <v>6614.72</v>
+        <v>6615.66</v>
       </c>
       <c r="AX9" s="2" t="n">
-        <v>7016.541</v>
+        <v>7017.011</v>
       </c>
       <c r="AY9" s="2" t="n">
-        <v>7827.325</v>
+        <v>7827.56</v>
       </c>
       <c r="AZ9" s="2" t="n">
-        <v>-0.5215</v>
+        <v>-0.482</v>
       </c>
       <c r="BA9" s="2" t="n">
-        <v>-0.576</v>
+        <v>-0.5567</v>
       </c>
       <c r="BB9" s="2" t="n">
-        <v>-0.6315</v>
+        <v>-0.6242</v>
       </c>
       <c r="BC9" s="2" t="n">
-        <v>-0.6072</v>
+        <v>-0.6038</v>
       </c>
       <c r="BD9" s="2" t="n">
-        <v>-0.3277</v>
+        <v>-0.3262</v>
       </c>
     </row>
     <row r="10">
@@ -2023,7 +2031,7 @@
         </is>
       </c>
       <c r="C10" s="2" t="n">
-        <v>2731.5</v>
+        <v>2753</v>
       </c>
       <c r="D10" s="2" t="n">
         <v>98.16</v>
@@ -2046,14 +2054,14 @@
       <c r="P10" s="2" t="inlineStr"/>
       <c r="Q10" s="2" t="inlineStr"/>
       <c r="R10" s="2" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>4</v>
       </c>
       <c r="T10" s="2" t="inlineStr">
         <is>
-          <t>0100101100</t>
+          <t>0101101100</t>
         </is>
       </c>
       <c r="U10" s="2" t="inlineStr">
@@ -2093,23 +2101,23 @@
       <c r="AE10" s="2" t="inlineStr"/>
       <c r="AF10" s="2" t="inlineStr"/>
       <c r="AG10" s="2" t="n">
-        <v>-30.75</v>
+        <v>-30.55</v>
       </c>
       <c r="AH10" s="2" t="n">
-        <v>-19.3</v>
+        <v>-18.65</v>
       </c>
       <c r="AI10" s="2" t="n"/>
       <c r="AJ10" s="2" t="n">
-        <v>7.16</v>
+        <v>7.81</v>
       </c>
       <c r="AK10" s="2" t="n">
-        <v>-0.23</v>
+        <v>0.42</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>57.6</v>
+        <v>58.3</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="AN10" s="2" t="inlineStr"/>
       <c r="AO10" s="2" t="inlineStr"/>
@@ -2127,40 +2135,40 @@
         </is>
       </c>
       <c r="AS10" s="2" t="n">
-        <v>2648.5</v>
+        <v>2652.8</v>
       </c>
       <c r="AT10" s="2" t="n">
-        <v>2677.55</v>
+        <v>2679.7</v>
       </c>
       <c r="AU10" s="2" t="n">
-        <v>2747.23</v>
+        <v>2748.305</v>
       </c>
       <c r="AV10" s="2" t="n">
-        <v>2745.235</v>
+        <v>2745.952</v>
       </c>
       <c r="AW10" s="2" t="n">
-        <v>2732.009</v>
+        <v>2732.439</v>
       </c>
       <c r="AX10" s="2" t="n">
-        <v>2666.455</v>
+        <v>2666.67</v>
       </c>
       <c r="AY10" s="2" t="n">
-        <v>2774.757</v>
+        <v>2774.864</v>
       </c>
       <c r="AZ10" s="2" t="n">
-        <v>-1.398</v>
+        <v>-1.3574</v>
       </c>
       <c r="BA10" s="2" t="n">
-        <v>-0.2842</v>
+        <v>-0.2639</v>
       </c>
       <c r="BB10" s="2" t="n">
-        <v>-0.2139</v>
+        <v>-0.2057</v>
       </c>
       <c r="BC10" s="2" t="n">
-        <v>0.07290000000000001</v>
+        <v>0.0771</v>
       </c>
       <c r="BD10" s="2" t="n">
-        <v>-0.3075</v>
+        <v>-0.3055</v>
       </c>
     </row>
     <row r="11">
@@ -2175,7 +2183,7 @@
         </is>
       </c>
       <c r="C11" s="2" t="n">
-        <v>12360</v>
+        <v>12435</v>
       </c>
       <c r="D11" s="2" t="n">
         <v>6.32</v>
@@ -2239,23 +2247,23 @@
       <c r="AE11" s="2" t="inlineStr"/>
       <c r="AF11" s="2" t="inlineStr"/>
       <c r="AG11" s="2" t="n">
-        <v>33.28</v>
+        <v>33.46</v>
       </c>
       <c r="AH11" s="2" t="n">
-        <v>7.51</v>
+        <v>8.19</v>
       </c>
       <c r="AI11" s="2" t="n"/>
       <c r="AJ11" s="2" t="n">
-        <v>10.98</v>
+        <v>11.66</v>
       </c>
       <c r="AK11" s="2" t="n">
-        <v>6.78</v>
+        <v>7.46</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>49</v>
+        <v>49.5</v>
       </c>
       <c r="AM11" s="2" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="AN11" s="2" t="inlineStr"/>
       <c r="AO11" s="2" t="inlineStr"/>
@@ -2267,40 +2275,40 @@
         </is>
       </c>
       <c r="AS11" s="2" t="n">
-        <v>11845</v>
+        <v>11860</v>
       </c>
       <c r="AT11" s="2" t="n">
-        <v>11658</v>
+        <v>11665.5</v>
       </c>
       <c r="AU11" s="2" t="n">
-        <v>11449.75</v>
+        <v>11453.5</v>
       </c>
       <c r="AV11" s="2" t="n">
-        <v>11570.5</v>
+        <v>11573</v>
       </c>
       <c r="AW11" s="2" t="n">
-        <v>11812.3</v>
+        <v>11813.8</v>
       </c>
       <c r="AX11" s="2" t="n">
-        <v>11374.778</v>
+        <v>11375.528</v>
       </c>
       <c r="AY11" s="2" t="n">
-        <v>10759.245</v>
+        <v>10759.62</v>
       </c>
       <c r="AZ11" s="2" t="n">
-        <v>1.1559</v>
+        <v>1.1901</v>
       </c>
       <c r="BA11" s="2" t="n">
-        <v>0.3855</v>
+        <v>0.4026</v>
       </c>
       <c r="BB11" s="2" t="n">
-        <v>0.2304</v>
+        <v>0.237</v>
       </c>
       <c r="BC11" s="2" t="n">
-        <v>0.1426</v>
+        <v>0.146</v>
       </c>
       <c r="BD11" s="2" t="n">
-        <v>0.3328</v>
+        <v>0.3346</v>
       </c>
     </row>
     <row r="12">
@@ -2315,10 +2323,10 @@
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>3447</v>
+        <v>3449</v>
       </c>
       <c r="D12" s="2" t="n">
-        <v>100.66</v>
+        <v>101.06</v>
       </c>
       <c r="E12" s="2" t="inlineStr"/>
       <c r="F12" s="2" t="inlineStr"/>
@@ -2379,23 +2387,23 @@
       <c r="AE12" s="2" t="inlineStr"/>
       <c r="AF12" s="2" t="inlineStr"/>
       <c r="AG12" s="2" t="n">
-        <v>2.04</v>
+        <v>2.05</v>
       </c>
       <c r="AH12" s="2" t="n">
-        <v>-6.69</v>
+        <v>-6.61</v>
       </c>
       <c r="AI12" s="2" t="n"/>
       <c r="AJ12" s="2" t="n">
-        <v>6.34</v>
+        <v>6.42</v>
       </c>
       <c r="AK12" s="2" t="n">
-        <v>6.74</v>
+        <v>6.82</v>
       </c>
       <c r="AL12" s="2" t="n">
         <v>31.3</v>
       </c>
       <c r="AM12" s="2" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="AN12" s="2" t="inlineStr"/>
       <c r="AO12" s="2" t="n">
@@ -2409,40 +2417,40 @@
         </is>
       </c>
       <c r="AS12" s="2" t="n">
-        <v>3424.4</v>
+        <v>3424.8</v>
       </c>
       <c r="AT12" s="2" t="n">
-        <v>3410.9</v>
+        <v>3411.1</v>
       </c>
       <c r="AU12" s="2" t="n">
-        <v>3363.79</v>
+        <v>3363.89</v>
       </c>
       <c r="AV12" s="2" t="n">
-        <v>3323.409</v>
+        <v>3323.476</v>
       </c>
       <c r="AW12" s="2" t="n">
-        <v>3324.289</v>
+        <v>3324.329</v>
       </c>
       <c r="AX12" s="2" t="n">
-        <v>3394.927</v>
+        <v>3394.947</v>
       </c>
       <c r="AY12" s="2" t="n">
-        <v>3234.783</v>
+        <v>3234.793</v>
       </c>
       <c r="AZ12" s="2" t="n">
-        <v>0.5143</v>
+        <v>0.5174</v>
       </c>
       <c r="BA12" s="2" t="n">
-        <v>0.9356</v>
+        <v>0.9372</v>
       </c>
       <c r="BB12" s="2" t="n">
-        <v>-0.5326</v>
+        <v>-0.532</v>
       </c>
       <c r="BC12" s="2" t="n">
-        <v>0.2354</v>
+        <v>0.2358</v>
       </c>
       <c r="BD12" s="2" t="n">
-        <v>0.0204</v>
+        <v>0.0205</v>
       </c>
     </row>
     <row r="13">
@@ -2457,7 +2465,7 @@
         </is>
       </c>
       <c r="C13" s="2" t="n">
-        <v>3395</v>
+        <v>3387</v>
       </c>
       <c r="D13" s="2" t="n">
         <v>91.12</v>
@@ -2529,20 +2537,20 @@
       <c r="AE13" s="2" t="inlineStr"/>
       <c r="AF13" s="2" t="inlineStr"/>
       <c r="AG13" s="2" t="n">
-        <v>108.24</v>
+        <v>108.18</v>
       </c>
       <c r="AH13" s="2" t="n">
-        <v>8.68</v>
+        <v>8.449999999999999</v>
       </c>
       <c r="AI13" s="2" t="n"/>
       <c r="AJ13" s="2" t="n">
-        <v>-21.55</v>
+        <v>-21.78</v>
       </c>
       <c r="AK13" s="2" t="n">
-        <v>-26.83</v>
+        <v>-27.06</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>44.1</v>
+        <v>44</v>
       </c>
       <c r="AM13" s="2" t="n">
         <v>17</v>
@@ -2561,40 +2569,40 @@
         </is>
       </c>
       <c r="AS13" s="2" t="n">
-        <v>3729.4</v>
+        <v>3727.8</v>
       </c>
       <c r="AT13" s="2" t="n">
-        <v>4060.8</v>
+        <v>4060</v>
       </c>
       <c r="AU13" s="2" t="n">
-        <v>3939.833</v>
+        <v>3939.433</v>
       </c>
       <c r="AV13" s="2" t="n">
-        <v>3907.887</v>
+        <v>3907.621</v>
       </c>
       <c r="AW13" s="2" t="n">
-        <v>3909.212</v>
+        <v>3909.052</v>
       </c>
       <c r="AX13" s="2" t="n">
-        <v>4102.665</v>
+        <v>4102.585</v>
       </c>
       <c r="AY13" s="2" t="n">
-        <v>3429</v>
+        <v>3428.96</v>
       </c>
       <c r="AZ13" s="2" t="n">
-        <v>-0.7508</v>
+        <v>-0.7609</v>
       </c>
       <c r="BA13" s="2" t="n">
-        <v>-0.6136</v>
+        <v>-0.6188</v>
       </c>
       <c r="BB13" s="2" t="n">
-        <v>1.0062</v>
+        <v>1.0041</v>
       </c>
       <c r="BC13" s="2" t="n">
-        <v>-0.9028</v>
+        <v>-0.9038</v>
       </c>
       <c r="BD13" s="2" t="n">
-        <v>1.0824</v>
+        <v>1.0818</v>
       </c>
     </row>
     <row r="14">
@@ -2609,7 +2617,7 @@
         </is>
       </c>
       <c r="C14" s="2" t="n">
-        <v>2169</v>
+        <v>2160.5</v>
       </c>
       <c r="D14" s="2" t="n">
         <v>80.95</v>
@@ -2632,14 +2640,14 @@
       <c r="P14" s="2" t="inlineStr"/>
       <c r="Q14" s="2" t="inlineStr"/>
       <c r="R14" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>2</v>
       </c>
       <c r="T14" s="2" t="inlineStr">
         <is>
-          <t>0100000100</t>
+          <t>0000000100</t>
         </is>
       </c>
       <c r="U14" s="2" t="inlineStr">
@@ -2663,7 +2671,7 @@
       <c r="Y14" s="2" t="inlineStr"/>
       <c r="Z14" s="2" t="inlineStr">
         <is>
-          <t>4→1·3d ← 1→4·11d</t>
+          <t>4→1·3d ← 4+→4·6d ← 1→4+·11d</t>
         </is>
       </c>
       <c r="AA14" s="2" t="inlineStr"/>
@@ -2675,23 +2683,23 @@
       <c r="AE14" s="2" t="inlineStr"/>
       <c r="AF14" s="2" t="inlineStr"/>
       <c r="AG14" s="2" t="n">
-        <v>36.61</v>
+        <v>36.52</v>
       </c>
       <c r="AH14" s="2" t="n">
-        <v>-8.41</v>
+        <v>-8.75</v>
       </c>
       <c r="AI14" s="2" t="n"/>
       <c r="AJ14" s="2" t="n">
-        <v>-5.14</v>
+        <v>-5.48</v>
       </c>
       <c r="AK14" s="2" t="n">
-        <v>2.71</v>
+        <v>2.38</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>20.6</v>
+        <v>20.5</v>
       </c>
       <c r="AM14" s="2" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AN14" s="2" t="inlineStr"/>
       <c r="AO14" s="2" t="n">
@@ -2705,40 +2713,40 @@
         </is>
       </c>
       <c r="AS14" s="2" t="n">
-        <v>2249.5</v>
+        <v>2247.8</v>
       </c>
       <c r="AT14" s="2" t="n">
-        <v>2358.1</v>
+        <v>2357.25</v>
       </c>
       <c r="AU14" s="2" t="n">
-        <v>2254.99</v>
+        <v>2254.565</v>
       </c>
       <c r="AV14" s="2" t="n">
-        <v>2205.84</v>
+        <v>2205.557</v>
       </c>
       <c r="AW14" s="2" t="n">
-        <v>2210.834</v>
+        <v>2210.664</v>
       </c>
       <c r="AX14" s="2" t="n">
-        <v>2484.218</v>
+        <v>2484.133</v>
       </c>
       <c r="AY14" s="2" t="n">
-        <v>2341.923</v>
+        <v>2341.881</v>
       </c>
       <c r="AZ14" s="2" t="n">
-        <v>0.0311</v>
+        <v>0.0123</v>
       </c>
       <c r="BA14" s="2" t="n">
-        <v>1.0358</v>
+        <v>1.0258</v>
       </c>
       <c r="BB14" s="2" t="n">
-        <v>0.2048</v>
+        <v>0.2008</v>
       </c>
       <c r="BC14" s="2" t="n">
-        <v>-0.4665</v>
+        <v>-0.4682</v>
       </c>
       <c r="BD14" s="2" t="n">
-        <v>0.3661</v>
+        <v>0.3652</v>
       </c>
     </row>
     <row r="15">
@@ -2753,7 +2761,7 @@
         </is>
       </c>
       <c r="C15" s="2" t="n">
-        <v>53600</v>
+        <v>53270</v>
       </c>
       <c r="D15" s="2" t="n">
         <v>67.83</v>
@@ -2770,7 +2778,7 @@
         <v>-9</v>
       </c>
       <c r="N15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O15" s="2" t="inlineStr"/>
       <c r="P15" s="2" t="inlineStr"/>
@@ -2807,7 +2815,7 @@
       <c r="Y15" s="2" t="inlineStr"/>
       <c r="Z15" s="2" t="inlineStr">
         <is>
-          <t>4+→4·11d ← 4→4+·13d</t>
+          <t>4+→4·7d ← 4→4+·14d</t>
         </is>
       </c>
       <c r="AA15" s="2" t="inlineStr"/>
@@ -2819,23 +2827,23 @@
       <c r="AE15" s="2" t="inlineStr"/>
       <c r="AF15" s="2" t="inlineStr"/>
       <c r="AG15" s="2" t="n">
-        <v>19.57</v>
+        <v>19.43</v>
       </c>
       <c r="AH15" s="2" t="n">
-        <v>-22.75</v>
+        <v>-23.2</v>
       </c>
       <c r="AI15" s="2" t="n"/>
       <c r="AJ15" s="2" t="n">
-        <v>-6.14</v>
+        <v>-6.6</v>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>1.6</v>
+        <v>1.15</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>15.6</v>
+        <v>15.4</v>
       </c>
       <c r="AM15" s="2" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="AN15" s="2" t="inlineStr"/>
       <c r="AO15" s="2" t="n">
@@ -2853,40 +2861,40 @@
         </is>
       </c>
       <c r="AS15" s="2" t="n">
-        <v>56984</v>
+        <v>56918</v>
       </c>
       <c r="AT15" s="2" t="n">
-        <v>59696</v>
+        <v>59663</v>
       </c>
       <c r="AU15" s="2" t="n">
-        <v>56886.264</v>
+        <v>56869.764</v>
       </c>
       <c r="AV15" s="2" t="n">
-        <v>55930.065</v>
+        <v>55919.065</v>
       </c>
       <c r="AW15" s="2" t="n">
-        <v>58122.58</v>
+        <v>58115.98</v>
       </c>
       <c r="AX15" s="2" t="n">
-        <v>64902.273</v>
+        <v>64898.973</v>
       </c>
       <c r="AY15" s="2" t="n">
-        <v>65382.936</v>
+        <v>65381.286</v>
       </c>
       <c r="AZ15" s="2" t="n">
-        <v>0.1811</v>
+        <v>0.1522</v>
       </c>
       <c r="BA15" s="2" t="n">
-        <v>0.9912</v>
+        <v>0.9758</v>
       </c>
       <c r="BB15" s="2" t="n">
-        <v>0.118</v>
+        <v>0.112</v>
       </c>
       <c r="BC15" s="2" t="n">
-        <v>-0.2478</v>
+        <v>-0.2504</v>
       </c>
       <c r="BD15" s="2" t="n">
-        <v>0.1957</v>
+        <v>0.1943</v>
       </c>
     </row>
     <row r="16">
@@ -2901,7 +2909,7 @@
         </is>
       </c>
       <c r="C16" s="2" t="n">
-        <v>4231</v>
+        <v>4211</v>
       </c>
       <c r="D16" s="2" t="n">
         <v>6.28</v>
@@ -2965,20 +2973,20 @@
       <c r="AE16" s="2" t="inlineStr"/>
       <c r="AF16" s="2" t="inlineStr"/>
       <c r="AG16" s="2" t="n">
-        <v>18.1</v>
+        <v>18</v>
       </c>
       <c r="AH16" s="2" t="n">
-        <v>-21.95</v>
+        <v>-22.3</v>
       </c>
       <c r="AI16" s="2" t="n"/>
       <c r="AJ16" s="2" t="n">
-        <v>-4.53</v>
+        <v>-4.88</v>
       </c>
       <c r="AK16" s="2" t="n">
-        <v>-2.69</v>
+        <v>-3.04</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
       <c r="AM16" s="2" t="n">
         <v>12</v>
@@ -2999,40 +3007,40 @@
         </is>
       </c>
       <c r="AS16" s="2" t="n">
-        <v>4480</v>
+        <v>4476</v>
       </c>
       <c r="AT16" s="2" t="n">
-        <v>4638.3</v>
+        <v>4636.3</v>
       </c>
       <c r="AU16" s="2" t="n">
-        <v>4552.75</v>
+        <v>4551.75</v>
       </c>
       <c r="AV16" s="2" t="n">
-        <v>4500.067</v>
+        <v>4499.4</v>
       </c>
       <c r="AW16" s="2" t="n">
-        <v>4835.42</v>
+        <v>4835.02</v>
       </c>
       <c r="AX16" s="2" t="n">
-        <v>5315.53</v>
+        <v>5315.33</v>
       </c>
       <c r="AY16" s="2" t="n">
-        <v>5101.65</v>
+        <v>5101.55</v>
       </c>
       <c r="AZ16" s="2" t="n">
-        <v>-0.6979</v>
+        <v>-0.72</v>
       </c>
       <c r="BA16" s="2" t="n">
-        <v>0.465</v>
+        <v>0.4535</v>
       </c>
       <c r="BB16" s="2" t="n">
-        <v>-0.7992</v>
+        <v>-0.8035</v>
       </c>
       <c r="BC16" s="2" t="n">
-        <v>-0.3371</v>
+        <v>-0.3391</v>
       </c>
       <c r="BD16" s="2" t="n">
-        <v>0.181</v>
+        <v>0.18</v>
       </c>
     </row>
     <row r="17">
@@ -3047,10 +3055,10 @@
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>5010</v>
+        <v>5001</v>
       </c>
       <c r="D17" s="2" t="n">
-        <v>5.75</v>
+        <v>5.21</v>
       </c>
       <c r="E17" s="2" t="inlineStr"/>
       <c r="F17" s="2" t="inlineStr"/>
@@ -3119,20 +3127,20 @@
       <c r="AE17" s="2" t="inlineStr"/>
       <c r="AF17" s="2" t="inlineStr"/>
       <c r="AG17" s="2" t="n">
-        <v>10.46</v>
+        <v>10.42</v>
       </c>
       <c r="AH17" s="2" t="n">
-        <v>-14.54</v>
+        <v>-14.67</v>
       </c>
       <c r="AI17" s="2" t="n"/>
       <c r="AJ17" s="2" t="n">
-        <v>3.76</v>
+        <v>3.62</v>
       </c>
       <c r="AK17" s="2" t="n">
-        <v>-3.83</v>
+        <v>-3.97</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>8.800000000000001</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="AM17" s="2" t="n">
         <v>16</v>
@@ -3149,40 +3157,40 @@
         </is>
       </c>
       <c r="AS17" s="2" t="n">
-        <v>5085.8</v>
+        <v>5084</v>
       </c>
       <c r="AT17" s="2" t="n">
-        <v>5172.3</v>
+        <v>5171.4</v>
       </c>
       <c r="AU17" s="2" t="n">
-        <v>5171.912</v>
+        <v>5171.462</v>
       </c>
       <c r="AV17" s="2" t="n">
-        <v>5178.524</v>
+        <v>5178.224</v>
       </c>
       <c r="AW17" s="2" t="n">
-        <v>5399.645</v>
+        <v>5399.465</v>
       </c>
       <c r="AX17" s="2" t="n">
-        <v>5622.794</v>
+        <v>5622.704</v>
       </c>
       <c r="AY17" s="2" t="n">
-        <v>5517.682</v>
+        <v>5517.637</v>
       </c>
       <c r="AZ17" s="2" t="n">
-        <v>-0.607</v>
+        <v>-0.6159</v>
       </c>
       <c r="BA17" s="2" t="n">
-        <v>0.0491</v>
+        <v>0.0446</v>
       </c>
       <c r="BB17" s="2" t="n">
-        <v>-0.345</v>
+        <v>-0.3468</v>
       </c>
       <c r="BC17" s="2" t="n">
-        <v>-0.458</v>
+        <v>-0.4589</v>
       </c>
       <c r="BD17" s="2" t="n">
-        <v>0.1046</v>
+        <v>0.1042</v>
       </c>
     </row>
     <row r="18">
@@ -3197,7 +3205,7 @@
         </is>
       </c>
       <c r="C18" s="2" t="n">
-        <v>14440</v>
+        <v>14160</v>
       </c>
       <c r="D18" s="2" t="n">
         <v>86.78</v>
@@ -3212,20 +3220,20 @@
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O18" s="2" t="inlineStr"/>
       <c r="P18" s="2" t="inlineStr"/>
       <c r="Q18" s="2" t="inlineStr"/>
       <c r="R18" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S18" s="2" t="n">
         <v>5</v>
       </c>
       <c r="T18" s="2" t="inlineStr">
         <is>
-          <t>0111111000</t>
+          <t>0011111000</t>
         </is>
       </c>
       <c r="U18" s="2" t="inlineStr">
@@ -3263,23 +3271,23 @@
       </c>
       <c r="AF18" s="2" t="inlineStr"/>
       <c r="AG18" s="2" t="n">
-        <v>34.57</v>
+        <v>34</v>
       </c>
       <c r="AH18" s="2" t="n">
-        <v>4.15</v>
+        <v>2.17</v>
       </c>
       <c r="AI18" s="2" t="n"/>
       <c r="AJ18" s="2" t="n">
-        <v>3.69</v>
+        <v>1.7</v>
       </c>
       <c r="AK18" s="2" t="n">
-        <v>10.81</v>
+        <v>8.83</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>79.3</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="AM18" s="2" t="n">
-        <v>23</v>
+        <v>19</v>
       </c>
       <c r="AN18" s="2" t="inlineStr"/>
       <c r="AO18" s="2" t="inlineStr"/>
@@ -3291,40 +3299,40 @@
         </is>
       </c>
       <c r="AS18" s="2" t="n">
-        <v>14604</v>
+        <v>14548</v>
       </c>
       <c r="AT18" s="2" t="n">
-        <v>14812</v>
+        <v>14784</v>
       </c>
       <c r="AU18" s="2" t="n">
-        <v>14075.111</v>
+        <v>14061.111</v>
       </c>
       <c r="AV18" s="2" t="n">
-        <v>13684.232</v>
+        <v>13674.899</v>
       </c>
       <c r="AW18" s="2" t="n">
-        <v>13876.257</v>
+        <v>13870.657</v>
       </c>
       <c r="AX18" s="2" t="n">
-        <v>13870.281</v>
+        <v>13867.481</v>
       </c>
       <c r="AY18" s="2" t="n">
-        <v>12876.072</v>
+        <v>12874.672</v>
       </c>
       <c r="AZ18" s="2" t="n">
-        <v>1.3501</v>
+        <v>1.2492</v>
       </c>
       <c r="BA18" s="2" t="n">
-        <v>1.8151</v>
+        <v>1.7616</v>
       </c>
       <c r="BB18" s="2" t="n">
-        <v>0.6906</v>
+        <v>0.6693</v>
       </c>
       <c r="BC18" s="2" t="n">
-        <v>-0.0117</v>
+        <v>-0.0222</v>
       </c>
       <c r="BD18" s="2" t="n">
-        <v>0.3457</v>
+        <v>0.34</v>
       </c>
     </row>
     <row r="19">
@@ -3339,7 +3347,7 @@
         </is>
       </c>
       <c r="C19" s="2" t="n">
-        <v>4450</v>
+        <v>4397</v>
       </c>
       <c r="D19" s="2" t="n">
         <v>13.4</v>
@@ -3365,7 +3373,7 @@
         <v>0</v>
       </c>
       <c r="S19" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T19" s="2" t="inlineStr">
         <is>
@@ -3374,7 +3382,7 @@
       </c>
       <c r="U19" s="2" t="inlineStr">
         <is>
-          <t>0010000010</t>
+          <t>0000000010</t>
         </is>
       </c>
       <c r="V19" s="2" t="inlineStr">
@@ -3393,7 +3401,7 @@
       <c r="Y19" s="2" t="inlineStr"/>
       <c r="Z19" s="2" t="inlineStr">
         <is>
-          <t>4+→4·10d ← 1→4+·14d</t>
+          <t>4+→4·6d ← 1→4+·14d</t>
         </is>
       </c>
       <c r="AA19" s="2" t="inlineStr"/>
@@ -3405,23 +3413,23 @@
       <c r="AE19" s="2" t="inlineStr"/>
       <c r="AF19" s="2" t="inlineStr"/>
       <c r="AG19" s="2" t="n">
-        <v>-2.97</v>
+        <v>-3.23</v>
       </c>
       <c r="AH19" s="2" t="n">
-        <v>-21.61</v>
+        <v>-22.52</v>
       </c>
       <c r="AI19" s="2" t="n"/>
       <c r="AJ19" s="2" t="n">
-        <v>-1.74</v>
+        <v>-2.65</v>
       </c>
       <c r="AK19" s="2" t="n">
-        <v>0.1</v>
+        <v>-0.8100000000000001</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>4.4</v>
+        <v>4.2</v>
       </c>
       <c r="AM19" s="2" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="AN19" s="2" t="inlineStr"/>
       <c r="AO19" s="2" t="n">
@@ -3435,40 +3443,40 @@
         </is>
       </c>
       <c r="AS19" s="2" t="n">
-        <v>4611.8</v>
+        <v>4601.2</v>
       </c>
       <c r="AT19" s="2" t="n">
-        <v>4746.7</v>
+        <v>4741.4</v>
       </c>
       <c r="AU19" s="2" t="n">
-        <v>4609.25</v>
+        <v>4606.6</v>
       </c>
       <c r="AV19" s="2" t="n">
-        <v>4569.4</v>
+        <v>4567.633</v>
       </c>
       <c r="AW19" s="2" t="n">
-        <v>4780.204</v>
+        <v>4779.144</v>
       </c>
       <c r="AX19" s="2" t="n">
-        <v>5593.966</v>
+        <v>5593.436</v>
       </c>
       <c r="AY19" s="2" t="n">
-        <v>5325.003</v>
+        <v>5324.738</v>
       </c>
       <c r="AZ19" s="2" t="n">
-        <v>0.2046</v>
+        <v>0.1463</v>
       </c>
       <c r="BA19" s="2" t="n">
-        <v>0.6095</v>
+        <v>0.5793</v>
       </c>
       <c r="BB19" s="2" t="n">
-        <v>-0.1771</v>
+        <v>-0.1886</v>
       </c>
       <c r="BC19" s="2" t="n">
-        <v>-0.8666</v>
+        <v>-0.8714</v>
       </c>
       <c r="BD19" s="2" t="n">
-        <v>-0.0297</v>
+        <v>-0.0323</v>
       </c>
     </row>
     <row r="20">
@@ -3483,10 +3491,10 @@
         </is>
       </c>
       <c r="C20" s="2" t="n">
-        <v>1782</v>
+        <v>1779</v>
       </c>
       <c r="D20" s="2" t="n">
-        <v>-6.96</v>
+        <v>-7.16</v>
       </c>
       <c r="E20" s="2" t="inlineStr"/>
       <c r="F20" s="2" t="inlineStr"/>
@@ -3547,20 +3555,20 @@
       <c r="AE20" s="2" t="inlineStr"/>
       <c r="AF20" s="2" t="inlineStr"/>
       <c r="AG20" s="2" t="n">
-        <v>-6</v>
+        <v>-6.03</v>
       </c>
       <c r="AH20" s="2" t="n">
-        <v>-33.76</v>
+        <v>-33.86</v>
       </c>
       <c r="AI20" s="2" t="n"/>
       <c r="AJ20" s="2" t="n">
-        <v>-8.23</v>
+        <v>-8.33</v>
       </c>
       <c r="AK20" s="2" t="n">
-        <v>-30.88</v>
+        <v>-30.98</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>7.3</v>
+        <v>7.2</v>
       </c>
       <c r="AM20" s="2" t="n">
         <v>22</v>
@@ -3579,40 +3587,40 @@
         </is>
       </c>
       <c r="AS20" s="2" t="n">
-        <v>1885.6</v>
+        <v>1885</v>
       </c>
       <c r="AT20" s="2" t="n">
-        <v>2019.5</v>
+        <v>2019.2</v>
       </c>
       <c r="AU20" s="2" t="n">
-        <v>2288.5</v>
+        <v>2288.35</v>
       </c>
       <c r="AV20" s="2" t="n">
-        <v>2403.667</v>
+        <v>2403.567</v>
       </c>
       <c r="AW20" s="2" t="n">
-        <v>2517.94</v>
+        <v>2517.88</v>
       </c>
       <c r="AX20" s="2" t="n">
-        <v>2594.15</v>
+        <v>2594.12</v>
       </c>
       <c r="AY20" s="2" t="n">
-        <v>2440.265</v>
+        <v>2440.25</v>
       </c>
       <c r="AZ20" s="2" t="n">
-        <v>-5.6403</v>
+        <v>-5.6472</v>
       </c>
       <c r="BA20" s="2" t="n">
-        <v>-4.1485</v>
+        <v>-4.1516</v>
       </c>
       <c r="BB20" s="2" t="n">
-        <v>-1.3404</v>
+        <v>-1.3416</v>
       </c>
       <c r="BC20" s="2" t="n">
-        <v>-0.701</v>
+        <v>-0.7016</v>
       </c>
       <c r="BD20" s="2" t="n">
-        <v>-0.06</v>
+        <v>-0.0603</v>
       </c>
     </row>
     <row r="21">
@@ -3627,7 +3635,7 @@
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>2967.5</v>
+        <v>2949</v>
       </c>
       <c r="D21" s="2" t="n">
         <v>80.2</v>
@@ -3693,23 +3701,23 @@
       <c r="AE21" s="2" t="inlineStr"/>
       <c r="AF21" s="2" t="inlineStr"/>
       <c r="AG21" s="2" t="n">
-        <v>40.64</v>
+        <v>40.47</v>
       </c>
       <c r="AH21" s="2" t="n">
-        <v>-0.6</v>
+        <v>-1.19</v>
       </c>
       <c r="AI21" s="2" t="n"/>
       <c r="AJ21" s="2" t="n">
-        <v>-7.25</v>
+        <v>-7.84</v>
       </c>
       <c r="AK21" s="2" t="n">
-        <v>2.5</v>
+        <v>1.91</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>30.2</v>
+        <v>29.9</v>
       </c>
       <c r="AM21" s="2" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AN21" s="2" t="inlineStr"/>
       <c r="AO21" s="2" t="n">
@@ -3727,40 +3735,40 @@
         </is>
       </c>
       <c r="AS21" s="2" t="n">
-        <v>3084.8</v>
+        <v>3081.1</v>
       </c>
       <c r="AT21" s="2" t="n">
-        <v>3258</v>
+        <v>3256.15</v>
       </c>
       <c r="AU21" s="2" t="n">
-        <v>3089.349</v>
+        <v>3088.424</v>
       </c>
       <c r="AV21" s="2" t="n">
-        <v>3011.297</v>
+        <v>3010.681</v>
       </c>
       <c r="AW21" s="2" t="n">
-        <v>3033.003</v>
+        <v>3032.633</v>
       </c>
       <c r="AX21" s="2" t="n">
-        <v>3272.108</v>
+        <v>3271.923</v>
       </c>
       <c r="AY21" s="2" t="n">
-        <v>2772.688</v>
+        <v>2772.596</v>
       </c>
       <c r="AZ21" s="2" t="n">
-        <v>0.6974</v>
+        <v>0.6675</v>
       </c>
       <c r="BA21" s="2" t="n">
-        <v>1.2551</v>
+        <v>1.2392</v>
       </c>
       <c r="BB21" s="2" t="n">
-        <v>0.3511</v>
+        <v>0.3448</v>
       </c>
       <c r="BC21" s="2" t="n">
-        <v>0.07729999999999999</v>
+        <v>0.07439999999999999</v>
       </c>
       <c r="BD21" s="2" t="n">
-        <v>0.4064</v>
+        <v>0.4047</v>
       </c>
     </row>
     <row r="22">
@@ -3775,7 +3783,7 @@
         </is>
       </c>
       <c r="C22" s="2" t="n">
-        <v>34870</v>
+        <v>34560</v>
       </c>
       <c r="D22" s="2" t="n">
         <v>98.61</v>
@@ -3792,7 +3800,7 @@
         <v>-9</v>
       </c>
       <c r="N22" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="O22" s="2" t="inlineStr"/>
       <c r="P22" s="2" t="inlineStr"/>
@@ -3843,20 +3851,20 @@
       </c>
       <c r="AF22" s="2" t="inlineStr"/>
       <c r="AG22" s="2" t="n">
-        <v>85.88</v>
+        <v>85.59</v>
       </c>
       <c r="AH22" s="2" t="n">
-        <v>19.48</v>
+        <v>18.45</v>
       </c>
       <c r="AI22" s="2" t="n"/>
       <c r="AJ22" s="2" t="n">
-        <v>-15.17</v>
+        <v>-16.2</v>
       </c>
       <c r="AK22" s="2" t="n">
-        <v>4.7</v>
+        <v>3.67</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>82.90000000000001</v>
+        <v>82.59999999999999</v>
       </c>
       <c r="AM22" s="2" t="n">
         <v>12</v>
@@ -3877,40 +3885,40 @@
         </is>
       </c>
       <c r="AS22" s="2" t="n">
-        <v>38320</v>
+        <v>38258</v>
       </c>
       <c r="AT22" s="2" t="n">
-        <v>39460</v>
+        <v>39429</v>
       </c>
       <c r="AU22" s="2" t="n">
-        <v>36216</v>
+        <v>36200.5</v>
       </c>
       <c r="AV22" s="2" t="n">
-        <v>35115</v>
+        <v>35104.667</v>
       </c>
       <c r="AW22" s="2" t="n">
-        <v>34889.6</v>
+        <v>34883.4</v>
       </c>
       <c r="AX22" s="2" t="n">
-        <v>31888.7</v>
+        <v>31885.6</v>
       </c>
       <c r="AY22" s="2" t="n">
-        <v>28263.061</v>
+        <v>28261.511</v>
       </c>
       <c r="AZ22" s="2" t="n">
-        <v>2.4984</v>
+        <v>2.4556</v>
       </c>
       <c r="BA22" s="2" t="n">
-        <v>2.1096</v>
+        <v>2.0865</v>
       </c>
       <c r="BB22" s="2" t="n">
-        <v>1.6</v>
+        <v>1.5905</v>
       </c>
       <c r="BC22" s="2" t="n">
-        <v>1.0214</v>
+        <v>1.0162</v>
       </c>
       <c r="BD22" s="2" t="n">
-        <v>0.8588</v>
+        <v>0.8559</v>
       </c>
     </row>
     <row r="23">
@@ -3925,7 +3933,7 @@
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>80950</v>
+        <v>80700</v>
       </c>
       <c r="D23" s="2" t="n">
         <v>42.39</v>
@@ -3946,19 +3954,19 @@
       <c r="P23" s="2" t="inlineStr"/>
       <c r="Q23" s="2" t="inlineStr"/>
       <c r="R23" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S23" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="T23" s="2" t="inlineStr">
         <is>
-          <t>0111111001</t>
+          <t>0011111001</t>
         </is>
       </c>
       <c r="U23" s="2" t="inlineStr">
         <is>
-          <t>0011111001</t>
+          <t>0011111000</t>
         </is>
       </c>
       <c r="V23" s="2" t="inlineStr">
@@ -3999,23 +4007,23 @@
         </is>
       </c>
       <c r="AG23" s="2" t="n">
-        <v>46.45</v>
+        <v>46.36</v>
       </c>
       <c r="AH23" s="2" t="n">
-        <v>8.27</v>
+        <v>7.96</v>
       </c>
       <c r="AI23" s="2" t="n"/>
       <c r="AJ23" s="2" t="n">
-        <v>6.68</v>
+        <v>6.38</v>
       </c>
       <c r="AK23" s="2" t="n">
-        <v>4.21</v>
+        <v>3.9</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>54.8</v>
+        <v>54.6</v>
       </c>
       <c r="AM23" s="2" t="n">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AN23" s="2" t="inlineStr"/>
       <c r="AO23" s="2" t="inlineStr"/>
@@ -4027,40 +4035,40 @@
         </is>
       </c>
       <c r="AS23" s="2" t="n">
-        <v>80112</v>
+        <v>80062</v>
       </c>
       <c r="AT23" s="2" t="n">
-        <v>80556</v>
+        <v>80531</v>
       </c>
       <c r="AU23" s="2" t="n">
-        <v>79289.04300000001</v>
+        <v>79276.54300000001</v>
       </c>
       <c r="AV23" s="2" t="n">
-        <v>78645.262</v>
+        <v>78636.929</v>
       </c>
       <c r="AW23" s="2" t="n">
-        <v>80517.15700000001</v>
+        <v>80512.15700000001</v>
       </c>
       <c r="AX23" s="2" t="n">
-        <v>78416.622</v>
+        <v>78414.122</v>
       </c>
       <c r="AY23" s="2" t="n">
-        <v>69992.361</v>
+        <v>69991.111</v>
       </c>
       <c r="AZ23" s="2" t="n">
-        <v>0.08409999999999999</v>
+        <v>0.0679</v>
       </c>
       <c r="BA23" s="2" t="n">
-        <v>0.6791</v>
+        <v>0.6708</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>0.2481</v>
+        <v>0.2449</v>
       </c>
       <c r="BC23" s="2" t="n">
-        <v>0.1533</v>
+        <v>0.1517</v>
       </c>
       <c r="BD23" s="2" t="n">
-        <v>0.4645</v>
+        <v>0.4636</v>
       </c>
     </row>
     <row r="24">
@@ -4075,7 +4083,7 @@
         </is>
       </c>
       <c r="C24" s="2" t="n">
-        <v>41310</v>
+        <v>41330</v>
       </c>
       <c r="D24" s="2" t="n">
         <v>111</v>
@@ -4141,17 +4149,17 @@
       </c>
       <c r="AF24" s="2" t="inlineStr"/>
       <c r="AG24" s="2" t="n">
-        <v>47.96</v>
+        <v>47.98</v>
       </c>
       <c r="AH24" s="2" t="n">
-        <v>3.4</v>
+        <v>3.47</v>
       </c>
       <c r="AI24" s="2" t="n"/>
       <c r="AJ24" s="2" t="n">
-        <v>-8.16</v>
+        <v>-8.09</v>
       </c>
       <c r="AK24" s="2" t="n">
-        <v>11.47</v>
+        <v>11.55</v>
       </c>
       <c r="AL24" s="2" t="n">
         <v>47.3</v>
@@ -4169,40 +4177,40 @@
         </is>
       </c>
       <c r="AS24" s="2" t="n">
-        <v>44110</v>
+        <v>44114</v>
       </c>
       <c r="AT24" s="2" t="n">
-        <v>45273</v>
+        <v>45275</v>
       </c>
       <c r="AU24" s="2" t="n">
-        <v>42382.5</v>
+        <v>42383.5</v>
       </c>
       <c r="AV24" s="2" t="n">
-        <v>39703.333</v>
+        <v>39704</v>
       </c>
       <c r="AW24" s="2" t="n">
-        <v>39005.4</v>
+        <v>39005.8</v>
       </c>
       <c r="AX24" s="2" t="n">
-        <v>41756.075</v>
+        <v>41756.275</v>
       </c>
       <c r="AY24" s="2" t="n">
-        <v>38647.544</v>
+        <v>38647.644</v>
       </c>
       <c r="AZ24" s="2" t="n">
-        <v>1.3916</v>
+        <v>1.394</v>
       </c>
       <c r="BA24" s="2" t="n">
-        <v>2.9147</v>
+        <v>2.916</v>
       </c>
       <c r="BB24" s="2" t="n">
-        <v>0.9141</v>
+        <v>0.9146</v>
       </c>
       <c r="BC24" s="2" t="n">
-        <v>0.4385</v>
+        <v>0.4387</v>
       </c>
       <c r="BD24" s="2" t="n">
-        <v>0.4796</v>
+        <v>0.4798</v>
       </c>
     </row>
     <row r="25">
@@ -4217,7 +4225,7 @@
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>10195</v>
+        <v>9962</v>
       </c>
       <c r="D25" s="2" t="n">
         <v>76.94</v>
@@ -4238,14 +4246,14 @@
       <c r="P25" s="2" t="inlineStr"/>
       <c r="Q25" s="2" t="inlineStr"/>
       <c r="R25" s="2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="S25" s="2" t="n">
         <v>4</v>
       </c>
       <c r="T25" s="2" t="inlineStr">
         <is>
-          <t>0111110000</t>
+          <t>0011010000</t>
         </is>
       </c>
       <c r="U25" s="2" t="inlineStr">
@@ -4285,23 +4293,23 @@
       </c>
       <c r="AF25" s="2" t="inlineStr"/>
       <c r="AG25" s="2" t="n">
-        <v>110.97</v>
+        <v>110.24</v>
       </c>
       <c r="AH25" s="2" t="n">
-        <v>29.17</v>
+        <v>26.26</v>
       </c>
       <c r="AI25" s="2" t="n"/>
       <c r="AJ25" s="2" t="n">
-        <v>-4.53</v>
+        <v>-7.43</v>
       </c>
       <c r="AK25" s="2" t="n">
-        <v>9.48</v>
+        <v>6.57</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>3.1</v>
+        <v>2.9</v>
       </c>
       <c r="AM25" s="2" t="n">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="AN25" s="2" t="inlineStr"/>
       <c r="AO25" s="2" t="n">
@@ -4315,40 +4323,40 @@
         </is>
       </c>
       <c r="AS25" s="2" t="n">
-        <v>10550.8</v>
+        <v>10504.2</v>
       </c>
       <c r="AT25" s="2" t="n">
-        <v>10688.9</v>
+        <v>10665.6</v>
       </c>
       <c r="AU25" s="2" t="n">
-        <v>9961.833000000001</v>
+        <v>9950.183000000001</v>
       </c>
       <c r="AV25" s="2" t="n">
-        <v>9679.179</v>
+        <v>9671.413</v>
       </c>
       <c r="AW25" s="2" t="n">
-        <v>9737.422</v>
+        <v>9732.762000000001</v>
       </c>
       <c r="AX25" s="2" t="n">
-        <v>12406.92</v>
+        <v>12404.59</v>
       </c>
       <c r="AY25" s="2" t="n">
-        <v>8477.306</v>
+        <v>8476.141</v>
       </c>
       <c r="AZ25" s="2" t="n">
-        <v>3.12</v>
+        <v>2.9999</v>
       </c>
       <c r="BA25" s="2" t="n">
-        <v>2.0719</v>
+        <v>2.0087</v>
       </c>
       <c r="BB25" s="2" t="n">
-        <v>0.347</v>
+        <v>0.3219</v>
       </c>
       <c r="BC25" s="2" t="n">
-        <v>0.6454</v>
+        <v>0.6355</v>
       </c>
       <c r="BD25" s="2" t="n">
-        <v>1.1097</v>
+        <v>1.1024</v>
       </c>
     </row>
     <row r="26">
@@ -4363,10 +4371,10 @@
         </is>
       </c>
       <c r="C26" s="2" t="n">
-        <v>3648</v>
+        <v>3655</v>
       </c>
       <c r="D26" s="2" t="n">
-        <v>101.74</v>
+        <v>102.64</v>
       </c>
       <c r="E26" s="2" t="inlineStr"/>
       <c r="F26" s="2" t="inlineStr"/>
@@ -4376,17 +4384,11 @@
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr"/>
-      <c r="I26" s="2" t="inlineStr">
-        <is>
-          <t>顶背离</t>
-        </is>
-      </c>
+      <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n">
         <v>-1</v>
       </c>
-      <c r="K26" s="2" t="n">
-        <v>-1</v>
-      </c>
+      <c r="K26" s="2" t="inlineStr"/>
       <c r="L26" s="2" t="inlineStr"/>
       <c r="M26" s="2" t="n">
         <v>-9</v>
@@ -4443,23 +4445,23 @@
       <c r="AE26" s="2" t="inlineStr"/>
       <c r="AF26" s="2" t="inlineStr"/>
       <c r="AG26" s="2" t="n">
-        <v>-2.68</v>
+        <v>-2.62</v>
       </c>
       <c r="AH26" s="2" t="n">
-        <v>-5.96</v>
+        <v>-5.75</v>
       </c>
       <c r="AI26" s="2" t="n"/>
       <c r="AJ26" s="2" t="n">
-        <v>8.33</v>
+        <v>8.529999999999999</v>
       </c>
       <c r="AK26" s="2" t="n">
-        <v>11.35</v>
+        <v>11.55</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>93.8</v>
+        <v>94</v>
       </c>
       <c r="AM26" s="2" t="n">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="AN26" s="2" t="inlineStr"/>
       <c r="AO26" s="2" t="inlineStr"/>
@@ -4477,40 +4479,40 @@
         </is>
       </c>
       <c r="AS26" s="2" t="n">
-        <v>3629.2</v>
+        <v>3630.6</v>
       </c>
       <c r="AT26" s="2" t="n">
-        <v>3589.1</v>
+        <v>3589.8</v>
       </c>
       <c r="AU26" s="2" t="n">
-        <v>3502.707</v>
+        <v>3503.057</v>
       </c>
       <c r="AV26" s="2" t="n">
-        <v>3435.649</v>
+        <v>3435.882</v>
       </c>
       <c r="AW26" s="2" t="n">
-        <v>3431.522</v>
+        <v>3431.662</v>
       </c>
       <c r="AX26" s="2" t="n">
-        <v>3291.916</v>
+        <v>3291.986</v>
       </c>
       <c r="AY26" s="2" t="n">
-        <v>3313.295</v>
+        <v>3313.33</v>
       </c>
       <c r="AZ26" s="2" t="n">
-        <v>1.0218</v>
+        <v>1.0321</v>
       </c>
       <c r="BA26" s="2" t="n">
-        <v>1.7693</v>
+        <v>1.7747</v>
       </c>
       <c r="BB26" s="2" t="n">
-        <v>0.3329</v>
+        <v>0.335</v>
       </c>
       <c r="BC26" s="2" t="n">
-        <v>0.5302</v>
+        <v>0.5313</v>
       </c>
       <c r="BD26" s="2" t="n">
-        <v>-0.0268</v>
+        <v>-0.0262</v>
       </c>
     </row>
     <row r="27">
@@ -4525,7 +4527,7 @@
         </is>
       </c>
       <c r="C27" s="2" t="n">
-        <v>3758</v>
+        <v>3757</v>
       </c>
       <c r="D27" s="2" t="n">
         <v>10.44</v>
@@ -4581,7 +4583,7 @@
       </c>
       <c r="Z27" s="2" t="inlineStr">
         <is>
-          <t>4→4+·8d ← 4+→4·9d ← 4→4+·14d</t>
+          <t>4→4+·18d</t>
         </is>
       </c>
       <c r="AA27" s="2" t="inlineStr"/>
@@ -4593,7 +4595,7 @@
       <c r="AE27" s="2" t="inlineStr"/>
       <c r="AF27" s="2" t="inlineStr"/>
       <c r="AG27" s="2" t="n">
-        <v>-9.66</v>
+        <v>-9.67</v>
       </c>
       <c r="AH27" s="2" t="n">
         <v>-21.01</v>
@@ -4621,40 +4623,40 @@
         </is>
       </c>
       <c r="AS27" s="2" t="n">
-        <v>3695.2</v>
+        <v>3695</v>
       </c>
       <c r="AT27" s="2" t="n">
-        <v>3743.8</v>
+        <v>3743.7</v>
       </c>
       <c r="AU27" s="2" t="n">
-        <v>3786.552</v>
+        <v>3786.502</v>
       </c>
       <c r="AV27" s="2" t="n">
-        <v>3775.444</v>
+        <v>3775.411</v>
       </c>
       <c r="AW27" s="2" t="n">
-        <v>3880.686</v>
+        <v>3880.666</v>
       </c>
       <c r="AX27" s="2" t="n">
-        <v>3822.189</v>
+        <v>3822.179</v>
       </c>
       <c r="AY27" s="2" t="n">
-        <v>4180.083</v>
+        <v>4180.078</v>
       </c>
       <c r="AZ27" s="2" t="n">
-        <v>-1.0252</v>
+        <v>-1.0266</v>
       </c>
       <c r="BA27" s="2" t="n">
-        <v>-0.1141</v>
+        <v>-0.1148</v>
       </c>
       <c r="BB27" s="2" t="n">
-        <v>-0.1048</v>
+        <v>-0.1051</v>
       </c>
       <c r="BC27" s="2" t="n">
-        <v>-0.2358</v>
+        <v>-0.2359</v>
       </c>
       <c r="BD27" s="2" t="n">
-        <v>-0.09660000000000001</v>
+        <v>-0.09669999999999999</v>
       </c>
     </row>
     <row r="28">
@@ -4669,7 +4671,7 @@
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>13790</v>
+        <v>13800</v>
       </c>
       <c r="D28" s="2" t="n">
         <v>107.6</v>
@@ -4737,17 +4739,17 @@
       </c>
       <c r="AF28" s="2" t="inlineStr"/>
       <c r="AG28" s="2" t="n">
-        <v>92.86</v>
+        <v>92.88</v>
       </c>
       <c r="AH28" s="2" t="n">
-        <v>15.6</v>
+        <v>15.71</v>
       </c>
       <c r="AI28" s="2" t="n"/>
       <c r="AJ28" s="2" t="n">
-        <v>-12.1</v>
+        <v>-11.99</v>
       </c>
       <c r="AK28" s="2" t="n">
-        <v>7.62</v>
+        <v>7.73</v>
       </c>
       <c r="AL28" s="2" t="n">
         <v>37.7</v>
@@ -4769,40 +4771,40 @@
         </is>
       </c>
       <c r="AS28" s="2" t="n">
-        <v>14914</v>
+        <v>14916</v>
       </c>
       <c r="AT28" s="2" t="n">
-        <v>15387.5</v>
+        <v>15388.5</v>
       </c>
       <c r="AU28" s="2" t="n">
-        <v>14453.958</v>
+        <v>14454.458</v>
       </c>
       <c r="AV28" s="2" t="n">
-        <v>13944.541</v>
+        <v>13944.874</v>
       </c>
       <c r="AW28" s="2" t="n">
-        <v>13728.978</v>
+        <v>13729.178</v>
       </c>
       <c r="AX28" s="2" t="n">
-        <v>14378.754</v>
+        <v>14378.854</v>
       </c>
       <c r="AY28" s="2" t="n">
-        <v>12042.454</v>
+        <v>12042.504</v>
       </c>
       <c r="AZ28" s="2" t="n">
-        <v>0.7992</v>
+        <v>0.8026</v>
       </c>
       <c r="BA28" s="2" t="n">
-        <v>2.0869</v>
+        <v>2.0887</v>
       </c>
       <c r="BB28" s="2" t="n">
-        <v>0.65</v>
+        <v>0.6508</v>
       </c>
       <c r="BC28" s="2" t="n">
-        <v>0.7628</v>
+        <v>0.7632</v>
       </c>
       <c r="BD28" s="2" t="n">
-        <v>0.9286</v>
+        <v>0.9288</v>
       </c>
     </row>
     <row r="29">
@@ -4817,7 +4819,7 @@
         </is>
       </c>
       <c r="C29" s="2" t="n">
-        <v>25335</v>
+        <v>25450</v>
       </c>
       <c r="D29" s="2" t="n">
         <v>15.87</v>
@@ -4865,41 +4867,47 @@
       </c>
       <c r="X29" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y29" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y29" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均</t>
+        </is>
+      </c>
       <c r="Z29" s="2" t="inlineStr">
         <is>
-          <t>4+→4·11d ← 4→4+·14d</t>
+          <t>4→4+·1d ← 4+→4·2d ← 4→4+·14d</t>
         </is>
       </c>
       <c r="AA29" s="2" t="inlineStr"/>
       <c r="AB29" s="2" t="inlineStr"/>
-      <c r="AC29" s="2" t="n">
-        <v>-1</v>
+      <c r="AC29" s="2" t="inlineStr">
+        <is>
+          <t>预1</t>
+        </is>
       </c>
       <c r="AD29" s="2" t="inlineStr"/>
       <c r="AE29" s="2" t="inlineStr"/>
       <c r="AF29" s="2" t="inlineStr"/>
       <c r="AG29" s="2" t="n">
-        <v>7.56</v>
+        <v>7.68</v>
       </c>
       <c r="AH29" s="2" t="n">
-        <v>-12.12</v>
+        <v>-11.7</v>
       </c>
       <c r="AI29" s="2" t="n"/>
       <c r="AJ29" s="2" t="n">
-        <v>5.72</v>
+        <v>6.13</v>
       </c>
       <c r="AK29" s="2" t="n">
-        <v>8.949999999999999</v>
+        <v>9.369999999999999</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>48.8</v>
+        <v>49.1</v>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="AN29" s="2" t="inlineStr"/>
       <c r="AO29" s="2" t="n">
@@ -4913,40 +4921,40 @@
         </is>
       </c>
       <c r="AS29" s="2" t="n">
-        <v>25212</v>
+        <v>25235</v>
       </c>
       <c r="AT29" s="2" t="n">
-        <v>25020</v>
+        <v>25031.5</v>
       </c>
       <c r="AU29" s="2" t="n">
-        <v>24079.5</v>
+        <v>24085.25</v>
       </c>
       <c r="AV29" s="2" t="n">
-        <v>23947.833</v>
+        <v>23951.667</v>
       </c>
       <c r="AW29" s="2" t="n">
-        <v>24573.3</v>
+        <v>24575.6</v>
       </c>
       <c r="AX29" s="2" t="n">
-        <v>25199.55</v>
+        <v>25200.7</v>
       </c>
       <c r="AY29" s="2" t="n">
-        <v>26071.592</v>
+        <v>26072.167</v>
       </c>
       <c r="AZ29" s="2" t="n">
-        <v>1.6711</v>
+        <v>1.6957</v>
       </c>
       <c r="BA29" s="2" t="n">
-        <v>1.246</v>
+        <v>1.2588</v>
       </c>
       <c r="BB29" s="2" t="n">
-        <v>0.2283</v>
+        <v>0.2332</v>
       </c>
       <c r="BC29" s="2" t="n">
-        <v>-0.1983</v>
+        <v>-0.1959</v>
       </c>
       <c r="BD29" s="2" t="n">
-        <v>0.0756</v>
+        <v>0.07679999999999999</v>
       </c>
     </row>
     <row r="30">
@@ -4961,10 +4969,10 @@
         </is>
       </c>
       <c r="C30" s="2" t="n">
-        <v>2262.5</v>
+        <v>2248</v>
       </c>
       <c r="D30" s="2" t="n">
-        <v>11.78</v>
+        <v>9.65</v>
       </c>
       <c r="E30" s="2" t="inlineStr"/>
       <c r="F30" s="2" t="inlineStr"/>
@@ -5020,29 +5028,25 @@
       </c>
       <c r="AA30" s="2" t="inlineStr"/>
       <c r="AB30" s="2" t="inlineStr"/>
-      <c r="AC30" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
-      </c>
+      <c r="AC30" s="2" t="inlineStr"/>
       <c r="AD30" s="2" t="inlineStr"/>
       <c r="AE30" s="2" t="inlineStr"/>
       <c r="AF30" s="2" t="inlineStr"/>
       <c r="AG30" s="2" t="n">
-        <v>-4.81</v>
+        <v>-4.96</v>
       </c>
       <c r="AH30" s="2" t="n">
-        <v>-12.56</v>
+        <v>-13.1</v>
       </c>
       <c r="AI30" s="2" t="n"/>
       <c r="AJ30" s="2" t="n">
-        <v>1.11</v>
+        <v>0.57</v>
       </c>
       <c r="AK30" s="2" t="n">
-        <v>-3.29</v>
+        <v>-3.83</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>40.6</v>
+        <v>40.4</v>
       </c>
       <c r="AM30" s="2" t="n">
         <v>16</v>
@@ -5057,40 +5061,40 @@
         </is>
       </c>
       <c r="AS30" s="2" t="n">
-        <v>2312.8</v>
+        <v>2309.9</v>
       </c>
       <c r="AT30" s="2" t="n">
-        <v>2366.85</v>
+        <v>2365.4</v>
       </c>
       <c r="AU30" s="2" t="n">
-        <v>2361.609</v>
+        <v>2360.884</v>
       </c>
       <c r="AV30" s="2" t="n">
-        <v>2394.367</v>
+        <v>2393.884</v>
       </c>
       <c r="AW30" s="2" t="n">
-        <v>2420.791</v>
+        <v>2420.501</v>
       </c>
       <c r="AX30" s="2" t="n">
-        <v>2381.9</v>
+        <v>2381.755</v>
       </c>
       <c r="AY30" s="2" t="n">
-        <v>2364.614</v>
+        <v>2364.542</v>
       </c>
       <c r="AZ30" s="2" t="n">
-        <v>-0.8165</v>
+        <v>-0.8478</v>
       </c>
       <c r="BA30" s="2" t="n">
-        <v>-0.6216</v>
+        <v>-0.6373</v>
       </c>
       <c r="BB30" s="2" t="n">
-        <v>0.2498</v>
+        <v>0.2435</v>
       </c>
       <c r="BC30" s="2" t="n">
-        <v>0.1312</v>
+        <v>0.128</v>
       </c>
       <c r="BD30" s="2" t="n">
-        <v>-0.0481</v>
+        <v>-0.0496</v>
       </c>
     </row>
     <row r="31">
@@ -5105,7 +5109,7 @@
         </is>
       </c>
       <c r="C31" s="2" t="n">
-        <v>2269</v>
+        <v>2293.5</v>
       </c>
       <c r="D31" s="2" t="n">
         <v>44.64</v>
@@ -5129,7 +5133,7 @@
         <v>8</v>
       </c>
       <c r="S31" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T31" s="2" t="inlineStr">
         <is>
@@ -5138,7 +5142,7 @@
       </c>
       <c r="U31" s="2" t="inlineStr">
         <is>
-          <t>0111111101</t>
+          <t>1111111101</t>
         </is>
       </c>
       <c r="V31" s="2" t="inlineStr">
@@ -5167,33 +5171,31 @@
       <c r="AA31" s="2" t="inlineStr"/>
       <c r="AB31" s="2" t="inlineStr"/>
       <c r="AC31" s="2" t="inlineStr"/>
-      <c r="AD31" s="2" t="inlineStr">
-        <is>
-          <t>预1</t>
-        </is>
+      <c r="AD31" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AE31" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AF31" s="2" t="inlineStr"/>
       <c r="AG31" s="2" t="n">
-        <v>22.05</v>
+        <v>22.37</v>
       </c>
       <c r="AH31" s="2" t="n">
-        <v>2.58</v>
+        <v>3.71</v>
       </c>
       <c r="AI31" s="2" t="n"/>
       <c r="AJ31" s="2" t="n">
-        <v>10.95</v>
+        <v>12.08</v>
       </c>
       <c r="AK31" s="2" t="n">
-        <v>-4.51</v>
+        <v>-3.38</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>78.59999999999999</v>
+        <v>79.2</v>
       </c>
       <c r="AM31" s="2" t="n">
-        <v>69</v>
+        <v>81</v>
       </c>
       <c r="AN31" s="2" t="inlineStr"/>
       <c r="AO31" s="2" t="inlineStr"/>
@@ -5207,40 +5209,40 @@
         </is>
       </c>
       <c r="AS31" s="2" t="n">
-        <v>2219.2</v>
+        <v>2224.1</v>
       </c>
       <c r="AT31" s="2" t="n">
-        <v>2195.2</v>
+        <v>2197.65</v>
       </c>
       <c r="AU31" s="2" t="n">
-        <v>2216.98</v>
+        <v>2218.205</v>
       </c>
       <c r="AV31" s="2" t="n">
-        <v>2219.897</v>
+        <v>2220.714</v>
       </c>
       <c r="AW31" s="2" t="n">
-        <v>2146.864</v>
+        <v>2147.354</v>
       </c>
       <c r="AX31" s="2" t="n">
-        <v>2013.003</v>
+        <v>2013.248</v>
       </c>
       <c r="AY31" s="2" t="n">
-        <v>2008.664</v>
+        <v>2008.787</v>
       </c>
       <c r="AZ31" s="2" t="n">
-        <v>0.3214</v>
+        <v>0.3798</v>
       </c>
       <c r="BA31" s="2" t="n">
-        <v>-0.3308</v>
+        <v>-0.3023</v>
       </c>
       <c r="BB31" s="2" t="n">
-        <v>0.5542</v>
+        <v>0.5662</v>
       </c>
       <c r="BC31" s="2" t="n">
-        <v>0.3321</v>
+        <v>0.3385</v>
       </c>
       <c r="BD31" s="2" t="n">
-        <v>0.2205</v>
+        <v>0.2237</v>
       </c>
     </row>
     <row r="32">
@@ -5255,7 +5257,7 @@
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>4860</v>
+        <v>4897</v>
       </c>
       <c r="D32" s="2" t="n">
         <v>4.42</v>
@@ -5276,19 +5278,19 @@
       <c r="P32" s="2" t="inlineStr"/>
       <c r="Q32" s="2" t="inlineStr"/>
       <c r="R32" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T32" s="2" t="inlineStr">
         <is>
-          <t>0000000000</t>
+          <t>0001000000</t>
         </is>
       </c>
       <c r="U32" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0001000100</t>
         </is>
       </c>
       <c r="V32" s="2" t="inlineStr">
@@ -5301,13 +5303,17 @@
       </c>
       <c r="X32" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y32" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y32" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z32" s="2" t="inlineStr">
         <is>
-          <t>4+→4·1d ← 4→4+·9d</t>
+          <t>4→4+·9d</t>
         </is>
       </c>
       <c r="AA32" s="2" t="inlineStr"/>
@@ -5321,23 +5327,23 @@
       </c>
       <c r="AF32" s="2" t="inlineStr"/>
       <c r="AG32" s="2" t="n">
-        <v>11.74</v>
+        <v>11.93</v>
       </c>
       <c r="AH32" s="2" t="n">
-        <v>-11.43</v>
+        <v>-10.73</v>
       </c>
       <c r="AI32" s="2" t="n"/>
       <c r="AJ32" s="2" t="n">
-        <v>7.19</v>
+        <v>7.89</v>
       </c>
       <c r="AK32" s="2" t="n">
-        <v>-5.59</v>
+        <v>-4.9</v>
       </c>
       <c r="AL32" s="2" t="n">
-        <v>34.8</v>
+        <v>35.4</v>
       </c>
       <c r="AM32" s="2" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="AN32" s="2" t="inlineStr"/>
       <c r="AO32" s="2" t="inlineStr"/>
@@ -5349,40 +5355,40 @@
         </is>
       </c>
       <c r="AS32" s="2" t="n">
-        <v>4819.6</v>
+        <v>4827</v>
       </c>
       <c r="AT32" s="2" t="n">
-        <v>4794.3</v>
+        <v>4798</v>
       </c>
       <c r="AU32" s="2" t="n">
-        <v>4823.811</v>
+        <v>4825.661</v>
       </c>
       <c r="AV32" s="2" t="n">
-        <v>4896.201</v>
+        <v>4897.434</v>
       </c>
       <c r="AW32" s="2" t="n">
-        <v>4889.272</v>
+        <v>4890.012</v>
       </c>
       <c r="AX32" s="2" t="n">
-        <v>4917.459</v>
+        <v>4917.829</v>
       </c>
       <c r="AY32" s="2" t="n">
-        <v>5138.06</v>
+        <v>5138.245</v>
       </c>
       <c r="AZ32" s="2" t="n">
-        <v>0.0912</v>
+        <v>0.1314</v>
       </c>
       <c r="BA32" s="2" t="n">
-        <v>-0.5252</v>
+        <v>-0.5054999999999999</v>
       </c>
       <c r="BB32" s="2" t="n">
-        <v>-0.4038</v>
+        <v>-0.396</v>
       </c>
       <c r="BC32" s="2" t="n">
-        <v>-0.3485</v>
+        <v>-0.3447</v>
       </c>
       <c r="BD32" s="2" t="n">
-        <v>0.1174</v>
+        <v>0.1193</v>
       </c>
     </row>
     <row r="33">
@@ -5464,14 +5470,14 @@
         <v>34.23</v>
       </c>
       <c r="AH33" s="2" t="n">
-        <v>1.11</v>
+        <v>1.13</v>
       </c>
       <c r="AI33" s="2" t="n"/>
       <c r="AJ33" s="2" t="n">
-        <v>6.05</v>
+        <v>6.07</v>
       </c>
       <c r="AK33" s="2" t="n">
-        <v>4.65</v>
+        <v>4.68</v>
       </c>
       <c r="AL33" s="2" t="n">
         <v>50.3</v>
@@ -5537,7 +5543,7 @@
         </is>
       </c>
       <c r="C34" s="2" t="n">
-        <v>7483</v>
+        <v>7512</v>
       </c>
       <c r="D34" s="2" t="n">
         <v>35.91</v>
@@ -5611,23 +5617,23 @@
         <v>1</v>
       </c>
       <c r="AG34" s="2" t="n">
-        <v>44.76</v>
+        <v>44.88</v>
       </c>
       <c r="AH34" s="2" t="n">
-        <v>10.01</v>
+        <v>10.46</v>
       </c>
       <c r="AI34" s="2" t="n"/>
       <c r="AJ34" s="2" t="n">
-        <v>8.98</v>
+        <v>9.43</v>
       </c>
       <c r="AK34" s="2" t="n">
-        <v>-4.8</v>
+        <v>-4.35</v>
       </c>
       <c r="AL34" s="2" t="n">
-        <v>86.09999999999999</v>
+        <v>86.40000000000001</v>
       </c>
       <c r="AM34" s="2" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="AN34" s="2" t="inlineStr"/>
       <c r="AO34" s="2" t="inlineStr"/>
@@ -5641,40 +5647,40 @@
         </is>
       </c>
       <c r="AS34" s="2" t="n">
-        <v>7322.6</v>
+        <v>7328.4</v>
       </c>
       <c r="AT34" s="2" t="n">
-        <v>7335.3</v>
+        <v>7338.2</v>
       </c>
       <c r="AU34" s="2" t="n">
-        <v>7320.673</v>
+        <v>7322.123</v>
       </c>
       <c r="AV34" s="2" t="n">
-        <v>7381.786</v>
+        <v>7382.752</v>
       </c>
       <c r="AW34" s="2" t="n">
-        <v>7321.698</v>
+        <v>7322.278</v>
       </c>
       <c r="AX34" s="2" t="n">
-        <v>6806.633</v>
+        <v>6806.923</v>
       </c>
       <c r="AY34" s="2" t="n">
-        <v>6475.107</v>
+        <v>6475.252</v>
       </c>
       <c r="AZ34" s="2" t="n">
-        <v>0.2246</v>
+        <v>0.2453</v>
       </c>
       <c r="BA34" s="2" t="n">
-        <v>-0.1987</v>
+        <v>-0.1884</v>
       </c>
       <c r="BB34" s="2" t="n">
-        <v>0.5661</v>
+        <v>0.5703</v>
       </c>
       <c r="BC34" s="2" t="n">
-        <v>0.1399</v>
+        <v>0.1421</v>
       </c>
       <c r="BD34" s="2" t="n">
-        <v>0.4476</v>
+        <v>0.4488</v>
       </c>
     </row>
     <row r="35">
@@ -5689,7 +5695,7 @@
         </is>
       </c>
       <c r="C35" s="2" t="n">
-        <v>4954</v>
+        <v>4988</v>
       </c>
       <c r="D35" s="2" t="n">
         <v>21.7</v>
@@ -5757,23 +5763,23 @@
       </c>
       <c r="AF35" s="2" t="inlineStr"/>
       <c r="AG35" s="2" t="n">
-        <v>11.74</v>
+        <v>11.91</v>
       </c>
       <c r="AH35" s="2" t="n">
-        <v>-10.32</v>
+        <v>-9.69</v>
       </c>
       <c r="AI35" s="2" t="n"/>
       <c r="AJ35" s="2" t="n">
-        <v>7.91</v>
+        <v>8.550000000000001</v>
       </c>
       <c r="AK35" s="2" t="n">
-        <v>-4.96</v>
+        <v>-4.32</v>
       </c>
       <c r="AL35" s="2" t="n">
-        <v>74.2</v>
+        <v>74.8</v>
       </c>
       <c r="AM35" s="2" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="AN35" s="2" t="inlineStr"/>
       <c r="AO35" s="2" t="inlineStr"/>
@@ -5785,40 +5791,40 @@
         </is>
       </c>
       <c r="AS35" s="2" t="n">
-        <v>4902.8</v>
+        <v>4909.6</v>
       </c>
       <c r="AT35" s="2" t="n">
-        <v>4897.4</v>
+        <v>4900.8</v>
       </c>
       <c r="AU35" s="2" t="n">
-        <v>4945.178</v>
+        <v>4946.878</v>
       </c>
       <c r="AV35" s="2" t="n">
-        <v>4981.433</v>
+        <v>4982.566</v>
       </c>
       <c r="AW35" s="2" t="n">
-        <v>4910.037</v>
+        <v>4910.717</v>
       </c>
       <c r="AX35" s="2" t="n">
-        <v>4844.593</v>
+        <v>4844.933</v>
       </c>
       <c r="AY35" s="2" t="n">
-        <v>5160.448</v>
+        <v>5160.618</v>
       </c>
       <c r="AZ35" s="2" t="n">
-        <v>-0.119</v>
+        <v>-0.083</v>
       </c>
       <c r="BA35" s="2" t="n">
-        <v>-0.3632</v>
+        <v>-0.3454</v>
       </c>
       <c r="BB35" s="2" t="n">
-        <v>0.0461</v>
+        <v>0.0533</v>
       </c>
       <c r="BC35" s="2" t="n">
-        <v>-0.4688</v>
+        <v>-0.4652</v>
       </c>
       <c r="BD35" s="2" t="n">
-        <v>0.1174</v>
+        <v>0.1191</v>
       </c>
     </row>
     <row r="36">
@@ -5833,7 +5839,7 @@
         </is>
       </c>
       <c r="C36" s="2" t="n">
-        <v>10575</v>
+        <v>10585</v>
       </c>
       <c r="D36" s="2" t="n">
         <v>96.47</v>
@@ -5899,17 +5905,17 @@
       <c r="AE36" s="2" t="inlineStr"/>
       <c r="AF36" s="2" t="inlineStr"/>
       <c r="AG36" s="2" t="n">
-        <v>69.23999999999999</v>
+        <v>69.27</v>
       </c>
       <c r="AH36" s="2" t="n">
-        <v>5.89</v>
+        <v>6.01</v>
       </c>
       <c r="AI36" s="2" t="n"/>
       <c r="AJ36" s="2" t="n">
-        <v>-10.87</v>
+        <v>-10.74</v>
       </c>
       <c r="AK36" s="2" t="n">
-        <v>0.41</v>
+        <v>0.54</v>
       </c>
       <c r="AL36" s="2" t="n">
         <v>26</v>
@@ -5931,40 +5937,40 @@
         </is>
       </c>
       <c r="AS36" s="2" t="n">
-        <v>11236</v>
+        <v>11238</v>
       </c>
       <c r="AT36" s="2" t="n">
-        <v>11854</v>
+        <v>11855</v>
       </c>
       <c r="AU36" s="2" t="n">
-        <v>11326.579</v>
+        <v>11327.079</v>
       </c>
       <c r="AV36" s="2" t="n">
-        <v>10986.148</v>
+        <v>10986.481</v>
       </c>
       <c r="AW36" s="2" t="n">
-        <v>10949.175</v>
+        <v>10949.375</v>
       </c>
       <c r="AX36" s="2" t="n">
-        <v>11784.736</v>
+        <v>11784.836</v>
       </c>
       <c r="AY36" s="2" t="n">
-        <v>9904.757</v>
+        <v>9904.807000000001</v>
       </c>
       <c r="AZ36" s="2" t="n">
-        <v>-0.6578000000000001</v>
+        <v>-0.6534</v>
       </c>
       <c r="BA36" s="2" t="n">
-        <v>1.268</v>
+        <v>1.2704</v>
       </c>
       <c r="BB36" s="2" t="n">
-        <v>0.2647</v>
+        <v>0.2657</v>
       </c>
       <c r="BC36" s="2" t="n">
-        <v>0.4228</v>
+        <v>0.4233</v>
       </c>
       <c r="BD36" s="2" t="n">
-        <v>0.6924</v>
+        <v>0.6927</v>
       </c>
     </row>
     <row r="37">
@@ -5979,10 +5985,10 @@
         </is>
       </c>
       <c r="C37" s="2" t="n">
-        <v>1735.5</v>
+        <v>1751</v>
       </c>
       <c r="D37" s="2" t="n">
-        <v>80.55</v>
+        <v>29.83</v>
       </c>
       <c r="E37" s="2" t="inlineStr"/>
       <c r="F37" s="2" t="inlineStr"/>
@@ -6049,23 +6055,23 @@
       </c>
       <c r="AF37" s="2" t="inlineStr"/>
       <c r="AG37" s="2" t="n">
-        <v>35.16</v>
+        <v>35.42</v>
       </c>
       <c r="AH37" s="2" t="n">
-        <v>3.45</v>
+        <v>4.4</v>
       </c>
       <c r="AI37" s="2" t="n"/>
       <c r="AJ37" s="2" t="n">
-        <v>7.04</v>
+        <v>7.99</v>
       </c>
       <c r="AK37" s="2" t="n">
-        <v>-7.68</v>
+        <v>-6.73</v>
       </c>
       <c r="AL37" s="2" t="n">
-        <v>71.5</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="AM37" s="2" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="AN37" s="2" t="inlineStr"/>
       <c r="AO37" s="2" t="inlineStr"/>
@@ -6079,40 +6085,40 @@
         </is>
       </c>
       <c r="AS37" s="2" t="n">
-        <v>1729.7</v>
+        <v>1732.8</v>
       </c>
       <c r="AT37" s="2" t="n">
-        <v>1727.55</v>
+        <v>1729.1</v>
       </c>
       <c r="AU37" s="2" t="n">
-        <v>1747.105</v>
+        <v>1747.88</v>
       </c>
       <c r="AV37" s="2" t="n">
-        <v>1767.716</v>
+        <v>1768.233</v>
       </c>
       <c r="AW37" s="2" t="n">
-        <v>1751.465</v>
+        <v>1751.775</v>
       </c>
       <c r="AX37" s="2" t="n">
-        <v>1680.17</v>
+        <v>1680.325</v>
       </c>
       <c r="AY37" s="2" t="n">
-        <v>1593.624</v>
+        <v>1593.701</v>
       </c>
       <c r="AZ37" s="2" t="n">
-        <v>-0.4576</v>
+        <v>-0.4114</v>
       </c>
       <c r="BA37" s="2" t="n">
-        <v>-0.5484</v>
+        <v>-0.5256</v>
       </c>
       <c r="BB37" s="2" t="n">
-        <v>0.4037</v>
+        <v>0.413</v>
       </c>
       <c r="BC37" s="2" t="n">
-        <v>-0.0863</v>
+        <v>-0.0815</v>
       </c>
       <c r="BD37" s="2" t="n">
-        <v>0.3516</v>
+        <v>0.3542</v>
       </c>
     </row>
     <row r="38">
@@ -6127,7 +6133,7 @@
         </is>
       </c>
       <c r="C38" s="2" t="n">
-        <v>4705</v>
+        <v>4737</v>
       </c>
       <c r="D38" s="2" t="n">
         <v>12.95</v>
@@ -6152,14 +6158,14 @@
       <c r="P38" s="2" t="inlineStr"/>
       <c r="Q38" s="2" t="inlineStr"/>
       <c r="R38" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S38" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T38" s="2" t="inlineStr">
         <is>
-          <t>0000000100</t>
+          <t>0100000100</t>
         </is>
       </c>
       <c r="U38" s="2" t="inlineStr">
@@ -6199,23 +6205,23 @@
       </c>
       <c r="AF38" s="2" t="inlineStr"/>
       <c r="AG38" s="2" t="n">
-        <v>29.81</v>
+        <v>29.99</v>
       </c>
       <c r="AH38" s="2" t="n">
-        <v>-6.27</v>
+        <v>-5.61</v>
       </c>
       <c r="AI38" s="2" t="n"/>
       <c r="AJ38" s="2" t="n">
-        <v>7.03</v>
+        <v>7.69</v>
       </c>
       <c r="AK38" s="2" t="n">
-        <v>-7.1</v>
+        <v>-6.44</v>
       </c>
       <c r="AL38" s="2" t="n">
-        <v>66.8</v>
+        <v>67.40000000000001</v>
       </c>
       <c r="AM38" s="2" t="n">
-        <v>55</v>
+        <v>65</v>
       </c>
       <c r="AN38" s="2" t="inlineStr"/>
       <c r="AO38" s="2" t="inlineStr"/>
@@ -6227,40 +6233,40 @@
         </is>
       </c>
       <c r="AS38" s="2" t="n">
-        <v>4687.6</v>
+        <v>4694</v>
       </c>
       <c r="AT38" s="2" t="n">
-        <v>4682</v>
+        <v>4685.2</v>
       </c>
       <c r="AU38" s="2" t="n">
-        <v>4738.751</v>
+        <v>4740.351</v>
       </c>
       <c r="AV38" s="2" t="n">
-        <v>4795.009</v>
+        <v>4796.076</v>
       </c>
       <c r="AW38" s="2" t="n">
-        <v>4758.794</v>
+        <v>4759.434</v>
       </c>
       <c r="AX38" s="2" t="n">
-        <v>4698.939</v>
+        <v>4699.259</v>
       </c>
       <c r="AY38" s="2" t="n">
-        <v>4708.841</v>
+        <v>4709.001</v>
       </c>
       <c r="AZ38" s="2" t="n">
-        <v>-0.2679</v>
+        <v>-0.2326</v>
       </c>
       <c r="BA38" s="2" t="n">
-        <v>-0.6443</v>
+        <v>-0.6269</v>
       </c>
       <c r="BB38" s="2" t="n">
-        <v>-0.0542</v>
+        <v>-0.0472</v>
       </c>
       <c r="BC38" s="2" t="n">
-        <v>-0.4302</v>
+        <v>-0.4267</v>
       </c>
       <c r="BD38" s="2" t="n">
-        <v>0.2981</v>
+        <v>0.2999</v>
       </c>
     </row>
     <row r="39">
@@ -6275,7 +6281,7 @@
         </is>
       </c>
       <c r="C39" s="2" t="n">
-        <v>7307</v>
+        <v>7308</v>
       </c>
       <c r="D39" s="2" t="n">
         <v>93.44</v>
@@ -6345,17 +6351,17 @@
       <c r="AE39" s="2" t="inlineStr"/>
       <c r="AF39" s="2" t="inlineStr"/>
       <c r="AG39" s="2" t="n">
-        <v>61.01</v>
+        <v>61.02</v>
       </c>
       <c r="AH39" s="2" t="n">
-        <v>17.43</v>
+        <v>17.47</v>
       </c>
       <c r="AI39" s="2" t="n"/>
       <c r="AJ39" s="2" t="n">
-        <v>7.12</v>
+        <v>7.17</v>
       </c>
       <c r="AK39" s="2" t="n">
-        <v>-1.63</v>
+        <v>-1.58</v>
       </c>
       <c r="AL39" s="2" t="n">
         <v>99.3</v>
@@ -6375,40 +6381,40 @@
         </is>
       </c>
       <c r="AS39" s="2" t="n">
-        <v>7409</v>
+        <v>7409.2</v>
       </c>
       <c r="AT39" s="2" t="n">
-        <v>7271.5</v>
+        <v>7271.6</v>
       </c>
       <c r="AU39" s="2" t="n">
-        <v>7244.167</v>
+        <v>7244.217</v>
       </c>
       <c r="AV39" s="2" t="n">
-        <v>7201.254</v>
+        <v>7201.288</v>
       </c>
       <c r="AW39" s="2" t="n">
-        <v>6899.59</v>
+        <v>6899.61</v>
       </c>
       <c r="AX39" s="2" t="n">
-        <v>6146.69</v>
+        <v>6146.7</v>
       </c>
       <c r="AY39" s="2" t="n">
-        <v>5733.35</v>
+        <v>5733.355</v>
       </c>
       <c r="AZ39" s="2" t="n">
-        <v>0.8643999999999999</v>
+        <v>0.8652</v>
       </c>
       <c r="BA39" s="2" t="n">
-        <v>0.4903</v>
+        <v>0.4906</v>
       </c>
       <c r="BB39" s="2" t="n">
-        <v>1.0923</v>
+        <v>1.0924</v>
       </c>
       <c r="BC39" s="2" t="n">
-        <v>0.8354</v>
+        <v>0.8355</v>
       </c>
       <c r="BD39" s="2" t="n">
-        <v>0.6101</v>
+        <v>0.6102</v>
       </c>
     </row>
     <row r="40">
@@ -6423,7 +6429,7 @@
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>7320</v>
+        <v>7340</v>
       </c>
       <c r="D40" s="2" t="n">
         <v>91.93000000000001</v>
@@ -6497,23 +6503,23 @@
       <c r="AE40" s="2" t="inlineStr"/>
       <c r="AF40" s="2" t="inlineStr"/>
       <c r="AG40" s="2" t="n">
-        <v>68.45</v>
+        <v>68.54000000000001</v>
       </c>
       <c r="AH40" s="2" t="n">
-        <v>18.76</v>
+        <v>19.12</v>
       </c>
       <c r="AI40" s="2" t="n"/>
       <c r="AJ40" s="2" t="n">
-        <v>8.77</v>
+        <v>9.130000000000001</v>
       </c>
       <c r="AK40" s="2" t="n">
-        <v>0.84</v>
+        <v>1.19</v>
       </c>
       <c r="AL40" s="2" t="n">
-        <v>99.59999999999999</v>
+        <v>99.7</v>
       </c>
       <c r="AM40" s="2" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="AN40" s="2" t="inlineStr"/>
       <c r="AO40" s="2" t="inlineStr"/>
@@ -6527,40 +6533,40 @@
         </is>
       </c>
       <c r="AS40" s="2" t="n">
-        <v>7426.6</v>
+        <v>7430.6</v>
       </c>
       <c r="AT40" s="2" t="n">
-        <v>7264.1</v>
+        <v>7266.1</v>
       </c>
       <c r="AU40" s="2" t="n">
-        <v>7158.114</v>
+        <v>7159.114</v>
       </c>
       <c r="AV40" s="2" t="n">
-        <v>7095.517</v>
+        <v>7096.183</v>
       </c>
       <c r="AW40" s="2" t="n">
-        <v>6872.561</v>
+        <v>6872.961</v>
       </c>
       <c r="AX40" s="2" t="n">
-        <v>6160.766</v>
+        <v>6160.966</v>
       </c>
       <c r="AY40" s="2" t="n">
-        <v>5830.213</v>
+        <v>5830.313</v>
       </c>
       <c r="AZ40" s="2" t="n">
-        <v>1.5198</v>
+        <v>1.5345</v>
       </c>
       <c r="BA40" s="2" t="n">
-        <v>0.8643</v>
+        <v>0.8717</v>
       </c>
       <c r="BB40" s="2" t="n">
-        <v>1.2384</v>
+        <v>1.2415</v>
       </c>
       <c r="BC40" s="2" t="n">
-        <v>0.7274</v>
+        <v>0.7291</v>
       </c>
       <c r="BD40" s="2" t="n">
-        <v>0.6845</v>
+        <v>0.6854</v>
       </c>
     </row>
     <row r="41">
@@ -6575,7 +6581,7 @@
         </is>
       </c>
       <c r="C41" s="2" t="n">
-        <v>3375</v>
+        <v>3393</v>
       </c>
       <c r="D41" s="2" t="n">
         <v>86.33</v>
@@ -6592,7 +6598,7 @@
         <v>9</v>
       </c>
       <c r="N41" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O41" s="2" t="inlineStr"/>
       <c r="P41" s="2" t="inlineStr"/>
@@ -6644,28 +6650,28 @@
         </is>
       </c>
       <c r="AD41" s="2" t="n">
-        <v>-1</v>
+        <v>1</v>
       </c>
       <c r="AE41" s="2" t="inlineStr"/>
       <c r="AF41" s="2" t="inlineStr"/>
       <c r="AG41" s="2" t="n">
-        <v>68.40000000000001</v>
+        <v>68.58</v>
       </c>
       <c r="AH41" s="2" t="n">
-        <v>20.55</v>
+        <v>21.22</v>
       </c>
       <c r="AI41" s="2" t="n"/>
       <c r="AJ41" s="2" t="n">
-        <v>9.029999999999999</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="AK41" s="2" t="n">
-        <v>-4.18</v>
+        <v>-3.51</v>
       </c>
       <c r="AL41" s="2" t="n">
-        <v>88.5</v>
+        <v>88.7</v>
       </c>
       <c r="AM41" s="2" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="AN41" s="2" t="inlineStr">
         <is>
@@ -6683,40 +6689,40 @@
         </is>
       </c>
       <c r="AS41" s="2" t="n">
-        <v>3419.8</v>
+        <v>3423.4</v>
       </c>
       <c r="AT41" s="2" t="n">
-        <v>3338.4</v>
+        <v>3340.2</v>
       </c>
       <c r="AU41" s="2" t="n">
-        <v>3349.478</v>
+        <v>3350.378</v>
       </c>
       <c r="AV41" s="2" t="n">
-        <v>3339.876</v>
+        <v>3340.476</v>
       </c>
       <c r="AW41" s="2" t="n">
-        <v>3220.359</v>
+        <v>3220.719</v>
       </c>
       <c r="AX41" s="2" t="n">
-        <v>2891.186</v>
+        <v>2891.366</v>
       </c>
       <c r="AY41" s="2" t="n">
-        <v>2635.013</v>
+        <v>2635.103</v>
       </c>
       <c r="AZ41" s="2" t="n">
-        <v>0.7726</v>
+        <v>0.8011</v>
       </c>
       <c r="BA41" s="2" t="n">
-        <v>0.3876</v>
+        <v>0.4017</v>
       </c>
       <c r="BB41" s="2" t="n">
-        <v>1.0267</v>
+        <v>1.0326</v>
       </c>
       <c r="BC41" s="2" t="n">
-        <v>0.8359</v>
+        <v>0.8391999999999999</v>
       </c>
       <c r="BD41" s="2" t="n">
-        <v>0.6840000000000001</v>
+        <v>0.6858</v>
       </c>
     </row>
     <row r="42">
@@ -6731,10 +6737,10 @@
         </is>
       </c>
       <c r="C42" s="2" t="n">
-        <v>76450</v>
+        <v>77000</v>
       </c>
       <c r="D42" s="2" t="n">
-        <v>14.37</v>
+        <v>96.77</v>
       </c>
       <c r="E42" s="2" t="inlineStr"/>
       <c r="F42" s="2" t="inlineStr"/>
@@ -6791,23 +6797,23 @@
       <c r="AE42" s="2" t="inlineStr"/>
       <c r="AF42" s="2" t="inlineStr"/>
       <c r="AG42" s="2" t="n">
-        <v>35.07</v>
+        <v>35.27</v>
       </c>
       <c r="AH42" s="2" t="n">
-        <v>2.15</v>
+        <v>2.91</v>
       </c>
       <c r="AI42" s="2" t="n"/>
       <c r="AJ42" s="2" t="n">
-        <v>7.02</v>
+        <v>7.78</v>
       </c>
       <c r="AK42" s="2" t="n">
-        <v>9.890000000000001</v>
+        <v>10.64</v>
       </c>
       <c r="AL42" s="2" t="n">
-        <v>28.5</v>
+        <v>28.9</v>
       </c>
       <c r="AM42" s="2" t="n">
-        <v>75</v>
+        <v>84</v>
       </c>
       <c r="AN42" s="2" t="inlineStr"/>
       <c r="AO42" s="2" t="n">
@@ -6821,40 +6827,40 @@
         </is>
       </c>
       <c r="AS42" s="2" t="n">
-        <v>74852</v>
+        <v>74962</v>
       </c>
       <c r="AT42" s="2" t="n">
-        <v>74589</v>
+        <v>74644</v>
       </c>
       <c r="AU42" s="2" t="n">
-        <v>71581.5</v>
+        <v>71609</v>
       </c>
       <c r="AV42" s="2" t="n">
-        <v>70506.333</v>
+        <v>70524.667</v>
       </c>
       <c r="AW42" s="2" t="n">
-        <v>72378.97900000001</v>
+        <v>72389.97900000001</v>
       </c>
       <c r="AX42" s="2" t="n">
-        <v>76222.49400000001</v>
+        <v>76227.99400000001</v>
       </c>
       <c r="AY42" s="2" t="n">
-        <v>70575.247</v>
+        <v>70577.997</v>
       </c>
       <c r="AZ42" s="2" t="n">
-        <v>1.8384</v>
+        <v>1.8781</v>
       </c>
       <c r="BA42" s="2" t="n">
-        <v>1.4417</v>
+        <v>1.4622</v>
       </c>
       <c r="BB42" s="2" t="n">
-        <v>-0.2464</v>
+        <v>-0.2385</v>
       </c>
       <c r="BC42" s="2" t="n">
-        <v>0.0919</v>
+        <v>0.0956</v>
       </c>
       <c r="BD42" s="2" t="n">
-        <v>0.3507</v>
+        <v>0.3527</v>
       </c>
     </row>
     <row r="43">
@@ -7219,13 +7225,17 @@
       </c>
       <c r="X45" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y45" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y45" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·周J超卖·底背离·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z45" s="2" t="inlineStr">
         <is>
-          <t>4+→4·1d ← 4→4+·7d ← 1→4·14d</t>
+          <t>4→4+·7d ← 1→4·14d</t>
         </is>
       </c>
       <c r="AA45" s="2" t="inlineStr"/>
@@ -7665,7 +7675,11 @@
         </is>
       </c>
       <c r="Y48" s="2" t="inlineStr"/>
-      <c r="Z48" s="2" t="inlineStr"/>
+      <c r="Z48" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·12d ← 4→4+·16d ← 4+→4·17d</t>
+        </is>
+      </c>
       <c r="AA48" s="2" t="inlineStr"/>
       <c r="AB48" s="2" t="inlineStr"/>
       <c r="AC48" s="2" t="n">
@@ -9165,7 +9179,7 @@
       <c r="Y58" s="2" t="inlineStr"/>
       <c r="Z58" s="2" t="inlineStr">
         <is>
-          <t>4+→4·4d ← 4→4+·5d</t>
+          <t>4+→4·4d ← 4→4+·5d ← 4+→4·6d</t>
         </is>
       </c>
       <c r="AA58" s="2" t="inlineStr"/>
@@ -9315,7 +9329,7 @@
       <c r="Y59" s="2" t="inlineStr"/>
       <c r="Z59" s="2" t="inlineStr">
         <is>
-          <t>4+→4·12d ← 4→4+·18d</t>
+          <t>4+→4·12d</t>
         </is>
       </c>
       <c r="AA59" s="2" t="inlineStr"/>
@@ -9891,11 +9905,19 @@
       </c>
       <c r="X63" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y63" s="2" t="inlineStr"/>
-      <c r="Z63" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y63" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·日线纠缠</t>
+        </is>
+      </c>
+      <c r="Z63" s="2" t="inlineStr">
+        <is>
+          <t>4→4+·2d ← 4+→4·13d ← 4→4+·15d</t>
+        </is>
+      </c>
       <c r="AA63" s="2" t="inlineStr"/>
       <c r="AB63" s="2" t="inlineStr"/>
       <c r="AC63" s="2" t="inlineStr"/>
@@ -11509,7 +11531,7 @@
       <c r="Y74" s="2" t="inlineStr"/>
       <c r="Z74" s="2" t="inlineStr">
         <is>
-          <t>4+→4·2d ← 4→4+·6d</t>
+          <t>4+→4·2d ← 4→4+·6d ← 4+→4·7d</t>
         </is>
       </c>
       <c r="AA74" s="2" t="inlineStr"/>
@@ -11657,7 +11679,7 @@
       <c r="Y75" s="2" t="inlineStr"/>
       <c r="Z75" s="2" t="inlineStr">
         <is>
-          <t>4+→4·8d ← 4→4+·9d ← 1→4·19d</t>
+          <t>4+→4·2d ← 4→4+·3d ← 4+→4·4d</t>
         </is>
       </c>
       <c r="AA75" s="2" t="inlineStr"/>
@@ -12095,7 +12117,7 @@
       <c r="Y78" s="2" t="inlineStr"/>
       <c r="Z78" s="2" t="inlineStr">
         <is>
-          <t>1+→1·15d ← 4→1+·18d</t>
+          <t>1+→1·15d ← 4+→1+·18d ← 4→4+·20d</t>
         </is>
       </c>
       <c r="AA78" s="2" t="inlineStr"/>
@@ -12243,15 +12265,15 @@
       </c>
       <c r="X79" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y79" s="2" t="inlineStr"/>
-      <c r="Z79" s="2" t="inlineStr">
-        <is>
-          <t>4+→4·8d</t>
-        </is>
-      </c>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y79" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·底背离</t>
+        </is>
+      </c>
+      <c r="Z79" s="2" t="inlineStr"/>
       <c r="AA79" s="2" t="inlineStr"/>
       <c r="AB79" s="2" t="inlineStr"/>
       <c r="AC79" s="2" t="n">
@@ -12991,7 +13013,7 @@
       <c r="Y84" s="2" t="inlineStr"/>
       <c r="Z84" s="2" t="inlineStr">
         <is>
-          <t>4+→4·3d ← 4→4+·5d</t>
+          <t>4+→4·3d ← 4→4+·5d ← 4+→4·7d</t>
         </is>
       </c>
       <c r="AA84" s="2" t="inlineStr"/>
@@ -13133,13 +13155,17 @@
       </c>
       <c r="X85" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y85" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y85" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·周J超卖</t>
+        </is>
+      </c>
       <c r="Z85" s="2" t="inlineStr">
         <is>
-          <t>4+→4·1d ← 4→4+·15d</t>
+          <t>4→4+·15d</t>
         </is>
       </c>
       <c r="AA85" s="2" t="inlineStr"/>
@@ -15840,12 +15866,12 @@
       </c>
       <c r="Y103" s="2" t="inlineStr">
         <is>
-          <t>周J超卖·日线纠缠</t>
+          <t>站稳短均·周J超卖·日线纠缠</t>
         </is>
       </c>
       <c r="Z103" s="2" t="inlineStr">
         <is>
-          <t>4→4+·1d ← 4+→4·9d ← 4→4+·17d</t>
+          <t>4→4+·1d ← 4+→4·9d ← 3→4+·20d</t>
         </is>
       </c>
       <c r="AA103" s="2" t="inlineStr"/>
@@ -16309,7 +16335,7 @@
       </c>
       <c r="Z106" s="2" t="inlineStr">
         <is>
-          <t>4→4+·1d ← 4+→4·10d</t>
+          <t>4→4+·1d ← 4+→4·2d ← 4→4+·3d</t>
         </is>
       </c>
       <c r="AA106" s="2" t="inlineStr"/>
@@ -17057,13 +17083,17 @@
       </c>
       <c r="X111" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y111" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y111" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·周J超卖</t>
+        </is>
+      </c>
       <c r="Z111" s="2" t="inlineStr">
         <is>
-          <t>4+→4·2d ← 4→4+·5d</t>
+          <t>4→4+·7d</t>
         </is>
       </c>
       <c r="AA111" s="2" t="inlineStr"/>
@@ -17199,11 +17229,19 @@
       </c>
       <c r="X112" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y112" s="2" t="inlineStr"/>
-      <c r="Z112" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y112" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均</t>
+        </is>
+      </c>
+      <c r="Z112" s="2" t="inlineStr">
+        <is>
+          <t>4→4+·1d ← 4+→4·2d ← 4→4+·9d</t>
+        </is>
+      </c>
       <c r="AA112" s="2" t="inlineStr"/>
       <c r="AB112" s="2" t="inlineStr"/>
       <c r="AC112" s="2" t="inlineStr"/>
@@ -17806,7 +17844,7 @@
       </c>
       <c r="Y116" s="2" t="inlineStr">
         <is>
-          <t>周J超卖·日线纠缠</t>
+          <t>站稳短均·周J超卖·日线纠缠</t>
         </is>
       </c>
       <c r="Z116" s="2" t="inlineStr">
@@ -17947,13 +17985,17 @@
       </c>
       <c r="X117" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y117" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y117" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z117" s="2" t="inlineStr">
         <is>
-          <t>3→4·3d</t>
+          <t>3→4+·3d</t>
         </is>
       </c>
       <c r="AA117" s="2" t="inlineStr"/>
@@ -18698,7 +18740,7 @@
       </c>
       <c r="Y122" s="2" t="inlineStr">
         <is>
-          <t>周J超卖·底背离·日线纠缠</t>
+          <t>站稳短均·周J超卖·底背离·日线纠缠</t>
         </is>
       </c>
       <c r="Z122" s="2" t="inlineStr">
@@ -20213,7 +20255,7 @@
       <c r="Y132" s="2" t="inlineStr"/>
       <c r="Z132" s="2" t="inlineStr">
         <is>
-          <t>1+→1·16d ← 4→1+·18d</t>
+          <t>1+→1·16d ← 4+→1+·18d ← 4→4+·20d</t>
         </is>
       </c>
       <c r="AA132" s="2" t="inlineStr"/>
@@ -20826,7 +20868,7 @@
       </c>
       <c r="Y136" s="2" t="inlineStr">
         <is>
-          <t>周J超卖·底背离·日线纠缠</t>
+          <t>站稳短均·周J超卖·底背离·日线纠缠</t>
         </is>
       </c>
       <c r="Z136" s="2" t="inlineStr">
@@ -21436,7 +21478,7 @@
       </c>
       <c r="Y140" s="2" t="inlineStr">
         <is>
-          <t>周J超卖·日线纠缠</t>
+          <t>站稳短均·周J超卖·日线纠缠</t>
         </is>
       </c>
       <c r="Z140" s="2" t="inlineStr">
@@ -21747,7 +21789,7 @@
       <c r="Y142" s="2" t="inlineStr"/>
       <c r="Z142" s="2" t="inlineStr">
         <is>
-          <t>4+→4·5d ← 4→4+·7d</t>
+          <t>4+→4·5d ← 4→4+·8d ← 4+→4·17d</t>
         </is>
       </c>
       <c r="AA142" s="2" t="inlineStr"/>
@@ -21895,7 +21937,11 @@
         </is>
       </c>
       <c r="Y143" s="2" t="inlineStr"/>
-      <c r="Z143" s="2" t="inlineStr"/>
+      <c r="Z143" s="2" t="inlineStr">
+        <is>
+          <t>4+→4·2d ← 4→4+·3d ← 4+→4·6d</t>
+        </is>
+      </c>
       <c r="AA143" s="2" t="inlineStr"/>
       <c r="AB143" s="2" t="inlineStr"/>
       <c r="AC143" s="2" t="n">
@@ -22791,7 +22837,7 @@
       <c r="Y149" s="2" t="inlineStr"/>
       <c r="Z149" s="2" t="inlineStr">
         <is>
-          <t>1→4·15d</t>
+          <t>4+→4·6d ← 4→4+·11d ← 1→4·15d</t>
         </is>
       </c>
       <c r="AA149" s="2" t="inlineStr"/>
@@ -23681,7 +23727,7 @@
       <c r="Y155" s="2" t="inlineStr"/>
       <c r="Z155" s="2" t="inlineStr">
         <is>
-          <t>4+→4·3d ← 4→4+·7d ← 4+→4·10d</t>
+          <t>4+→4·3d</t>
         </is>
       </c>
       <c r="AA155" s="2" t="inlineStr"/>
@@ -25877,13 +25923,17 @@
       </c>
       <c r="X170" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y170" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y170" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均</t>
+        </is>
+      </c>
       <c r="Z170" s="2" t="inlineStr">
         <is>
-          <t>4+→4·7d ← 4→4+·18d</t>
+          <t>4→4+·19d</t>
         </is>
       </c>
       <c r="AA170" s="2" t="inlineStr"/>
@@ -26041,7 +26091,7 @@
       <c r="Y171" s="2" t="inlineStr"/>
       <c r="Z171" s="2" t="inlineStr">
         <is>
-          <t>4+→4·11d ← 4→4+·18d</t>
+          <t>4+→4·2d ← 4→4+·18d</t>
         </is>
       </c>
       <c r="AA171" s="2" t="inlineStr"/>
@@ -26341,7 +26391,7 @@
       <c r="Y173" s="2" t="inlineStr"/>
       <c r="Z173" s="2" t="inlineStr">
         <is>
-          <t>4→1·3d</t>
+          <t>4→1·3d ← 4+→4·4d ← 4→4+·5d</t>
         </is>
       </c>
       <c r="AA173" s="2" t="inlineStr"/>
@@ -27255,7 +27305,7 @@
       <c r="Y179" s="2" t="inlineStr"/>
       <c r="Z179" s="2" t="inlineStr">
         <is>
-          <t>1→4·9d</t>
+          <t>4+→4·7d ← 1→4+·9d</t>
         </is>
       </c>
       <c r="AA179" s="2" t="inlineStr"/>
@@ -27549,7 +27599,7 @@
       <c r="Y181" s="2" t="inlineStr"/>
       <c r="Z181" s="2" t="inlineStr">
         <is>
-          <t>4+→4·9d ← 4→4+·20d</t>
+          <t>4+→4·2d ← 4→4+·3d ← 4+→4·4d</t>
         </is>
       </c>
       <c r="AA181" s="2" t="inlineStr"/>
@@ -28231,7 +28281,7 @@
         </is>
       </c>
       <c r="C186" s="2" t="n">
-        <v>1389</v>
+        <v>1393</v>
       </c>
       <c r="D186" s="2" t="n">
         <v>47.18</v>
@@ -28293,23 +28343,23 @@
       <c r="AE186" s="2" t="inlineStr"/>
       <c r="AF186" s="2" t="inlineStr"/>
       <c r="AG186" s="2" t="n">
-        <v>32.32</v>
+        <v>32.4</v>
       </c>
       <c r="AH186" s="2" t="n">
-        <v>0.29</v>
+        <v>0.61</v>
       </c>
       <c r="AI186" s="2" t="n"/>
       <c r="AJ186" s="2" t="n">
-        <v>7.25</v>
+        <v>7.56</v>
       </c>
       <c r="AK186" s="2" t="n">
-        <v>-5.99</v>
+        <v>-5.68</v>
       </c>
       <c r="AL186" s="2" t="n">
-        <v>79.09999999999999</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="AM186" s="2" t="n">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="AN186" s="2" t="inlineStr"/>
       <c r="AO186" s="2" t="inlineStr"/>
@@ -28323,40 +28373,40 @@
         </is>
       </c>
       <c r="AS186" s="2" t="n">
-        <v>1386.8</v>
+        <v>1387.6</v>
       </c>
       <c r="AT186" s="2" t="n">
-        <v>1376.8</v>
+        <v>1377.2</v>
       </c>
       <c r="AU186" s="2" t="n">
-        <v>1390.517</v>
+        <v>1390.717</v>
       </c>
       <c r="AV186" s="2" t="n">
-        <v>1388.915</v>
+        <v>1389.048</v>
       </c>
       <c r="AW186" s="2" t="n">
-        <v>1349.996</v>
+        <v>1350.076</v>
       </c>
       <c r="AX186" s="2" t="n">
-        <v>1298.934</v>
+        <v>1298.974</v>
       </c>
       <c r="AY186" s="2" t="n">
-        <v>1300.685</v>
+        <v>1300.705</v>
       </c>
       <c r="AZ186" s="2" t="n">
-        <v>-0.011</v>
+        <v>0.0041</v>
       </c>
       <c r="BA186" s="2" t="n">
-        <v>-0.3414</v>
+        <v>-0.3339</v>
       </c>
       <c r="BB186" s="2" t="n">
-        <v>0.3495</v>
+        <v>0.3526</v>
       </c>
       <c r="BC186" s="2" t="n">
-        <v>0.116</v>
+        <v>0.1176</v>
       </c>
       <c r="BD186" s="2" t="n">
-        <v>0.3232</v>
+        <v>0.324</v>
       </c>
     </row>
     <row r="187">
@@ -28371,7 +28421,7 @@
         </is>
       </c>
       <c r="C187" s="2" t="n">
-        <v>7016</v>
+        <v>6911</v>
       </c>
       <c r="D187" s="2" t="n">
         <v>104.12</v>
@@ -28437,23 +28487,23 @@
       <c r="AE187" s="2" t="inlineStr"/>
       <c r="AF187" s="2" t="inlineStr"/>
       <c r="AG187" s="2" t="n">
-        <v>88.15000000000001</v>
+        <v>87.7</v>
       </c>
       <c r="AH187" s="2" t="n">
-        <v>17.72</v>
+        <v>15.99</v>
       </c>
       <c r="AI187" s="2" t="n"/>
       <c r="AJ187" s="2" t="n">
-        <v>-15.44</v>
+        <v>-17.17</v>
       </c>
       <c r="AK187" s="2" t="n">
-        <v>-12.8</v>
+        <v>-14.53</v>
       </c>
       <c r="AL187" s="2" t="n">
-        <v>21.8</v>
+        <v>21.6</v>
       </c>
       <c r="AM187" s="2" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AN187" s="2" t="inlineStr"/>
       <c r="AO187" s="2" t="n">
@@ -28471,40 +28521,40 @@
         </is>
       </c>
       <c r="AS187" s="2" t="n">
-        <v>7363.6</v>
+        <v>7342.6</v>
       </c>
       <c r="AT187" s="2" t="n">
-        <v>7980.9</v>
+        <v>7970.4</v>
       </c>
       <c r="AU187" s="2" t="n">
-        <v>7905.027</v>
+        <v>7899.777</v>
       </c>
       <c r="AV187" s="2" t="n">
-        <v>7663.406</v>
+        <v>7659.906</v>
       </c>
       <c r="AW187" s="2" t="n">
-        <v>7562.643</v>
+        <v>7560.543</v>
       </c>
       <c r="AX187" s="2" t="n">
-        <v>8479.188</v>
+        <v>8478.138000000001</v>
       </c>
       <c r="AY187" s="2" t="n">
-        <v>6205.301</v>
+        <v>6204.776</v>
       </c>
       <c r="AZ187" s="2" t="n">
-        <v>-2.2389</v>
+        <v>-2.3044</v>
       </c>
       <c r="BA187" s="2" t="n">
-        <v>0.2582</v>
+        <v>0.2235</v>
       </c>
       <c r="BB187" s="2" t="n">
-        <v>0.2285</v>
+        <v>0.214</v>
       </c>
       <c r="BC187" s="2" t="n">
-        <v>0.3434</v>
+        <v>0.3369</v>
       </c>
       <c r="BD187" s="2" t="n">
-        <v>0.8815</v>
+        <v>0.877</v>
       </c>
     </row>
     <row r="188">
@@ -29849,13 +29899,17 @@
       </c>
       <c r="X197" s="2" t="inlineStr">
         <is>
-          <t>4</t>
-        </is>
-      </c>
-      <c r="Y197" s="2" t="inlineStr"/>
+          <t>4+</t>
+        </is>
+      </c>
+      <c r="Y197" s="2" t="inlineStr">
+        <is>
+          <t>站稳短均·周J超卖·日线纠缠</t>
+        </is>
+      </c>
       <c r="Z197" s="2" t="inlineStr">
         <is>
-          <t>4+→4·1d ← 4→4+·18d ← 4+→4·19d</t>
+          <t>4→4+·18d ← 4+→4·19d</t>
         </is>
       </c>
       <c r="AA197" s="2" t="inlineStr"/>
@@ -30341,7 +30395,7 @@
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Stage (Weinstein 大阶段 v2.2引擎: EMA30W(150日EMA)锚, 判定优先级从高到低): ①均线排列覆盖: MA20&gt;MA50&gt;MA100&gt;MA150(简单均线)多头排列→强制Stage2; MA20&lt;MA50&lt;MA100&lt;MA150空头排列→强制Stage4(忽略斜率, 解决慢磨盲区) ②斜率双确认: EMA30W变化年化(4周×13与13周×3.88)均&gt;+8%→2; 均&lt;-6%→4(不对称) ③放平带: 52周位置+价格确认分1/3(3:pos&gt;0.55且价≥0.95×EMA30W; 1:pos&lt;0.45且价≤1.05×; 0.45~0.55滞回)。降级层(v2.2): 151-252根新股→①可用②仅≥215根③用上市以来位置, 标记列带'新'; ≤150根→NA</t>
+          <t xml:space="preserve">  Stage (Weinstein 大阶段 v2.3引擎: EMA30W(150日EMA)锚, 判定优先级从高到低): ①均线排列覆盖: MA20&gt;MA50&gt;MA100&gt;MA150(简单均线)多头排列→强制Stage2; MA20&lt;MA50&lt;MA100&lt;MA150空头排列→强制Stage4(忽略斜率, 解决慢磨盲区) ②斜率双确认: EMA30W变化年化(4周×13与13周×3.88)均&gt;+8%→2; 均&lt;-6%→4(不对称) ③放平带: 52周位置+价格确认分1/3(3:pos&gt;0.55且价≥0.95×EMA30W; 1:pos&lt;0.45且价≤1.05×; 0.45~0.55滞回)。降级层(v2.2): 151-252根新股→①可用②仅≥215根③用上市以来位置, 标记列带'新'; ≤150根→NA</t>
         </is>
       </c>
     </row>
@@ -30362,14 +30416,14 @@
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  子档(v2.1): 4+=止跌(日线MA5/10/20纠缠+快线&gt;慢线+周J超卖或底背离, 价&lt;EMA10W) | 1=筑底(不区分价格vs EMA10W) | 1+=强筑底(站稳MA5/10/20全三条+全上行+周MACD DIF&gt;DEA) | 2A=修复态或刚确立(≤10日) | 2B=满配(slope10&gt;0·EMA10W&gt;EMA30W·10日前也是) | 2C=满配+延伸/减速/顶背离 | 3/4不分档</t>
+          <t xml:space="preserve">  子档(v2.3): 4+=双路径: A止跌(纠缠/快慢线+周J超卖或底背离, 价&lt;EMA10W) ∨ B短期修复(站稳MA5/10/20三条) | 1=筑底(不区分价格vs EMA10W) | 1+=强筑底(站稳MA5/10/20全三条+全上行+周MACD DIF&gt;DEA) | 2A=修复态或刚确立(≤10日) | 2B=满配(slope10&gt;0·EMA10W&gt;EMA30W·10日前也是) | 2C=满配+延伸/减速/顶背离 | 3/4不分档</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  子档标记: 状态描述列(与子档列分开)。4+→周J超卖·底背离·日线纠缠(止跌命中条件); 1+→预金叉(EMA10W/30W将≤20日内纠缠或金叉)·纠缠·底背离; 2C→延伸(价超EMA30W达25%)·减速·顶背离; 新=降级层(上市151-252根弱规则档)</t>
+          <t xml:space="preserve">  子档标记: 状态描述列(与子档列分开)。4+→站稳短均(路径B)·周J超卖·底背离·日线纠缠(路径A); 1+→预金叉(EMA10W/30W将≤20日内纠缠或金叉)·纠缠·底背离; 2C→延伸(价超EMA30W达25%)·减速·顶背离; 新=降级层(上市151-252根弱规则档)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-18
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -899,14 +899,14 @@
         <v>80.18000000000001</v>
       </c>
       <c r="AI2" s="2" t="n">
-        <v>-0.06</v>
+        <v>0.37</v>
       </c>
       <c r="AJ2" s="2" t="n"/>
       <c r="AK2" s="2" t="n">
-        <v>-28.57</v>
+        <v>-22.32</v>
       </c>
       <c r="AL2" s="2" t="n">
-        <v>-16.09</v>
+        <v>-12.74</v>
       </c>
       <c r="AM2" s="2" t="n">
         <v>2.4</v>
@@ -1056,14 +1056,14 @@
         <v>96.52</v>
       </c>
       <c r="AI3" s="2" t="n">
-        <v>17.75</v>
+        <v>15.97</v>
       </c>
       <c r="AJ3" s="2" t="n"/>
       <c r="AK3" s="2" t="n">
-        <v>-14.31</v>
+        <v>-12.88</v>
       </c>
       <c r="AL3" s="2" t="n">
-        <v>-1.24</v>
+        <v>3.47</v>
       </c>
       <c r="AM3" s="2" t="n">
         <v>55.6</v>
@@ -1205,14 +1205,14 @@
         <v>130.74</v>
       </c>
       <c r="AI4" s="2" t="n">
-        <v>35.66</v>
+        <v>41.27</v>
       </c>
       <c r="AJ4" s="2" t="n"/>
       <c r="AK4" s="2" t="n">
-        <v>-34.03</v>
+        <v>-23.63</v>
       </c>
       <c r="AL4" s="2" t="n">
-        <v>-23.18</v>
+        <v>-14.73</v>
       </c>
       <c r="AM4" s="2" t="n">
         <v>61.3</v>
@@ -1354,14 +1354,14 @@
         <v>27.53</v>
       </c>
       <c r="AI5" s="2" t="n">
-        <v>-8.56</v>
+        <v>-9.539999999999999</v>
       </c>
       <c r="AJ5" s="2" t="n"/>
       <c r="AK5" s="2" t="n">
-        <v>3.73</v>
+        <v>3.07</v>
       </c>
       <c r="AL5" s="2" t="n">
-        <v>3.99</v>
+        <v>2.07</v>
       </c>
       <c r="AM5" s="2" t="n">
         <v>13.8</v>
@@ -1497,14 +1497,14 @@
         <v>45.11</v>
       </c>
       <c r="AI6" s="2" t="n">
-        <v>-8.06</v>
+        <v>-7.1</v>
       </c>
       <c r="AJ6" s="2" t="n"/>
       <c r="AK6" s="2" t="n">
-        <v>-4.98</v>
+        <v>-6.01</v>
       </c>
       <c r="AL6" s="2" t="n">
-        <v>-0.92</v>
+        <v>1.05</v>
       </c>
       <c r="AM6" s="2" t="n">
         <v>22.5</v>
@@ -1658,14 +1658,14 @@
         <v>41.56</v>
       </c>
       <c r="AI7" s="2" t="n">
-        <v>9.82</v>
+        <v>9</v>
       </c>
       <c r="AJ7" s="2" t="n"/>
       <c r="AK7" s="2" t="n">
-        <v>15.7</v>
+        <v>12.66</v>
       </c>
       <c r="AL7" s="2" t="n">
-        <v>11.07</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="AM7" s="2" t="n">
         <v>98.40000000000001</v>
@@ -1815,14 +1815,14 @@
         <v>16.94</v>
       </c>
       <c r="AI8" s="2" t="n">
-        <v>-1.15</v>
+        <v>0.03</v>
       </c>
       <c r="AJ8" s="2" t="n"/>
       <c r="AK8" s="2" t="n">
-        <v>11.84</v>
+        <v>12.05</v>
       </c>
       <c r="AL8" s="2" t="n">
-        <v>6.14</v>
+        <v>4.39</v>
       </c>
       <c r="AM8" s="2" t="n">
         <v>74.59999999999999</v>
@@ -1958,14 +1958,14 @@
         <v>-32.79</v>
       </c>
       <c r="AI9" s="2" t="n">
-        <v>-27.95</v>
+        <v>-27.86</v>
       </c>
       <c r="AJ9" s="2" t="n"/>
       <c r="AK9" s="2" t="n">
-        <v>7.98</v>
+        <v>6.98</v>
       </c>
       <c r="AL9" s="2" t="n">
-        <v>-0.08</v>
+        <v>-0.6</v>
       </c>
       <c r="AM9" s="2" t="n">
         <v>8.5</v>
@@ -2111,14 +2111,14 @@
         <v>-30.66</v>
       </c>
       <c r="AI10" s="2" t="n">
-        <v>-20.49</v>
+        <v>-18.74</v>
       </c>
       <c r="AJ10" s="2" t="n"/>
       <c r="AK10" s="2" t="n">
-        <v>5.86</v>
+        <v>7.72</v>
       </c>
       <c r="AL10" s="2" t="n">
-        <v>1.52</v>
+        <v>0.33</v>
       </c>
       <c r="AM10" s="2" t="n">
         <v>57.9</v>
@@ -2262,14 +2262,14 @@
         <v>33.18</v>
       </c>
       <c r="AI11" s="2" t="n">
-        <v>6.38</v>
+        <v>7.56</v>
       </c>
       <c r="AJ11" s="2" t="n"/>
       <c r="AK11" s="2" t="n">
-        <v>12.9</v>
+        <v>11.03</v>
       </c>
       <c r="AL11" s="2" t="n">
-        <v>5.86</v>
+        <v>6.83</v>
       </c>
       <c r="AM11" s="2" t="n">
         <v>48.7</v>
@@ -2356,14 +2356,14 @@
       <c r="P12" s="2" t="inlineStr"/>
       <c r="Q12" s="2" t="inlineStr"/>
       <c r="R12" s="2" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="S12" s="2" t="n">
         <v>8</v>
       </c>
       <c r="T12" s="2" t="inlineStr">
         <is>
-          <t>0011111001</t>
+          <t>0011101001</t>
         </is>
       </c>
       <c r="U12" s="2" t="inlineStr">
@@ -2407,14 +2407,14 @@
         <v>1.92</v>
       </c>
       <c r="AI12" s="2" t="n">
-        <v>-6.51</v>
+        <v>-6.75</v>
       </c>
       <c r="AJ12" s="2" t="n"/>
       <c r="AK12" s="2" t="n">
-        <v>7.59</v>
+        <v>6.28</v>
       </c>
       <c r="AL12" s="2" t="n">
-        <v>8.720000000000001</v>
+        <v>6.68</v>
       </c>
       <c r="AM12" s="2" t="n">
         <v>31</v>
@@ -2558,14 +2558,14 @@
         <v>108.01</v>
       </c>
       <c r="AI13" s="2" t="n">
-        <v>10.28</v>
+        <v>8.15</v>
       </c>
       <c r="AJ13" s="2" t="n"/>
       <c r="AK13" s="2" t="n">
-        <v>-25.39</v>
+        <v>-22.07</v>
       </c>
       <c r="AL13" s="2" t="n">
-        <v>-29.38</v>
+        <v>-27.36</v>
       </c>
       <c r="AM13" s="2" t="n">
         <v>43.9</v>
@@ -2705,14 +2705,14 @@
         <v>36.08</v>
       </c>
       <c r="AI14" s="2" t="n">
-        <v>-9.33</v>
+        <v>-10.1</v>
       </c>
       <c r="AJ14" s="2" t="n"/>
       <c r="AK14" s="2" t="n">
-        <v>-8.16</v>
+        <v>-6.83</v>
       </c>
       <c r="AL14" s="2" t="n">
-        <v>-0.64</v>
+        <v>1.02</v>
       </c>
       <c r="AM14" s="2" t="n">
         <v>20</v>
@@ -2846,14 +2846,14 @@
         <v>19.67</v>
       </c>
       <c r="AI15" s="2" t="n">
-        <v>-22.05</v>
+        <v>-22.1</v>
       </c>
       <c r="AJ15" s="2" t="n"/>
       <c r="AK15" s="2" t="n">
-        <v>-4.54</v>
+        <v>-5.5</v>
       </c>
       <c r="AL15" s="2" t="n">
-        <v>2.13</v>
+        <v>2.25</v>
       </c>
       <c r="AM15" s="2" t="n">
         <v>15.6</v>
@@ -2993,14 +2993,14 @@
         <v>17.94</v>
       </c>
       <c r="AI16" s="2" t="n">
-        <v>-22.35</v>
+        <v>-22.24</v>
       </c>
       <c r="AJ16" s="2" t="n"/>
       <c r="AK16" s="2" t="n">
-        <v>-5.76</v>
+        <v>-4.81</v>
       </c>
       <c r="AL16" s="2" t="n">
-        <v>-2.46</v>
+        <v>-2.97</v>
       </c>
       <c r="AM16" s="2" t="n">
         <v>7.9</v>
@@ -3144,14 +3144,14 @@
         <v>10.44</v>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>-14.7</v>
+        <v>-14.31</v>
       </c>
       <c r="AJ17" s="2" t="n"/>
       <c r="AK17" s="2" t="n">
-        <v>1.06</v>
+        <v>3.99</v>
       </c>
       <c r="AL17" s="2" t="n">
-        <v>-1.62</v>
+        <v>-3.6</v>
       </c>
       <c r="AM17" s="2" t="n">
         <v>8.800000000000001</v>
@@ -3289,14 +3289,14 @@
         <v>34.05</v>
       </c>
       <c r="AI18" s="2" t="n">
-        <v>2.3</v>
+        <v>2.7</v>
       </c>
       <c r="AJ18" s="2" t="n"/>
       <c r="AK18" s="2" t="n">
-        <v>-0.26</v>
+        <v>2.24</v>
       </c>
       <c r="AL18" s="2" t="n">
-        <v>9.75</v>
+        <v>9.359999999999999</v>
       </c>
       <c r="AM18" s="2" t="n">
         <v>78.40000000000001</v>
@@ -3432,14 +3432,14 @@
         <v>-3.32</v>
       </c>
       <c r="AI19" s="2" t="n">
-        <v>-23.37</v>
+        <v>-22.58</v>
       </c>
       <c r="AJ19" s="2" t="n"/>
       <c r="AK19" s="2" t="n">
-        <v>-4.97</v>
+        <v>-2.72</v>
       </c>
       <c r="AL19" s="2" t="n">
-        <v>-1.07</v>
+        <v>-0.88</v>
       </c>
       <c r="AM19" s="2" t="n">
         <v>4.1</v>
@@ -3577,14 +3577,14 @@
         <v>-5.81</v>
       </c>
       <c r="AI20" s="2" t="n">
-        <v>-31.39</v>
+        <v>-32.85</v>
       </c>
       <c r="AJ20" s="2" t="n"/>
       <c r="AK20" s="2" t="n">
-        <v>-5.47</v>
+        <v>-7.32</v>
       </c>
       <c r="AL20" s="2" t="n">
-        <v>-28.73</v>
+        <v>-29.97</v>
       </c>
       <c r="AM20" s="2" t="n">
         <v>7.5</v>
@@ -3677,14 +3677,14 @@
       <c r="P21" s="2" t="inlineStr"/>
       <c r="Q21" s="2" t="inlineStr"/>
       <c r="R21" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S21" s="2" t="n">
         <v>1</v>
       </c>
       <c r="T21" s="2" t="inlineStr">
         <is>
-          <t>0010011000</t>
+          <t>0010001000</t>
         </is>
       </c>
       <c r="U21" s="2" t="inlineStr">
@@ -3724,14 +3724,14 @@
         <v>40.39</v>
       </c>
       <c r="AI21" s="2" t="n">
-        <v>-1.03</v>
+        <v>-1.14</v>
       </c>
       <c r="AJ21" s="2" t="n"/>
       <c r="AK21" s="2" t="n">
-        <v>-11.75</v>
+        <v>-7.79</v>
       </c>
       <c r="AL21" s="2" t="n">
-        <v>3.13</v>
+        <v>1.97</v>
       </c>
       <c r="AM21" s="2" t="n">
         <v>29.8</v>
@@ -3877,14 +3877,14 @@
         <v>85.56</v>
       </c>
       <c r="AI22" s="2" t="n">
-        <v>19.96</v>
+        <v>18.75</v>
       </c>
       <c r="AJ22" s="2" t="n"/>
       <c r="AK22" s="2" t="n">
-        <v>-14.26</v>
+        <v>-15.9</v>
       </c>
       <c r="AL22" s="2" t="n">
-        <v>3.51</v>
+        <v>3.97</v>
       </c>
       <c r="AM22" s="2" t="n">
         <v>82.59999999999999</v>
@@ -4034,14 +4034,14 @@
         <v>46.38</v>
       </c>
       <c r="AI23" s="2" t="n">
-        <v>7.49</v>
+        <v>8.41</v>
       </c>
       <c r="AJ23" s="2" t="n"/>
       <c r="AK23" s="2" t="n">
-        <v>5.41</v>
+        <v>6.83</v>
       </c>
       <c r="AL23" s="2" t="n">
-        <v>4.26</v>
+        <v>4.35</v>
       </c>
       <c r="AM23" s="2" t="n">
         <v>54.7</v>
@@ -4128,19 +4128,19 @@
       <c r="P24" s="2" t="inlineStr"/>
       <c r="Q24" s="2" t="inlineStr"/>
       <c r="R24" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S24" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T24" s="2" t="inlineStr">
         <is>
-          <t>0111110110</t>
+          <t>0111100110</t>
         </is>
       </c>
       <c r="U24" s="2" t="inlineStr">
         <is>
-          <t>0111110110</t>
+          <t>0111100110</t>
         </is>
       </c>
       <c r="V24" s="2" t="inlineStr">
@@ -4179,14 +4179,14 @@
         <v>47.89</v>
       </c>
       <c r="AI24" s="2" t="n">
-        <v>0.03</v>
+        <v>3.51</v>
       </c>
       <c r="AJ24" s="2" t="n"/>
       <c r="AK24" s="2" t="n">
-        <v>-10.31</v>
+        <v>-8.06</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>8.5</v>
+        <v>11.58</v>
       </c>
       <c r="AM24" s="2" t="n">
         <v>47.2</v>
@@ -4324,14 +4324,14 @@
         <v>110.58</v>
       </c>
       <c r="AI25" s="2" t="n">
-        <v>27.53</v>
+        <v>28.06</v>
       </c>
       <c r="AJ25" s="2" t="n"/>
       <c r="AK25" s="2" t="n">
-        <v>-10.74</v>
+        <v>-5.63</v>
       </c>
       <c r="AL25" s="2" t="n">
-        <v>1.77</v>
+        <v>8.369999999999999</v>
       </c>
       <c r="AM25" s="2" t="n">
         <v>3</v>
@@ -4471,14 +4471,14 @@
         <v>87.66</v>
       </c>
       <c r="AI26" s="2" t="n">
-        <v>15.48</v>
+        <v>16.21</v>
       </c>
       <c r="AJ26" s="2" t="n"/>
       <c r="AK26" s="2" t="n">
-        <v>-22.77</v>
+        <v>-16.95</v>
       </c>
       <c r="AL26" s="2" t="n">
-        <v>-17.67</v>
+        <v>-14.31</v>
       </c>
       <c r="AM26" s="2" t="n">
         <v>21.6</v>
@@ -4626,14 +4626,14 @@
         <v>-2.71</v>
       </c>
       <c r="AI27" s="2" t="n">
-        <v>-5.55</v>
+        <v>-5.71</v>
       </c>
       <c r="AJ27" s="2" t="n"/>
       <c r="AK27" s="2" t="n">
-        <v>9.550000000000001</v>
+        <v>8.58</v>
       </c>
       <c r="AL27" s="2" t="n">
-        <v>13.27</v>
+        <v>11.59</v>
       </c>
       <c r="AM27" s="2" t="n">
         <v>93.7</v>
@@ -4781,14 +4781,14 @@
         <v>-9.43</v>
       </c>
       <c r="AI28" s="2" t="n">
-        <v>-23.08</v>
+        <v>-19.92</v>
       </c>
       <c r="AJ28" s="2" t="n"/>
       <c r="AK28" s="2" t="n">
-        <v>2.65</v>
+        <v>7.21</v>
       </c>
       <c r="AL28" s="2" t="n">
-        <v>-0.16</v>
+        <v>1.08</v>
       </c>
       <c r="AM28" s="2" t="n">
         <v>26.4</v>
@@ -4926,14 +4926,14 @@
         <v>92.92</v>
       </c>
       <c r="AI29" s="2" t="n">
-        <v>15.89</v>
+        <v>16.24</v>
       </c>
       <c r="AJ29" s="2" t="n"/>
       <c r="AK29" s="2" t="n">
-        <v>-10.26</v>
+        <v>-11.46</v>
       </c>
       <c r="AL29" s="2" t="n">
-        <v>7.3</v>
+        <v>8.26</v>
       </c>
       <c r="AM29" s="2" t="n">
         <v>37.7</v>
@@ -5081,14 +5081,14 @@
         <v>7.88</v>
       </c>
       <c r="AI30" s="2" t="n">
-        <v>-11.96</v>
+        <v>-10.7</v>
       </c>
       <c r="AJ30" s="2" t="n"/>
       <c r="AK30" s="2" t="n">
-        <v>6.75</v>
+        <v>7.13</v>
       </c>
       <c r="AL30" s="2" t="n">
-        <v>8.91</v>
+        <v>10.37</v>
       </c>
       <c r="AM30" s="2" t="n">
         <v>49.7</v>
@@ -5230,14 +5230,14 @@
         <v>-4.78</v>
       </c>
       <c r="AI31" s="2" t="n">
-        <v>-12.19</v>
+        <v>-12.16</v>
       </c>
       <c r="AJ31" s="2" t="n"/>
       <c r="AK31" s="2" t="n">
-        <v>-0.55</v>
+        <v>1.51</v>
       </c>
       <c r="AL31" s="2" t="n">
-        <v>-3.15</v>
+        <v>-2.89</v>
       </c>
       <c r="AM31" s="2" t="n">
         <v>40.7</v>
@@ -5377,14 +5377,14 @@
         <v>22.24</v>
       </c>
       <c r="AI32" s="2" t="n">
-        <v>2.16</v>
+        <v>3.63</v>
       </c>
       <c r="AJ32" s="2" t="n"/>
       <c r="AK32" s="2" t="n">
-        <v>10.92</v>
+        <v>12.01</v>
       </c>
       <c r="AL32" s="2" t="n">
-        <v>-1.92</v>
+        <v>-3.45</v>
       </c>
       <c r="AM32" s="2" t="n">
         <v>79</v>
@@ -5518,14 +5518,14 @@
         <v>11.87</v>
       </c>
       <c r="AI33" s="2" t="n">
-        <v>-10.72</v>
+        <v>-10.66</v>
       </c>
       <c r="AJ33" s="2" t="n"/>
       <c r="AK33" s="2" t="n">
-        <v>7.78</v>
+        <v>7.96</v>
       </c>
       <c r="AL33" s="2" t="n">
-        <v>-3.36</v>
+        <v>-4.83</v>
       </c>
       <c r="AM33" s="2" t="n">
         <v>35.2</v>
@@ -5663,14 +5663,14 @@
         <v>34.32</v>
       </c>
       <c r="AI34" s="2" t="n">
-        <v>1.48</v>
+        <v>1.82</v>
       </c>
       <c r="AJ34" s="2" t="n"/>
       <c r="AK34" s="2" t="n">
-        <v>8.43</v>
+        <v>6.75</v>
       </c>
       <c r="AL34" s="2" t="n">
-        <v>6.28</v>
+        <v>5.36</v>
       </c>
       <c r="AM34" s="2" t="n">
         <v>50.5</v>
@@ -5816,14 +5816,14 @@
         <v>44.6</v>
       </c>
       <c r="AI35" s="2" t="n">
-        <v>9.73</v>
+        <v>9.82</v>
       </c>
       <c r="AJ35" s="2" t="n"/>
       <c r="AK35" s="2" t="n">
-        <v>7.32</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AL35" s="2" t="n">
-        <v>-4.97</v>
+        <v>-4.98</v>
       </c>
       <c r="AM35" s="2" t="n">
         <v>85.90000000000001</v>
@@ -5967,14 +5967,14 @@
         <v>11.97</v>
       </c>
       <c r="AI36" s="2" t="n">
-        <v>-9.619999999999999</v>
+        <v>-9.16</v>
       </c>
       <c r="AJ36" s="2" t="n"/>
       <c r="AK36" s="2" t="n">
-        <v>7.4</v>
+        <v>9.08</v>
       </c>
       <c r="AL36" s="2" t="n">
-        <v>-1.61</v>
+        <v>-3.79</v>
       </c>
       <c r="AM36" s="2" t="n">
         <v>75</v>
@@ -6066,7 +6066,7 @@
         <v>3</v>
       </c>
       <c r="S37" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T37" s="2" t="inlineStr">
         <is>
@@ -6075,7 +6075,7 @@
       </c>
       <c r="U37" s="2" t="inlineStr">
         <is>
-          <t>0110011000</t>
+          <t>0110001000</t>
         </is>
       </c>
       <c r="V37" s="2" t="inlineStr">
@@ -6110,14 +6110,14 @@
         <v>69.38</v>
       </c>
       <c r="AI37" s="2" t="n">
-        <v>5.76</v>
+        <v>6.83</v>
       </c>
       <c r="AJ37" s="2" t="n"/>
       <c r="AK37" s="2" t="n">
-        <v>-12.46</v>
+        <v>-9.93</v>
       </c>
       <c r="AL37" s="2" t="n">
-        <v>-0.13</v>
+        <v>1.35</v>
       </c>
       <c r="AM37" s="2" t="n">
         <v>26.1</v>
@@ -6263,14 +6263,14 @@
         <v>35.32</v>
       </c>
       <c r="AI38" s="2" t="n">
-        <v>3.94</v>
+        <v>4.4</v>
       </c>
       <c r="AJ38" s="2" t="n"/>
       <c r="AK38" s="2" t="n">
-        <v>7.89</v>
+        <v>7.99</v>
       </c>
       <c r="AL38" s="2" t="n">
-        <v>-7.07</v>
+        <v>-6.73</v>
       </c>
       <c r="AM38" s="2" t="n">
         <v>71.90000000000001</v>
@@ -6414,14 +6414,14 @@
         <v>29.93</v>
       </c>
       <c r="AI39" s="2" t="n">
-        <v>-5.26</v>
+        <v>-5.51</v>
       </c>
       <c r="AJ39" s="2" t="n"/>
       <c r="AK39" s="2" t="n">
-        <v>7.7</v>
+        <v>7.79</v>
       </c>
       <c r="AL39" s="2" t="n">
-        <v>-5.56</v>
+        <v>-6.33</v>
       </c>
       <c r="AM39" s="2" t="n">
         <v>67.2</v>
@@ -6561,14 +6561,14 @@
         <v>60.79</v>
       </c>
       <c r="AI40" s="2" t="n">
-        <v>19.28</v>
+        <v>17.09</v>
       </c>
       <c r="AJ40" s="2" t="n"/>
       <c r="AK40" s="2" t="n">
-        <v>12.57</v>
+        <v>6.78</v>
       </c>
       <c r="AL40" s="2" t="n">
-        <v>2.42</v>
+        <v>-1.96</v>
       </c>
       <c r="AM40" s="2" t="n">
         <v>99.09999999999999</v>
@@ -6714,14 +6714,14 @@
         <v>68.59</v>
       </c>
       <c r="AI41" s="2" t="n">
-        <v>20.57</v>
+        <v>19.71</v>
       </c>
       <c r="AJ41" s="2" t="n"/>
       <c r="AK41" s="2" t="n">
-        <v>13.03</v>
+        <v>9.720000000000001</v>
       </c>
       <c r="AL41" s="2" t="n">
-        <v>4.61</v>
+        <v>1.78</v>
       </c>
       <c r="AM41" s="2" t="n">
         <v>99.7</v>
@@ -6867,14 +6867,14 @@
         <v>68.56</v>
       </c>
       <c r="AI42" s="2" t="n">
-        <v>22.69</v>
+        <v>21.57</v>
       </c>
       <c r="AJ42" s="2" t="n"/>
       <c r="AK42" s="2" t="n">
-        <v>14.11</v>
+        <v>10.05</v>
       </c>
       <c r="AL42" s="2" t="n">
-        <v>0.09</v>
+        <v>-3.16</v>
       </c>
       <c r="AM42" s="2" t="n">
         <v>88.7</v>
@@ -7012,14 +7012,14 @@
         <v>34.74</v>
       </c>
       <c r="AI43" s="2" t="n">
-        <v>3.95</v>
+        <v>1.37</v>
       </c>
       <c r="AJ43" s="2" t="n"/>
       <c r="AK43" s="2" t="n">
-        <v>10.17</v>
+        <v>6.24</v>
       </c>
       <c r="AL43" s="2" t="n">
-        <v>12.83</v>
+        <v>9.1</v>
       </c>
       <c r="AM43" s="2" t="n">
         <v>28</v>
@@ -15668,7 +15668,7 @@
         </is>
       </c>
       <c r="C101" s="2" t="n">
-        <v>15.42</v>
+        <v>15.44</v>
       </c>
       <c r="D101" s="2" t="n">
         <v>29.76</v>
@@ -15691,14 +15691,14 @@
       <c r="P101" s="2" t="inlineStr"/>
       <c r="Q101" s="2" t="inlineStr"/>
       <c r="R101" s="2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="S101" s="2" t="n">
         <v>6</v>
       </c>
       <c r="T101" s="2" t="inlineStr">
         <is>
-          <t>0111111001</t>
+          <t>0111111011</t>
         </is>
       </c>
       <c r="U101" s="2" t="inlineStr">
@@ -15739,22 +15739,22 @@
       <c r="AF101" s="2" t="inlineStr"/>
       <c r="AG101" s="2" t="inlineStr"/>
       <c r="AH101" s="2" t="n">
-        <v>45.83</v>
+        <v>45.87</v>
       </c>
       <c r="AI101" s="2" t="n">
-        <v>9.369999999999999</v>
+        <v>9.51</v>
       </c>
       <c r="AJ101" s="2" t="n">
-        <v>12.74</v>
+        <v>12.89</v>
       </c>
       <c r="AK101" s="2" t="n">
-        <v>0.99</v>
+        <v>1.13</v>
       </c>
       <c r="AL101" s="2" t="n">
-        <v>0.4</v>
+        <v>0.54</v>
       </c>
       <c r="AM101" s="2" t="n">
-        <v>55.3</v>
+        <v>55.4</v>
       </c>
       <c r="AN101" s="2" t="n">
         <v>54</v>
@@ -15769,19 +15769,19 @@
         </is>
       </c>
       <c r="AT101" s="2" t="n">
-        <v>15.34</v>
+        <v>15.344</v>
       </c>
       <c r="AU101" s="2" t="n">
-        <v>15.243</v>
+        <v>15.245</v>
       </c>
       <c r="AV101" s="2" t="n">
-        <v>14.943</v>
+        <v>14.944</v>
       </c>
       <c r="AW101" s="2" t="n">
         <v>15.288</v>
       </c>
       <c r="AX101" s="2" t="n">
-        <v>15.355</v>
+        <v>15.356</v>
       </c>
       <c r="AY101" s="2" t="n">
         <v>14.804</v>
@@ -15790,19 +15790,19 @@
         <v>14.254</v>
       </c>
       <c r="BA101" s="2" t="n">
-        <v>1.1935</v>
+        <v>1.2005</v>
       </c>
       <c r="BB101" s="2" t="n">
-        <v>-0.08690000000000001</v>
+        <v>-0.0834</v>
       </c>
       <c r="BC101" s="2" t="n">
-        <v>0.2571</v>
+        <v>0.2585</v>
       </c>
       <c r="BD101" s="2" t="n">
-        <v>0.0547</v>
+        <v>0.0554</v>
       </c>
       <c r="BE101" s="2" t="n">
-        <v>0.4583</v>
+        <v>0.4587</v>
       </c>
     </row>
     <row r="102">
@@ -19008,7 +19008,7 @@
         </is>
       </c>
       <c r="C123" s="2" t="n">
-        <v>709.325</v>
+        <v>709.33</v>
       </c>
       <c r="D123" s="2" t="n">
         <v>101.54</v>
@@ -19107,10 +19107,10 @@
         </is>
       </c>
       <c r="AT123" s="2" t="n">
-        <v>737.809</v>
+        <v>737.8099999999999</v>
       </c>
       <c r="AU123" s="2" t="n">
-        <v>733.069</v>
+        <v>733.0700000000001</v>
       </c>
       <c r="AV123" s="2" t="n">
         <v>735.775</v>
@@ -19119,7 +19119,7 @@
         <v>708.13</v>
       </c>
       <c r="AX123" s="2" t="n">
-        <v>654.955</v>
+        <v>654.956</v>
       </c>
       <c r="AY123" s="2" t="n">
         <v>627.479</v>
@@ -19131,7 +19131,7 @@
         <v>0.3963</v>
       </c>
       <c r="BB123" s="2" t="n">
-        <v>1.2094</v>
+        <v>1.2095</v>
       </c>
       <c r="BC123" s="2" t="n">
         <v>1.2651</v>
@@ -19309,7 +19309,7 @@
         <v>18.82</v>
       </c>
       <c r="D125" s="2" t="n">
-        <v>-15.04</v>
+        <v>-15.01</v>
       </c>
       <c r="E125" s="2" t="inlineStr"/>
       <c r="F125" s="2" t="inlineStr">
@@ -20186,10 +20186,10 @@
         </is>
       </c>
       <c r="AT130" s="2" t="n">
-        <v>249.787</v>
+        <v>249.788</v>
       </c>
       <c r="AU130" s="2" t="n">
-        <v>264.157</v>
+        <v>264.158</v>
       </c>
       <c r="AV130" s="2" t="n">
         <v>263.114</v>
@@ -20204,13 +20204,13 @@
         <v>240.697</v>
       </c>
       <c r="AZ130" s="2" t="n">
-        <v>175.784</v>
+        <v>175.785</v>
       </c>
       <c r="BA130" s="2" t="n">
-        <v>-1.3522</v>
+        <v>-1.3521</v>
       </c>
       <c r="BB130" s="2" t="n">
-        <v>0.9452</v>
+        <v>0.9453</v>
       </c>
       <c r="BC130" s="2" t="n">
         <v>1.0014</v>
@@ -28232,7 +28232,7 @@
         <v>134.18</v>
       </c>
       <c r="D184" s="2" t="n">
-        <v>9.630000000000001</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="E184" s="2" t="inlineStr"/>
       <c r="F184" s="2" t="inlineStr"/>
@@ -28552,19 +28552,19 @@
       <c r="P186" s="2" t="inlineStr"/>
       <c r="Q186" s="2" t="inlineStr"/>
       <c r="R186" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="S186" s="2" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="T186" s="2" t="inlineStr">
         <is>
-          <t>0111111100</t>
+          <t>0111101100</t>
         </is>
       </c>
       <c r="U186" s="2" t="inlineStr">
         <is>
-          <t>0111111100</t>
+          <t>0111101100</t>
         </is>
       </c>
       <c r="V186" s="2" t="inlineStr">
@@ -28597,14 +28597,14 @@
         <v>32.28</v>
       </c>
       <c r="AI186" s="2" t="n">
-        <v>1.13</v>
+        <v>0.52</v>
       </c>
       <c r="AJ186" s="2" t="n"/>
       <c r="AK186" s="2" t="n">
-        <v>8.4</v>
+        <v>7.48</v>
       </c>
       <c r="AL186" s="2" t="n">
-        <v>-4.56</v>
+        <v>-5.76</v>
       </c>
       <c r="AM186" s="2" t="n">
         <v>79.09999999999999</v>
@@ -30412,7 +30412,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-17 | 197 只</t>
+          <t>截至: 2026-10-18 | 197 只</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
auto: 更新 Swing Pattern (海外) 2026-10-25
</commit_message>
<xml_diff>
--- a/OVERSEAS_Swing_Pattern.xlsx
+++ b/OVERSEAS_Swing_Pattern.xlsx
@@ -4239,7 +4239,7 @@
         <v>78584.819</v>
       </c>
       <c r="BB23" s="2" t="n">
-        <v>70593.933</v>
+        <v>70593.93399999999</v>
       </c>
       <c r="BC23" s="2" t="n">
         <v>-0.1989</v>
@@ -7624,7 +7624,7 @@
         <v>173.94</v>
       </c>
       <c r="D46" s="2" t="n">
-        <v>0.58</v>
+        <v>0.57</v>
       </c>
       <c r="E46" s="2" t="inlineStr"/>
       <c r="F46" s="2" t="inlineStr"/>
@@ -15440,10 +15440,10 @@
         </is>
       </c>
       <c r="C97" s="2" t="n">
-        <v>14.3</v>
+        <v>14.31</v>
       </c>
       <c r="D97" s="2" t="n">
-        <v>6.33</v>
+        <v>7.58</v>
       </c>
       <c r="E97" s="2" t="inlineStr"/>
       <c r="F97" s="2" t="inlineStr"/>
@@ -15511,22 +15511,22 @@
       <c r="AH97" s="2" t="inlineStr"/>
       <c r="AI97" s="2" t="inlineStr"/>
       <c r="AJ97" s="2" t="n">
-        <v>34.23</v>
+        <v>34.25</v>
       </c>
       <c r="AK97" s="2" t="n">
-        <v>1.28</v>
+        <v>1.35</v>
       </c>
       <c r="AL97" s="2" t="n">
-        <v>3.15</v>
+        <v>3.22</v>
       </c>
       <c r="AM97" s="2" t="n">
-        <v>-8.23</v>
+        <v>-8.16</v>
       </c>
       <c r="AN97" s="2" t="n">
-        <v>-5.04</v>
+        <v>-4.97</v>
       </c>
       <c r="AO97" s="2" t="n">
-        <v>45.7</v>
+        <v>45.8</v>
       </c>
       <c r="AP97" s="2" t="n">
         <v>15</v>
@@ -15541,10 +15541,10 @@
         </is>
       </c>
       <c r="AV97" s="2" t="n">
-        <v>14.616</v>
+        <v>14.618</v>
       </c>
       <c r="AW97" s="2" t="n">
-        <v>14.98</v>
+        <v>14.981</v>
       </c>
       <c r="AX97" s="2" t="n">
         <v>14.941</v>
@@ -15562,19 +15562,19 @@
         <v>14.348</v>
       </c>
       <c r="BC97" s="2" t="n">
-        <v>-0.9039</v>
+        <v>-0.9005</v>
       </c>
       <c r="BD97" s="2" t="n">
-        <v>-0.0104</v>
+        <v>-0.008699999999999999</v>
       </c>
       <c r="BE97" s="2" t="n">
-        <v>-0.0968</v>
+        <v>-0.0961</v>
       </c>
       <c r="BF97" s="2" t="n">
-        <v>-0.1338</v>
+        <v>-0.1334</v>
       </c>
       <c r="BG97" s="2" t="n">
-        <v>0.3423</v>
+        <v>0.3425</v>
       </c>
     </row>
     <row r="98">
@@ -15592,7 +15592,7 @@
         <v>123.69</v>
       </c>
       <c r="D98" s="2" t="n">
-        <v>-1</v>
+        <v>-0.99</v>
       </c>
       <c r="E98" s="2" t="inlineStr">
         <is>
@@ -15843,7 +15843,7 @@
         </is>
       </c>
       <c r="AV99" s="2" t="n">
-        <v>332.729</v>
+        <v>332.73</v>
       </c>
       <c r="AW99" s="2" t="n">
         <v>340.76</v>
@@ -15864,7 +15864,7 @@
         <v>340.985</v>
       </c>
       <c r="BC99" s="2" t="n">
-        <v>-1.2067</v>
+        <v>-1.2066</v>
       </c>
       <c r="BD99" s="2" t="n">
         <v>-0.4998</v>
@@ -17122,7 +17122,7 @@
         <v>86.95999999999999</v>
       </c>
       <c r="D108" s="2" t="n">
-        <v>2.77</v>
+        <v>2.76</v>
       </c>
       <c r="E108" s="2" t="inlineStr"/>
       <c r="F108" s="2" t="inlineStr"/>
@@ -30922,7 +30922,7 @@
         <v>59.05</v>
       </c>
       <c r="D198" s="2" t="n">
-        <v>-1.18</v>
+        <v>-1.21</v>
       </c>
       <c r="E198" s="2" t="inlineStr"/>
       <c r="F198" s="2" t="inlineStr"/>
@@ -31082,7 +31082,7 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>截至: 2026-10-24 | 197 只</t>
+          <t>截至: 2026-10-25 | 197 只</t>
         </is>
       </c>
     </row>

</xml_diff>